<commit_message>
Stop tag insertion from overwriting the OKVED/MO name cell (column 0)
In one table (t29Ved14 "Платежи по инвестиционной деятельности" section),
the name cell in column 0 is horizontally merged with the first data
column for every row. The tag-insertion loop in generate_word_template()
wrote by column index without checking whether that index's cell was
actually the same physical cell as column 0, so it overwrote the OKVED/MO
name text with a data tag in 12 rows.

Now skips writing a tag into any column whose cell is the same merged
cell as column 0, since there is no distinct cell there to hold it.
</commit_message>
<xml_diff>
--- a/output/unfilled_tags.xlsx
+++ b/output/unfilled_tags.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1714"/>
+  <dimension ref="A1:A1713"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10961,574 +10961,574 @@
     <row r="1507">
       <c r="A1507" t="inlineStr">
         <is>
-          <t>OKVED_32_PlPoInvDeyt</t>
+          <t>OKVED_32_DolUch</t>
         </is>
       </c>
     </row>
     <row r="1508">
       <c r="A1508" t="inlineStr">
         <is>
-          <t>OKVED_32_DolUch</t>
+          <t>OKVED_32_PrCenBum</t>
         </is>
       </c>
     </row>
     <row r="1509">
       <c r="A1509" t="inlineStr">
         <is>
-          <t>OKVED_32_PrCenBum</t>
+          <t>OKVED_32_ProcDolgObyazVklInvAkt</t>
         </is>
       </c>
     </row>
     <row r="1510">
       <c r="A1510" t="inlineStr">
         <is>
-          <t>OKVED_32_ProcDolgObyazVklInvAkt</t>
+          <t>OKVED_32_PrPoFin</t>
         </is>
       </c>
     </row>
     <row r="1511">
       <c r="A1511" t="inlineStr">
         <is>
-          <t>OKVED_32_PrPoFin</t>
+          <t>OKVED_32_Saldo</t>
         </is>
       </c>
     </row>
     <row r="1512">
       <c r="A1512" t="inlineStr">
         <is>
-          <t>OKVED_32_Saldo</t>
+          <t>OKVED_33_DolUch</t>
         </is>
       </c>
     </row>
     <row r="1513">
       <c r="A1513" t="inlineStr">
         <is>
-          <t>OKVED_33_DolUch</t>
+          <t>OKVED_33_ProcDolgObyazVklInvAkt</t>
         </is>
       </c>
     </row>
     <row r="1514">
       <c r="A1514" t="inlineStr">
         <is>
-          <t>OKVED_33_ProcDolgObyazVklInvAkt</t>
+          <t>OKVED_33_PrPoFin</t>
         </is>
       </c>
     </row>
     <row r="1515">
       <c r="A1515" t="inlineStr">
         <is>
-          <t>OKVED_33_PrPoFin</t>
+          <t>OKVED_E_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1516">
       <c r="A1516" t="inlineStr">
         <is>
-          <t>OKVED_E_PostDeyt1</t>
+          <t>OKVED_E_DrPost</t>
         </is>
       </c>
     </row>
     <row r="1517">
       <c r="A1517" t="inlineStr">
         <is>
-          <t>OKVED_E_DrPost</t>
+          <t>OKVED_38_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1518">
       <c r="A1518" t="inlineStr">
         <is>
-          <t>OKVED_38_PostDeyt1</t>
+          <t>OKVED_38_DrPost</t>
         </is>
       </c>
     </row>
     <row r="1519">
       <c r="A1519" t="inlineStr">
         <is>
-          <t>OKVED_38_DrPost</t>
+          <t>OKVED_F_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1520">
       <c r="A1520" t="inlineStr">
         <is>
-          <t>OKVED_F_PostDeyt1</t>
+          <t>OKVED_41_PostDeyt</t>
         </is>
       </c>
     </row>
     <row r="1521">
       <c r="A1521" t="inlineStr">
         <is>
-          <t>OKVED_41_PostDeyt</t>
+          <t>OKVED_41_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1522">
       <c r="A1522" t="inlineStr">
         <is>
-          <t>OKVED_41_PostDeyt1</t>
+          <t>OKVED_42_PostDeyt</t>
         </is>
       </c>
     </row>
     <row r="1523">
       <c r="A1523" t="inlineStr">
         <is>
-          <t>OKVED_42_PostDeyt</t>
+          <t>OKVED_42_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1524">
       <c r="A1524" t="inlineStr">
         <is>
-          <t>OKVED_42_PostDeyt1</t>
+          <t>OKVED_42_DrPost</t>
         </is>
       </c>
     </row>
     <row r="1525">
       <c r="A1525" t="inlineStr">
         <is>
-          <t>OKVED_42_DrPost</t>
+          <t>OKVED_43_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1526">
       <c r="A1526" t="inlineStr">
         <is>
-          <t>OKVED_43_PostDeyt1</t>
+          <t>OKVED_43_DrPost</t>
         </is>
       </c>
     </row>
     <row r="1527">
       <c r="A1527" t="inlineStr">
         <is>
-          <t>OKVED_43_DrPost</t>
+          <t>OKVED_G_PostDeyt</t>
         </is>
       </c>
     </row>
     <row r="1528">
       <c r="A1528" t="inlineStr">
         <is>
-          <t>OKVED_G_PostDeyt</t>
+          <t>OKVED_G_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1529">
       <c r="A1529" t="inlineStr">
         <is>
-          <t>OKVED_G_PostDeyt1</t>
+          <t>OKVED_46_PostDeyt</t>
         </is>
       </c>
     </row>
     <row r="1530">
       <c r="A1530" t="inlineStr">
         <is>
-          <t>OKVED_46_PostDeyt</t>
+          <t>OKVED_46_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1531">
       <c r="A1531" t="inlineStr">
         <is>
-          <t>OKVED_46_PostDeyt1</t>
+          <t>OKVED_47_PostDeyt</t>
         </is>
       </c>
     </row>
     <row r="1532">
       <c r="A1532" t="inlineStr">
         <is>
-          <t>OKVED_47_PostDeyt</t>
+          <t>OKVED_47_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1533">
       <c r="A1533" t="inlineStr">
         <is>
-          <t>OKVED_47_PostDeyt1</t>
+          <t>OKVED_H_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1534">
       <c r="A1534" t="inlineStr">
         <is>
-          <t>OKVED_H_PostDeyt1</t>
+          <t>OKVED_49_PostDeyt</t>
         </is>
       </c>
     </row>
     <row r="1535">
       <c r="A1535" t="inlineStr">
         <is>
-          <t>OKVED_49_PostDeyt</t>
+          <t>OKVED_49_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1536">
       <c r="A1536" t="inlineStr">
         <is>
-          <t>OKVED_49_PostDeyt1</t>
+          <t>OKVED_50_PostDeyt</t>
         </is>
       </c>
     </row>
     <row r="1537">
       <c r="A1537" t="inlineStr">
         <is>
-          <t>OKVED_50_PostDeyt</t>
+          <t>OKVED_50_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1538">
       <c r="A1538" t="inlineStr">
         <is>
-          <t>OKVED_50_PostDeyt1</t>
+          <t>OKVED_50_DrPost</t>
         </is>
       </c>
     </row>
     <row r="1539">
       <c r="A1539" t="inlineStr">
         <is>
-          <t>OKVED_50_DrPost</t>
+          <t>OKVED_51_PostDeyt</t>
         </is>
       </c>
     </row>
     <row r="1540">
       <c r="A1540" t="inlineStr">
         <is>
-          <t>OKVED_51_PostDeyt</t>
+          <t>OKVED_51_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1541">
       <c r="A1541" t="inlineStr">
         <is>
-          <t>OKVED_51_PostDeyt1</t>
+          <t>OKVED_51_DrPost</t>
         </is>
       </c>
     </row>
     <row r="1542">
       <c r="A1542" t="inlineStr">
         <is>
-          <t>OKVED_51_DrPost</t>
+          <t>OKVED_52_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1543">
       <c r="A1543" t="inlineStr">
         <is>
-          <t>OKVED_52_PostDeyt1</t>
+          <t>OKVED_I_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1544">
       <c r="A1544" t="inlineStr">
         <is>
-          <t>OKVED_I_PostDeyt1</t>
+          <t>OKVED_I_DrPost</t>
         </is>
       </c>
     </row>
     <row r="1545">
       <c r="A1545" t="inlineStr">
         <is>
-          <t>OKVED_I_DrPost</t>
+          <t>OKVED_55_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1546">
       <c r="A1546" t="inlineStr">
         <is>
-          <t>OKVED_55_PostDeyt1</t>
+          <t>OKVED_55_DrPost</t>
         </is>
       </c>
     </row>
     <row r="1547">
       <c r="A1547" t="inlineStr">
         <is>
-          <t>OKVED_55_DrPost</t>
+          <t>OKVED_K_PostDeyt</t>
         </is>
       </c>
     </row>
     <row r="1548">
       <c r="A1548" t="inlineStr">
         <is>
-          <t>OKVED_K_PostDeyt</t>
+          <t>OKVED_K_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1549">
       <c r="A1549" t="inlineStr">
         <is>
-          <t>OKVED_K_PostDeyt1</t>
+          <t>OKVED_K_DrPost</t>
         </is>
       </c>
     </row>
     <row r="1550">
       <c r="A1550" t="inlineStr">
         <is>
-          <t>OKVED_K_DrPost</t>
+          <t>OKVED_64_PostDeyt</t>
         </is>
       </c>
     </row>
     <row r="1551">
       <c r="A1551" t="inlineStr">
         <is>
-          <t>OKVED_64_PostDeyt</t>
+          <t>OKVED_64_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1552">
       <c r="A1552" t="inlineStr">
         <is>
-          <t>OKVED_64_PostDeyt1</t>
+          <t>OKVED_64_DrPost</t>
         </is>
       </c>
     </row>
     <row r="1553">
       <c r="A1553" t="inlineStr">
         <is>
-          <t>OKVED_64_DrPost</t>
+          <t>OKVED_L_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1554">
       <c r="A1554" t="inlineStr">
         <is>
-          <t>OKVED_L_PostDeyt1</t>
+          <t>OKVED_68_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1555">
       <c r="A1555" t="inlineStr">
         <is>
-          <t>OKVED_68_PostDeyt1</t>
+          <t>OKVED_M_PostDeyt</t>
         </is>
       </c>
     </row>
     <row r="1556">
       <c r="A1556" t="inlineStr">
         <is>
-          <t>OKVED_M_PostDeyt</t>
+          <t>OKVED_70_PlCredit</t>
         </is>
       </c>
     </row>
     <row r="1557">
       <c r="A1557" t="inlineStr">
         <is>
-          <t>OKVED_70_PlCredit</t>
+          <t>OKVED_70_PostDeyt</t>
         </is>
       </c>
     </row>
     <row r="1558">
       <c r="A1558" t="inlineStr">
         <is>
-          <t>OKVED_70_PostDeyt</t>
+          <t>OKVED_71_PostDeyt</t>
         </is>
       </c>
     </row>
     <row r="1559">
       <c r="A1559" t="inlineStr">
         <is>
-          <t>OKVED_71_PostDeyt</t>
+          <t>OKVED_74_PostDeyt</t>
         </is>
       </c>
     </row>
     <row r="1560">
       <c r="A1560" t="inlineStr">
         <is>
-          <t>OKVED_74_PostDeyt</t>
+          <t>OKVED_74_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1561">
       <c r="A1561" t="inlineStr">
         <is>
-          <t>OKVED_74_PostDeyt1</t>
+          <t>OKVED_74_DrPost</t>
         </is>
       </c>
     </row>
     <row r="1562">
       <c r="A1562" t="inlineStr">
         <is>
-          <t>OKVED_74_DrPost</t>
+          <t>OKVED_N_PostDeyt</t>
         </is>
       </c>
     </row>
     <row r="1563">
       <c r="A1563" t="inlineStr">
         <is>
-          <t>OKVED_N_PostDeyt</t>
+          <t>OKVED_N_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1564">
       <c r="A1564" t="inlineStr">
         <is>
-          <t>OKVED_N_PostDeyt1</t>
+          <t>OKVED_79_PostDeyt</t>
         </is>
       </c>
     </row>
     <row r="1565">
       <c r="A1565" t="inlineStr">
         <is>
-          <t>OKVED_79_PostDeyt</t>
+          <t>OKVED_79_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1566">
       <c r="A1566" t="inlineStr">
         <is>
-          <t>OKVED_79_PostDeyt1</t>
+          <t>OKVED_79_DrPost</t>
         </is>
       </c>
     </row>
     <row r="1567">
       <c r="A1567" t="inlineStr">
         <is>
-          <t>OKVED_79_DrPost</t>
+          <t>OKVED_81_PlCredit</t>
         </is>
       </c>
     </row>
     <row r="1568">
       <c r="A1568" t="inlineStr">
         <is>
-          <t>OKVED_81_PlCredit</t>
+          <t>OKVED_81_PostDeyt</t>
         </is>
       </c>
     </row>
     <row r="1569">
       <c r="A1569" t="inlineStr">
         <is>
-          <t>OKVED_81_PostDeyt</t>
+          <t>OKVED_81_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1570">
       <c r="A1570" t="inlineStr">
         <is>
-          <t>OKVED_81_PostDeyt1</t>
+          <t>OKVED_S_PlCredit</t>
         </is>
       </c>
     </row>
     <row r="1571">
       <c r="A1571" t="inlineStr">
         <is>
-          <t>OKVED_S_PlCredit</t>
+          <t>OKVED_S_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1572">
       <c r="A1572" t="inlineStr">
         <is>
-          <t>OKVED_S_PostDeyt1</t>
+          <t>OKVED_94_PlCredit</t>
         </is>
       </c>
     </row>
     <row r="1573">
       <c r="A1573" t="inlineStr">
         <is>
-          <t>OKVED_94_PlCredit</t>
+          <t>OKVED_94_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1574">
       <c r="A1574" t="inlineStr">
         <is>
-          <t>OKVED_94_PostDeyt1</t>
+          <t>OKVED_01_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1575">
       <c r="A1575" t="inlineStr">
         <is>
-          <t>OKVED_01_PlPoFin1</t>
+          <t>OKVED_01_PlPoFin2</t>
         </is>
       </c>
     </row>
     <row r="1576">
       <c r="A1576" t="inlineStr">
         <is>
-          <t>OKVED_01_PlPoFin2</t>
+          <t>OKVED_B_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1577">
       <c r="A1577" t="inlineStr">
         <is>
-          <t>OKVED_B_PlPoFin1</t>
+          <t>OKVED_07_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1578">
       <c r="A1578" t="inlineStr">
         <is>
-          <t>OKVED_07_PlPoFin1</t>
+          <t>OKVED_32_PlPoFin</t>
         </is>
       </c>
     </row>
     <row r="1579">
       <c r="A1579" t="inlineStr">
         <is>
-          <t>OKVED_32_PlPoFin</t>
+          <t>OKVED_32_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1580">
       <c r="A1580" t="inlineStr">
         <is>
-          <t>OKVED_32_PlPoFin1</t>
+          <t>OKVED_32_PlPoFin2</t>
         </is>
       </c>
     </row>
     <row r="1581">
       <c r="A1581" t="inlineStr">
         <is>
-          <t>OKVED_32_PlPoFin2</t>
+          <t>OKVED_32_PlPoFin3</t>
         </is>
       </c>
     </row>
     <row r="1582">
       <c r="A1582" t="inlineStr">
         <is>
-          <t>OKVED_32_PlPoFin3</t>
+          <t>OKVED_32_PrPoFin</t>
         </is>
       </c>
     </row>
     <row r="1583">
       <c r="A1583" t="inlineStr">
         <is>
-          <t>OKVED_32_PrPoFin</t>
+          <t>OKVED_33_PlPoFin</t>
         </is>
       </c>
     </row>
     <row r="1584">
       <c r="A1584" t="inlineStr">
         <is>
-          <t>OKVED_33_PlPoFin</t>
+          <t>OKVED_33_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1585">
       <c r="A1585" t="inlineStr">
         <is>
-          <t>OKVED_33_PlPoFin1</t>
+          <t>OKVED_33_PlPoFin2</t>
         </is>
       </c>
     </row>
     <row r="1586">
       <c r="A1586" t="inlineStr">
         <is>
-          <t>OKVED_33_PlPoFin2</t>
+          <t>OKVED_33_PlPoFin3</t>
         </is>
       </c>
     </row>
     <row r="1587">
       <c r="A1587" t="inlineStr">
         <is>
-          <t>OKVED_33_PlPoFin3</t>
+          <t>OKVED_33_PrPoFin</t>
         </is>
       </c>
     </row>
     <row r="1588">
       <c r="A1588" t="inlineStr">
         <is>
-          <t>OKVED_33_PrPoFin</t>
+          <t>OKVED_35_PlPoFin1</t>
         </is>
       </c>
     </row>
@@ -11542,651 +11542,651 @@
     <row r="1590">
       <c r="A1590" t="inlineStr">
         <is>
-          <t>OKVED_35_PlPoFin1</t>
+          <t>OKVED_E_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1591">
       <c r="A1591" t="inlineStr">
         <is>
-          <t>OKVED_E_PlPoFin1</t>
+          <t>OKVED_E_PlPoFin2</t>
         </is>
       </c>
     </row>
     <row r="1592">
       <c r="A1592" t="inlineStr">
         <is>
-          <t>OKVED_E_PlPoFin2</t>
+          <t>OKVED_38_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1593">
       <c r="A1593" t="inlineStr">
         <is>
-          <t>OKVED_38_PlPoFin1</t>
+          <t>OKVED_38_PlPoFin2</t>
         </is>
       </c>
     </row>
     <row r="1594">
       <c r="A1594" t="inlineStr">
         <is>
-          <t>OKVED_38_PlPoFin2</t>
+          <t>OKVED_F_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1595">
       <c r="A1595" t="inlineStr">
         <is>
-          <t>OKVED_F_PlPoFin1</t>
+          <t>OKVED_41_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1596">
       <c r="A1596" t="inlineStr">
         <is>
-          <t>OKVED_41_PlPoFin1</t>
+          <t>OKVED_42_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1597">
       <c r="A1597" t="inlineStr">
         <is>
-          <t>OKVED_42_PlPoFin1</t>
+          <t>OKVED_43_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1598">
       <c r="A1598" t="inlineStr">
         <is>
-          <t>OKVED_43_PlPoFin1</t>
+          <t>OKVED_43_PlPoFin2</t>
         </is>
       </c>
     </row>
     <row r="1599">
       <c r="A1599" t="inlineStr">
         <is>
-          <t>OKVED_43_PlPoFin2</t>
+          <t>OKVED_43_PrPoFin</t>
         </is>
       </c>
     </row>
     <row r="1600">
       <c r="A1600" t="inlineStr">
         <is>
-          <t>OKVED_43_PrPoFin</t>
+          <t>OKVED_G_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1601">
       <c r="A1601" t="inlineStr">
         <is>
-          <t>OKVED_G_PlPoFin1</t>
+          <t>OKVED_46_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1602">
       <c r="A1602" t="inlineStr">
         <is>
-          <t>OKVED_46_PlPoFin1</t>
+          <t>OKVED_47_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1603">
       <c r="A1603" t="inlineStr">
         <is>
-          <t>OKVED_47_PlPoFin1</t>
+          <t>OKVED_H_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1604">
       <c r="A1604" t="inlineStr">
         <is>
-          <t>OKVED_H_PlPoFin1</t>
+          <t>OKVED_49_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1605">
       <c r="A1605" t="inlineStr">
         <is>
-          <t>OKVED_49_PlPoFin1</t>
+          <t>OKVED_49_PlPoFin2</t>
         </is>
       </c>
     </row>
     <row r="1606">
       <c r="A1606" t="inlineStr">
         <is>
-          <t>OKVED_49_PlPoFin2</t>
+          <t>OKVED_49_PrPoFin</t>
         </is>
       </c>
     </row>
     <row r="1607">
       <c r="A1607" t="inlineStr">
         <is>
-          <t>OKVED_49_PrPoFin</t>
+          <t>OKVED_50_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1608">
       <c r="A1608" t="inlineStr">
         <is>
-          <t>OKVED_50_PlPoFin1</t>
+          <t>OKVED_50_PrPoFin</t>
         </is>
       </c>
     </row>
     <row r="1609">
       <c r="A1609" t="inlineStr">
         <is>
-          <t>OKVED_50_PrPoFin</t>
+          <t>OKVED_51_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1610">
       <c r="A1610" t="inlineStr">
         <is>
-          <t>OKVED_51_PlPoFin1</t>
+          <t>OKVED_51_PlPoFin2</t>
         </is>
       </c>
     </row>
     <row r="1611">
       <c r="A1611" t="inlineStr">
         <is>
-          <t>OKVED_51_PlPoFin2</t>
+          <t>OKVED_52_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1612">
       <c r="A1612" t="inlineStr">
         <is>
-          <t>OKVED_52_PlPoFin1</t>
+          <t>OKVED_I_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1613">
       <c r="A1613" t="inlineStr">
         <is>
-          <t>OKVED_I_PlPoFin1</t>
+          <t>OKVED_I_PlPoFin2</t>
         </is>
       </c>
     </row>
     <row r="1614">
       <c r="A1614" t="inlineStr">
         <is>
-          <t>OKVED_I_PlPoFin2</t>
+          <t>OKVED_I_PrPoFin</t>
         </is>
       </c>
     </row>
     <row r="1615">
       <c r="A1615" t="inlineStr">
         <is>
-          <t>OKVED_I_PrPoFin</t>
+          <t>OKVED_55_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1616">
       <c r="A1616" t="inlineStr">
         <is>
-          <t>OKVED_55_PlPoFin1</t>
+          <t>OKVED_55_PlPoFin2</t>
         </is>
       </c>
     </row>
     <row r="1617">
       <c r="A1617" t="inlineStr">
         <is>
-          <t>OKVED_55_PlPoFin2</t>
+          <t>OKVED_55_PrPoFin</t>
         </is>
       </c>
     </row>
     <row r="1618">
       <c r="A1618" t="inlineStr">
         <is>
-          <t>OKVED_55_PrPoFin</t>
+          <t>OKVED_K_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1619">
       <c r="A1619" t="inlineStr">
         <is>
-          <t>OKVED_K_PlPoFin1</t>
+          <t>OKVED_K_PrPoFin</t>
         </is>
       </c>
     </row>
     <row r="1620">
       <c r="A1620" t="inlineStr">
         <is>
-          <t>OKVED_K_PrPoFin</t>
+          <t>OKVED_64_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1621">
       <c r="A1621" t="inlineStr">
         <is>
-          <t>OKVED_64_PlPoFin1</t>
+          <t>OKVED_64_PrPoFin</t>
         </is>
       </c>
     </row>
     <row r="1622">
       <c r="A1622" t="inlineStr">
         <is>
-          <t>OKVED_64_PrPoFin</t>
+          <t>OKVED_L_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1623">
       <c r="A1623" t="inlineStr">
         <is>
-          <t>OKVED_L_PlPoFin1</t>
+          <t>OKVED_68_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1624">
       <c r="A1624" t="inlineStr">
         <is>
-          <t>OKVED_68_PlPoFin1</t>
+          <t>OKVED_M_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1625">
       <c r="A1625" t="inlineStr">
         <is>
-          <t>OKVED_M_PlPoFin1</t>
+          <t>OKVED_70_PlPoFin</t>
         </is>
       </c>
     </row>
     <row r="1626">
       <c r="A1626" t="inlineStr">
         <is>
-          <t>OKVED_70_PlPoFin</t>
+          <t>OKVED_70_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1627">
       <c r="A1627" t="inlineStr">
         <is>
-          <t>OKVED_70_PlPoFin1</t>
+          <t>OKVED_70_PlPoFin2</t>
         </is>
       </c>
     </row>
     <row r="1628">
       <c r="A1628" t="inlineStr">
         <is>
-          <t>OKVED_70_PlPoFin2</t>
+          <t>OKVED_70_PlPoFin3</t>
         </is>
       </c>
     </row>
     <row r="1629">
       <c r="A1629" t="inlineStr">
         <is>
-          <t>OKVED_70_PlPoFin3</t>
+          <t>OKVED_70_PrPoFin</t>
         </is>
       </c>
     </row>
     <row r="1630">
       <c r="A1630" t="inlineStr">
         <is>
-          <t>OKVED_70_PrPoFin</t>
+          <t>OKVED_71_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1631">
       <c r="A1631" t="inlineStr">
         <is>
-          <t>OKVED_71_PlPoFin1</t>
+          <t>OKVED_74_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1632">
       <c r="A1632" t="inlineStr">
         <is>
-          <t>OKVED_74_PlPoFin1</t>
+          <t>OKVED_74_PlPoFin2</t>
         </is>
       </c>
     </row>
     <row r="1633">
       <c r="A1633" t="inlineStr">
         <is>
-          <t>OKVED_74_PlPoFin2</t>
+          <t>OKVED_74_PlPoFin3</t>
         </is>
       </c>
     </row>
     <row r="1634">
       <c r="A1634" t="inlineStr">
         <is>
-          <t>OKVED_74_PlPoFin3</t>
+          <t>OKVED_74_SaldoDenPot</t>
         </is>
       </c>
     </row>
     <row r="1635">
       <c r="A1635" t="inlineStr">
         <is>
-          <t>OKVED_74_SaldoDenPot</t>
+          <t>OKVED_N_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1636">
       <c r="A1636" t="inlineStr">
         <is>
-          <t>OKVED_N_PlPoFin1</t>
+          <t>OKVED_N_PlPoFin2</t>
         </is>
       </c>
     </row>
     <row r="1637">
       <c r="A1637" t="inlineStr">
         <is>
-          <t>OKVED_N_PlPoFin2</t>
+          <t>OKVED_79_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1638">
       <c r="A1638" t="inlineStr">
         <is>
-          <t>OKVED_79_PlPoFin1</t>
+          <t>OKVED_79_PlPoFin2</t>
         </is>
       </c>
     </row>
     <row r="1639">
       <c r="A1639" t="inlineStr">
         <is>
-          <t>OKVED_79_PlPoFin2</t>
+          <t>OKVED_79_PrPoFin</t>
         </is>
       </c>
     </row>
     <row r="1640">
       <c r="A1640" t="inlineStr">
         <is>
-          <t>OKVED_79_PrPoFin</t>
+          <t>OKVED_81_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1641">
       <c r="A1641" t="inlineStr">
         <is>
-          <t>OKVED_81_PlPoFin1</t>
+          <t>OKVED_81_PlPoFin2</t>
         </is>
       </c>
     </row>
     <row r="1642">
       <c r="A1642" t="inlineStr">
         <is>
-          <t>OKVED_81_PlPoFin2</t>
+          <t>OKVED_81_PlPoFin3</t>
         </is>
       </c>
     </row>
     <row r="1643">
       <c r="A1643" t="inlineStr">
         <is>
-          <t>OKVED_81_PlPoFin3</t>
+          <t>OKVED_81_SaldoDenPot</t>
         </is>
       </c>
     </row>
     <row r="1644">
       <c r="A1644" t="inlineStr">
         <is>
-          <t>OKVED_81_SaldoDenPot</t>
+          <t>OKVED_S_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1645">
       <c r="A1645" t="inlineStr">
         <is>
-          <t>OKVED_S_PlPoFin1</t>
+          <t>OKVED_S_PlPoFin2</t>
         </is>
       </c>
     </row>
     <row r="1646">
       <c r="A1646" t="inlineStr">
         <is>
-          <t>OKVED_S_PlPoFin2</t>
+          <t>OKVED_S_PlPoFin3</t>
         </is>
       </c>
     </row>
     <row r="1647">
       <c r="A1647" t="inlineStr">
         <is>
-          <t>OKVED_S_PlPoFin3</t>
+          <t>OKVED_94_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1648">
       <c r="A1648" t="inlineStr">
         <is>
-          <t>OKVED_94_PlPoFin1</t>
+          <t>OKVED_94_PlPoFin2</t>
         </is>
       </c>
     </row>
     <row r="1649">
       <c r="A1649" t="inlineStr">
         <is>
-          <t>OKVED_94_PlPoFin2</t>
+          <t>OKVED_94_PlPoFin3</t>
         </is>
       </c>
     </row>
     <row r="1650">
       <c r="A1650" t="inlineStr">
         <is>
-          <t>OKVED_94_PlPoFin3</t>
+          <t>OKVED_01_Velch</t>
         </is>
       </c>
     </row>
     <row r="1651">
       <c r="A1651" t="inlineStr">
         <is>
-          <t>OKVED_01_Velch</t>
+          <t>OKVED_11_Velch</t>
         </is>
       </c>
     </row>
     <row r="1652">
       <c r="A1652" t="inlineStr">
         <is>
-          <t>OKVED_11_Velch</t>
+          <t>OKVED_32_Velch</t>
         </is>
       </c>
     </row>
     <row r="1653">
       <c r="A1653" t="inlineStr">
         <is>
-          <t>OKVED_32_Velch</t>
+          <t>OKVED_33_Velch</t>
         </is>
       </c>
     </row>
     <row r="1654">
       <c r="A1654" t="inlineStr">
         <is>
-          <t>OKVED_33_Velch</t>
+          <t>OKVED_E_Velch</t>
         </is>
       </c>
     </row>
     <row r="1655">
       <c r="A1655" t="inlineStr">
         <is>
-          <t>OKVED_E_Velch</t>
+          <t>OKVED_36_Velch</t>
         </is>
       </c>
     </row>
     <row r="1656">
       <c r="A1656" t="inlineStr">
         <is>
-          <t>OKVED_36_Velch</t>
+          <t>OKVED_38_Velch</t>
         </is>
       </c>
     </row>
     <row r="1657">
       <c r="A1657" t="inlineStr">
         <is>
-          <t>OKVED_38_Velch</t>
+          <t>OKVED_F_Velch</t>
         </is>
       </c>
     </row>
     <row r="1658">
       <c r="A1658" t="inlineStr">
         <is>
-          <t>OKVED_F_Velch</t>
+          <t>OKVED_41_Velch</t>
         </is>
       </c>
     </row>
     <row r="1659">
       <c r="A1659" t="inlineStr">
         <is>
-          <t>OKVED_41_Velch</t>
+          <t>OKVED_42_Velch</t>
         </is>
       </c>
     </row>
     <row r="1660">
       <c r="A1660" t="inlineStr">
         <is>
-          <t>OKVED_42_Velch</t>
+          <t>OKVED_43_Velch</t>
         </is>
       </c>
     </row>
     <row r="1661">
       <c r="A1661" t="inlineStr">
         <is>
-          <t>OKVED_43_Velch</t>
+          <t>OKVED_47_Velch</t>
         </is>
       </c>
     </row>
     <row r="1662">
       <c r="A1662" t="inlineStr">
         <is>
-          <t>OKVED_47_Velch</t>
+          <t>OKVED_49_Velch</t>
         </is>
       </c>
     </row>
     <row r="1663">
       <c r="A1663" t="inlineStr">
         <is>
-          <t>OKVED_49_Velch</t>
+          <t>OKVED_I_Velch</t>
         </is>
       </c>
     </row>
     <row r="1664">
       <c r="A1664" t="inlineStr">
         <is>
-          <t>OKVED_I_Velch</t>
+          <t>OKVED_55_Velch</t>
         </is>
       </c>
     </row>
     <row r="1665">
       <c r="A1665" t="inlineStr">
         <is>
-          <t>OKVED_55_Velch</t>
+          <t>OKVED_56_Velch</t>
         </is>
       </c>
     </row>
     <row r="1666">
       <c r="A1666" t="inlineStr">
         <is>
-          <t>OKVED_56_Velch</t>
+          <t>OKVED_J_Velch</t>
         </is>
       </c>
     </row>
     <row r="1667">
       <c r="A1667" t="inlineStr">
         <is>
-          <t>OKVED_J_Velch</t>
+          <t>OKVED_63_Velch</t>
         </is>
       </c>
     </row>
     <row r="1668">
       <c r="A1668" t="inlineStr">
         <is>
-          <t>OKVED_63_Velch</t>
+          <t>OKVED_L_Velch</t>
         </is>
       </c>
     </row>
     <row r="1669">
       <c r="A1669" t="inlineStr">
         <is>
-          <t>OKVED_L_Velch</t>
+          <t>OKVED_68_Velch</t>
         </is>
       </c>
     </row>
     <row r="1670">
       <c r="A1670" t="inlineStr">
         <is>
-          <t>OKVED_68_Velch</t>
+          <t>OKVED_M_Velch</t>
         </is>
       </c>
     </row>
     <row r="1671">
       <c r="A1671" t="inlineStr">
         <is>
-          <t>OKVED_M_Velch</t>
+          <t>OKVED_69_Velch</t>
         </is>
       </c>
     </row>
     <row r="1672">
       <c r="A1672" t="inlineStr">
         <is>
-          <t>OKVED_69_Velch</t>
+          <t>OKVED_70_Velch</t>
         </is>
       </c>
     </row>
     <row r="1673">
       <c r="A1673" t="inlineStr">
         <is>
-          <t>OKVED_70_Velch</t>
+          <t>OKVED_71_Velch</t>
         </is>
       </c>
     </row>
     <row r="1674">
       <c r="A1674" t="inlineStr">
         <is>
-          <t>OKVED_71_Velch</t>
+          <t>OKVED_74_Velch</t>
         </is>
       </c>
     </row>
     <row r="1675">
       <c r="A1675" t="inlineStr">
         <is>
-          <t>OKVED_74_Velch</t>
+          <t>OKVED_N_Velch</t>
         </is>
       </c>
     </row>
     <row r="1676">
       <c r="A1676" t="inlineStr">
         <is>
-          <t>OKVED_N_Velch</t>
+          <t>OKVED_77_Velch</t>
         </is>
       </c>
     </row>
     <row r="1677">
       <c r="A1677" t="inlineStr">
         <is>
-          <t>OKVED_77_Velch</t>
+          <t>OKVED_79_Velch</t>
         </is>
       </c>
     </row>
     <row r="1678">
       <c r="A1678" t="inlineStr">
         <is>
-          <t>OKVED_79_Velch</t>
+          <t>OKVED_81_Velch</t>
         </is>
       </c>
     </row>
     <row r="1679">
       <c r="A1679" t="inlineStr">
         <is>
-          <t>OKVED_81_Velch</t>
+          <t>OKVED_82_Velch</t>
         </is>
       </c>
     </row>
     <row r="1680">
       <c r="A1680" t="inlineStr">
         <is>
-          <t>OKVED_82_Velch</t>
+          <t>OKVED_O_Velch</t>
         </is>
       </c>
     </row>
     <row r="1681">
       <c r="A1681" t="inlineStr">
         <is>
-          <t>OKVED_O_Velch</t>
+          <t>OKVED_84_Velch</t>
         </is>
       </c>
     </row>
     <row r="1682">
       <c r="A1682" t="inlineStr">
         <is>
-          <t>OKVED_84_Velch</t>
+          <t>OKVED_85_Velch</t>
         </is>
       </c>
     </row>
@@ -12200,215 +12200,208 @@
     <row r="1684">
       <c r="A1684" t="inlineStr">
         <is>
-          <t>OKVED_85_Velch</t>
+          <t>OKVED_Q_Velch</t>
         </is>
       </c>
     </row>
     <row r="1685">
       <c r="A1685" t="inlineStr">
         <is>
-          <t>OKVED_Q_Velch</t>
+          <t>OKVED_88_Velch</t>
         </is>
       </c>
     </row>
     <row r="1686">
       <c r="A1686" t="inlineStr">
         <is>
-          <t>OKVED_88_Velch</t>
+          <t>OKVED_R_Velch</t>
         </is>
       </c>
     </row>
     <row r="1687">
       <c r="A1687" t="inlineStr">
         <is>
-          <t>OKVED_R_Velch</t>
+          <t>OKVED_93_Velch</t>
         </is>
       </c>
     </row>
     <row r="1688">
       <c r="A1688" t="inlineStr">
         <is>
-          <t>OKVED_93_Velch</t>
+          <t>OKVED_S_Velch</t>
         </is>
       </c>
     </row>
     <row r="1689">
       <c r="A1689" t="inlineStr">
         <is>
-          <t>OKVED_S_Velch</t>
+          <t>OKVED_94_Velch</t>
         </is>
       </c>
     </row>
     <row r="1690">
       <c r="A1690" t="inlineStr">
         <is>
-          <t>OKVED_94_Velch</t>
+          <t>OKVED_96_Velch</t>
         </is>
       </c>
     </row>
     <row r="1691">
       <c r="A1691" t="inlineStr">
         <is>
-          <t>OKVED_96_Velch</t>
+          <t>OKVED_43_UstKap_23</t>
         </is>
       </c>
     </row>
     <row r="1692">
       <c r="A1692" t="inlineStr">
         <is>
-          <t>OKVED_43_UstKap_23</t>
+          <t>OKVED_43_ChiAkt_23</t>
         </is>
       </c>
     </row>
     <row r="1693">
       <c r="A1693" t="inlineStr">
         <is>
-          <t>OKVED_43_ChiAkt_23</t>
+          <t>OKVED_J_UstKap_23</t>
         </is>
       </c>
     </row>
     <row r="1694">
       <c r="A1694" t="inlineStr">
         <is>
-          <t>OKVED_J_UstKap_23</t>
+          <t>OKVED_J_UstKap_24</t>
         </is>
       </c>
     </row>
     <row r="1695">
       <c r="A1695" t="inlineStr">
         <is>
-          <t>OKVED_J_UstKap_24</t>
+          <t>OKVED_63_UstKap_23</t>
         </is>
       </c>
     </row>
     <row r="1696">
       <c r="A1696" t="inlineStr">
         <is>
-          <t>OKVED_63_UstKap_23</t>
+          <t>OKVED_63_UstKap_24</t>
         </is>
       </c>
     </row>
     <row r="1697">
       <c r="A1697" t="inlineStr">
         <is>
-          <t>OKVED_63_UstKap_24</t>
+          <t>OKVED_69_UstKap_23</t>
         </is>
       </c>
     </row>
     <row r="1698">
       <c r="A1698" t="inlineStr">
         <is>
-          <t>OKVED_69_UstKap_23</t>
+          <t>OKVED_69_UstKap_24</t>
         </is>
       </c>
     </row>
     <row r="1699">
       <c r="A1699" t="inlineStr">
         <is>
-          <t>OKVED_69_UstKap_24</t>
+          <t>OKVED_69_ChiAkt_23</t>
         </is>
       </c>
     </row>
     <row r="1700">
       <c r="A1700" t="inlineStr">
         <is>
-          <t>OKVED_69_ChiAkt_23</t>
+          <t>OKVED_O_UstKap_23</t>
         </is>
       </c>
     </row>
     <row r="1701">
       <c r="A1701" t="inlineStr">
         <is>
-          <t>OKVED_O_UstKap_23</t>
+          <t>OKVED_O_UstKap_24</t>
         </is>
       </c>
     </row>
     <row r="1702">
       <c r="A1702" t="inlineStr">
         <is>
-          <t>OKVED_O_UstKap_24</t>
+          <t>OKVED_84_UstKap_23</t>
         </is>
       </c>
     </row>
     <row r="1703">
       <c r="A1703" t="inlineStr">
         <is>
-          <t>OKVED_84_UstKap_23</t>
+          <t>OKVED_84_UstKap_24</t>
         </is>
       </c>
     </row>
     <row r="1704">
       <c r="A1704" t="inlineStr">
         <is>
-          <t>OKVED_84_UstKap_24</t>
+          <t>OKVED_85_UstKap_23</t>
         </is>
       </c>
     </row>
     <row r="1705">
       <c r="A1705" t="inlineStr">
         <is>
-          <t>OKVED_85_UstKap_23</t>
+          <t>OKVED_85_UstKap_24</t>
         </is>
       </c>
     </row>
     <row r="1706">
       <c r="A1706" t="inlineStr">
         <is>
-          <t>OKVED_85_UstKap_24</t>
+          <t>OKVED_85_UstKap_23</t>
         </is>
       </c>
     </row>
     <row r="1707">
       <c r="A1707" t="inlineStr">
         <is>
-          <t>OKVED_85_UstKap_23</t>
+          <t>OKVED_85_UstKap_24</t>
         </is>
       </c>
     </row>
     <row r="1708">
       <c r="A1708" t="inlineStr">
         <is>
-          <t>OKVED_85_UstKap_24</t>
+          <t>OKVED_Q_UstKap_23</t>
         </is>
       </c>
     </row>
     <row r="1709">
       <c r="A1709" t="inlineStr">
         <is>
-          <t>OKVED_Q_UstKap_23</t>
+          <t>OKVED_Q_UstKap_24</t>
         </is>
       </c>
     </row>
     <row r="1710">
       <c r="A1710" t="inlineStr">
         <is>
-          <t>OKVED_Q_UstKap_24</t>
+          <t>OKVED_88_UstKap_23</t>
         </is>
       </c>
     </row>
     <row r="1711">
       <c r="A1711" t="inlineStr">
         <is>
-          <t>OKVED_88_UstKap_23</t>
+          <t>OKVED_88_UstKap_24</t>
         </is>
       </c>
     </row>
     <row r="1712">
       <c r="A1712" t="inlineStr">
         <is>
-          <t>OKVED_88_UstKap_24</t>
+          <t>OKVED_R_UstKap_24</t>
         </is>
       </c>
     </row>
     <row r="1713">
       <c r="A1713" t="inlineStr">
-        <is>
-          <t>OKVED_R_UstKap_24</t>
-        </is>
-      </c>
-    </row>
-    <row r="1714">
-      <c r="A1714" t="inlineStr">
         <is>
           <t>OKVED_93_UstKap_24</t>
         </is>

</xml_diff>

<commit_message>
Disambiguate the two identically-named "прочие поступления" rows in t29Ved14 mapping
Same collision as the "прочие платежи" fix, on the receipts side: two
line items in t29Ved14.xlsx (текущая деятельность col7, инвестиционная
деятельность col20) were both named exactly "прочие поступления" in
column_mapping_v2.csv, so file_word_to_indicator collapsed them onto
whichever loaded last — every "прочие поступления" column in tables
sourced from this file got tagged with that one indicator regardless of
which receipts group it belonged to.

Renamed both entries to include their group name, matching the
already-fixed "прочие платежи" pattern.

Verified against the reference bulletin files: tables 107-112 now match
exactly, with no new regressions. Overall numeric match rate improved
from 98.2% to 98.6%.
</commit_message>
<xml_diff>
--- a/output/unfilled_tags.xlsx
+++ b/output/unfilled_tags.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1714"/>
+  <dimension ref="A1:A1661"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9393,3022 +9393,2651 @@
     <row r="1283">
       <c r="A1283" t="inlineStr">
         <is>
-          <t>OKVED_01_PrPostDeyt</t>
+          <t>OKVED_32_ArendPlDeVsego</t>
         </is>
       </c>
     </row>
     <row r="1284">
       <c r="A1284" t="inlineStr">
         <is>
-          <t>OKVED_B_PrPostDeyt</t>
+          <t>OKVED_E_ArendPlDeVsego</t>
         </is>
       </c>
     </row>
     <row r="1285">
       <c r="A1285" t="inlineStr">
         <is>
-          <t>OKVED_07_PrPostDeyt</t>
+          <t>OKVED_36_ArendPlDeVsego</t>
         </is>
       </c>
     </row>
     <row r="1286">
       <c r="A1286" t="inlineStr">
         <is>
-          <t>OKVED_11_PrPostDeyt</t>
+          <t>OKVED_38_ArendPlDeVsego</t>
         </is>
       </c>
     </row>
     <row r="1287">
       <c r="A1287" t="inlineStr">
         <is>
-          <t>OKVED_32_ArendPlDeVsego</t>
+          <t>OKVED_41_ArendPlDeVsego</t>
         </is>
       </c>
     </row>
     <row r="1288">
       <c r="A1288" t="inlineStr">
         <is>
-          <t>OKVED_32_PrPostDeyt</t>
+          <t>OKVED_43_ArendPlDeVsego</t>
         </is>
       </c>
     </row>
     <row r="1289">
       <c r="A1289" t="inlineStr">
         <is>
-          <t>OKVED_33_PrPostDeyt</t>
+          <t>OKVED_49_ArendPlDeVsego</t>
         </is>
       </c>
     </row>
     <row r="1290">
       <c r="A1290" t="inlineStr">
         <is>
-          <t>OKVED_35_PrPostDeyt</t>
+          <t>OKVED_50_ArendPlDeVsego</t>
         </is>
       </c>
     </row>
     <row r="1291">
       <c r="A1291" t="inlineStr">
         <is>
-          <t>OKVED_E_ArendPlDeVsego</t>
+          <t>OKVED_I_ArendPlDeVsego</t>
         </is>
       </c>
     </row>
     <row r="1292">
       <c r="A1292" t="inlineStr">
         <is>
-          <t>OKVED_36_ArendPlDeVsego</t>
+          <t>OKVED_55_ArendPlDeVsego</t>
         </is>
       </c>
     </row>
     <row r="1293">
       <c r="A1293" t="inlineStr">
         <is>
-          <t>OKVED_38_ArendPlDeVsego</t>
+          <t>OKVED_56_ArendPlDeVsego</t>
         </is>
       </c>
     </row>
     <row r="1294">
       <c r="A1294" t="inlineStr">
         <is>
-          <t>OKVED_41_ArendPlDeVsego</t>
+          <t>OKVED_J_OtProdDeVsego</t>
         </is>
       </c>
     </row>
     <row r="1295">
       <c r="A1295" t="inlineStr">
         <is>
-          <t>OKVED_43_ArendPlDeVsego</t>
+          <t>OKVED_J_ArendPlDeVsego</t>
         </is>
       </c>
     </row>
     <row r="1296">
       <c r="A1296" t="inlineStr">
         <is>
-          <t>OKVED_43_PrPostDeyt</t>
+          <t>OKVED_63_OtProdDeVsego</t>
         </is>
       </c>
     </row>
     <row r="1297">
       <c r="A1297" t="inlineStr">
         <is>
-          <t>OKVED_G_PrPostDeyt</t>
+          <t>OKVED_63_ArendPlDeVsego</t>
         </is>
       </c>
     </row>
     <row r="1298">
       <c r="A1298" t="inlineStr">
         <is>
-          <t>OKVED_46_PrPostDeyt</t>
+          <t>OKVED_64_ArendPlDeVsego</t>
         </is>
       </c>
     </row>
     <row r="1299">
       <c r="A1299" t="inlineStr">
         <is>
-          <t>OKVED_H_PrPostDeyt</t>
+          <t>OKVED_69_ArendPlDeVsego</t>
         </is>
       </c>
     </row>
     <row r="1300">
       <c r="A1300" t="inlineStr">
         <is>
-          <t>OKVED_49_ArendPlDeVsego</t>
+          <t>OKVED_79_ArendPlDeVsego</t>
         </is>
       </c>
     </row>
     <row r="1301">
       <c r="A1301" t="inlineStr">
         <is>
-          <t>OKVED_49_PrPostDeyt</t>
+          <t>OKVED_81_ArendPlDeVsego</t>
         </is>
       </c>
     </row>
     <row r="1302">
       <c r="A1302" t="inlineStr">
         <is>
-          <t>OKVED_50_ArendPlDeVsego</t>
+          <t>OKVED_82_ArendPlDeVsego</t>
         </is>
       </c>
     </row>
     <row r="1303">
       <c r="A1303" t="inlineStr">
         <is>
-          <t>OKVED_50_PrPostDeyt</t>
+          <t>OKVED_O_ArendPlDeVsego</t>
         </is>
       </c>
     </row>
     <row r="1304">
       <c r="A1304" t="inlineStr">
         <is>
-          <t>OKVED_51_PrPostDeyt</t>
+          <t>OKVED_84_ArendPlDeVsego</t>
         </is>
       </c>
     </row>
     <row r="1305">
       <c r="A1305" t="inlineStr">
         <is>
-          <t>OKVED_52_PrPostDeyt</t>
+          <t>OKVED_85_ArendPlDeVsego</t>
         </is>
       </c>
     </row>
     <row r="1306">
       <c r="A1306" t="inlineStr">
         <is>
-          <t>OKVED_I_ArendPlDeVsego</t>
+          <t>OKVED_85_ArendPlDeVsego</t>
         </is>
       </c>
     </row>
     <row r="1307">
       <c r="A1307" t="inlineStr">
         <is>
-          <t>OKVED_55_ArendPlDeVsego</t>
+          <t>OKVED_88_OtProdDeVsego</t>
         </is>
       </c>
     </row>
     <row r="1308">
       <c r="A1308" t="inlineStr">
         <is>
-          <t>OKVED_56_ArendPlDeVsego</t>
+          <t>OKVED_88_ArendPlDeVsego</t>
         </is>
       </c>
     </row>
     <row r="1309">
       <c r="A1309" t="inlineStr">
         <is>
-          <t>OKVED_56_PrPostDeyt</t>
+          <t>OKVED_R_OtProdDeVsego</t>
         </is>
       </c>
     </row>
     <row r="1310">
       <c r="A1310" t="inlineStr">
         <is>
-          <t>OKVED_J_OtProdDeVsego</t>
+          <t>OKVED_R_ArendPlDeVsego</t>
         </is>
       </c>
     </row>
     <row r="1311">
       <c r="A1311" t="inlineStr">
         <is>
-          <t>OKVED_J_ArendPlDeVsego</t>
+          <t>OKVED_93_OtProdDeVsego</t>
         </is>
       </c>
     </row>
     <row r="1312">
       <c r="A1312" t="inlineStr">
         <is>
-          <t>OKVED_J_PrPostDeyt</t>
+          <t>OKVED_93_ArendPlDeVsego</t>
         </is>
       </c>
     </row>
     <row r="1313">
       <c r="A1313" t="inlineStr">
         <is>
-          <t>OKVED_63_OtProdDeVsego</t>
+          <t>OKVED_S_ArendPlDeVsego</t>
         </is>
       </c>
     </row>
     <row r="1314">
       <c r="A1314" t="inlineStr">
         <is>
-          <t>OKVED_63_ArendPlDeVsego</t>
+          <t>OKVED_94_ArendPlDeVsego</t>
         </is>
       </c>
     </row>
     <row r="1315">
       <c r="A1315" t="inlineStr">
         <is>
-          <t>OKVED_63_PrPostDeyt</t>
+          <t>OKVED_96_ArendPlDeVsego</t>
         </is>
       </c>
     </row>
     <row r="1316">
       <c r="A1316" t="inlineStr">
         <is>
-          <t>OKVED_64_ArendPlDeVsego</t>
+          <t>OKVED_11_ProcPoDolgObyaz</t>
         </is>
       </c>
     </row>
     <row r="1317">
       <c r="A1317" t="inlineStr">
         <is>
-          <t>OKVED_64_PrPostDeyt</t>
+          <t>OKVED_32_ProcPoDolgObyaz</t>
         </is>
       </c>
     </row>
     <row r="1318">
       <c r="A1318" t="inlineStr">
         <is>
-          <t>OKVED_M_PrPostDeyt</t>
+          <t>OKVED_32_NalogNaPri</t>
         </is>
       </c>
     </row>
     <row r="1319">
       <c r="A1319" t="inlineStr">
         <is>
-          <t>OKVED_69_ArendPlDeVsego</t>
+          <t>OKVED_33_NalogNaPri</t>
         </is>
       </c>
     </row>
     <row r="1320">
       <c r="A1320" t="inlineStr">
         <is>
-          <t>OKVED_69_PrPostDeyt</t>
+          <t>OKVED_36_ProcPoDolgObyaz</t>
         </is>
       </c>
     </row>
     <row r="1321">
       <c r="A1321" t="inlineStr">
         <is>
-          <t>OKVED_70_PrPostDeyt</t>
+          <t>OKVED_38_NalogNaPri</t>
         </is>
       </c>
     </row>
     <row r="1322">
       <c r="A1322" t="inlineStr">
         <is>
-          <t>OKVED_71_PrPostDeyt</t>
+          <t>OKVED_49_ProcPoDolgObyaz</t>
         </is>
       </c>
     </row>
     <row r="1323">
       <c r="A1323" t="inlineStr">
         <is>
-          <t>OKVED_74_PrPostDeyt</t>
+          <t>OKVED_56_ProcPoDolgObyaz</t>
         </is>
       </c>
     </row>
     <row r="1324">
       <c r="A1324" t="inlineStr">
         <is>
-          <t>OKVED_79_ArendPlDeVsego</t>
+          <t>OKVED_56_NalogNaPri</t>
         </is>
       </c>
     </row>
     <row r="1325">
       <c r="A1325" t="inlineStr">
         <is>
-          <t>OKVED_81_ArendPlDeVsego</t>
+          <t>OKVED_J_ProcPoDolgObyaz</t>
         </is>
       </c>
     </row>
     <row r="1326">
       <c r="A1326" t="inlineStr">
         <is>
-          <t>OKVED_81_PrPostDeyt</t>
+          <t>OKVED_J_NalogNaPri</t>
         </is>
       </c>
     </row>
     <row r="1327">
       <c r="A1327" t="inlineStr">
         <is>
-          <t>OKVED_82_ArendPlDeVsego</t>
+          <t>OKVED_63_ProcPoDolgObyaz</t>
         </is>
       </c>
     </row>
     <row r="1328">
       <c r="A1328" t="inlineStr">
         <is>
-          <t>OKVED_82_PrPostDeyt</t>
+          <t>OKVED_63_NalogNaPri</t>
         </is>
       </c>
     </row>
     <row r="1329">
       <c r="A1329" t="inlineStr">
         <is>
-          <t>OKVED_O_ArendPlDeVsego</t>
+          <t>OKVED_M_ProcPoDolgObyaz</t>
         </is>
       </c>
     </row>
     <row r="1330">
       <c r="A1330" t="inlineStr">
         <is>
-          <t>OKVED_O_PrPostDeyt</t>
+          <t>OKVED_69_ProcPoDolgObyaz</t>
         </is>
       </c>
     </row>
     <row r="1331">
       <c r="A1331" t="inlineStr">
         <is>
-          <t>OKVED_84_ArendPlDeVsego</t>
+          <t>OKVED_69_NalogNaPri</t>
         </is>
       </c>
     </row>
     <row r="1332">
       <c r="A1332" t="inlineStr">
         <is>
-          <t>OKVED_84_PrPostDeyt</t>
+          <t>OKVED_71_ProcPoDolgObyaz</t>
         </is>
       </c>
     </row>
     <row r="1333">
       <c r="A1333" t="inlineStr">
         <is>
-          <t>OKVED_85_ArendPlDeVsego</t>
+          <t>OKVED_71_NalogNaPri</t>
         </is>
       </c>
     </row>
     <row r="1334">
       <c r="A1334" t="inlineStr">
         <is>
-          <t>OKVED_85_PrPostDeyt</t>
+          <t>OKVED_74_ProcPoDolgObyaz</t>
         </is>
       </c>
     </row>
     <row r="1335">
       <c r="A1335" t="inlineStr">
         <is>
-          <t>OKVED_85_ArendPlDeVsego</t>
+          <t>OKVED_77_ProcPoDolgObyaz</t>
         </is>
       </c>
     </row>
     <row r="1336">
       <c r="A1336" t="inlineStr">
         <is>
-          <t>OKVED_85_PrPostDeyt</t>
+          <t>OKVED_79_NalogNaPri</t>
         </is>
       </c>
     </row>
     <row r="1337">
       <c r="A1337" t="inlineStr">
         <is>
-          <t>OKVED_88_OtProdDeVsego</t>
+          <t>OKVED_81_NalogNaPri</t>
         </is>
       </c>
     </row>
     <row r="1338">
       <c r="A1338" t="inlineStr">
         <is>
-          <t>OKVED_88_ArendPlDeVsego</t>
+          <t>OKVED_O_PostavPoSyrMatRabUsl</t>
         </is>
       </c>
     </row>
     <row r="1339">
       <c r="A1339" t="inlineStr">
         <is>
-          <t>OKVED_88_PrPostDeyt</t>
+          <t>OKVED_O_VSvyaziSOplTrudRab</t>
         </is>
       </c>
     </row>
     <row r="1340">
       <c r="A1340" t="inlineStr">
         <is>
-          <t>OKVED_R_OtProdDeVsego</t>
+          <t>OKVED_O_ProcPoDolgObyaz</t>
         </is>
       </c>
     </row>
     <row r="1341">
       <c r="A1341" t="inlineStr">
         <is>
-          <t>OKVED_R_ArendPlDeVsego</t>
+          <t>OKVED_84_PostavPoSyrMatRabUsl</t>
         </is>
       </c>
     </row>
     <row r="1342">
       <c r="A1342" t="inlineStr">
         <is>
-          <t>OKVED_R_PrPostDeyt</t>
+          <t>OKVED_84_VSvyaziSOplTrudRab</t>
         </is>
       </c>
     </row>
     <row r="1343">
       <c r="A1343" t="inlineStr">
         <is>
-          <t>OKVED_93_OtProdDeVsego</t>
+          <t>OKVED_84_ProcPoDolgObyaz</t>
         </is>
       </c>
     </row>
     <row r="1344">
       <c r="A1344" t="inlineStr">
         <is>
-          <t>OKVED_93_ArendPlDeVsego</t>
+          <t>OKVED_85_ProcPoDolgObyaz</t>
         </is>
       </c>
     </row>
     <row r="1345">
       <c r="A1345" t="inlineStr">
         <is>
-          <t>OKVED_93_PrPostDeyt</t>
+          <t>OKVED_85_NalogNaPri</t>
         </is>
       </c>
     </row>
     <row r="1346">
       <c r="A1346" t="inlineStr">
         <is>
-          <t>OKVED_S_ArendPlDeVsego</t>
+          <t>OKVED_85_ProcPoDolgObyaz</t>
         </is>
       </c>
     </row>
     <row r="1347">
       <c r="A1347" t="inlineStr">
         <is>
-          <t>OKVED_94_ArendPlDeVsego</t>
+          <t>OKVED_85_NalogNaPri</t>
         </is>
       </c>
     </row>
     <row r="1348">
       <c r="A1348" t="inlineStr">
         <is>
-          <t>OKVED_96_ArendPlDeVsego</t>
+          <t>OKVED_Q_ProcPoDolgObyaz</t>
         </is>
       </c>
     </row>
     <row r="1349">
       <c r="A1349" t="inlineStr">
         <is>
-          <t>OKVED_96_PrPostDeyt</t>
+          <t>OKVED_Q_NalogNaPri</t>
         </is>
       </c>
     </row>
     <row r="1350">
       <c r="A1350" t="inlineStr">
         <is>
-          <t>OKVED_11_ProcPoDolgObyaz</t>
+          <t>OKVED_R_PostavPoSyrMatRabUsl</t>
         </is>
       </c>
     </row>
     <row r="1351">
       <c r="A1351" t="inlineStr">
         <is>
-          <t>OKVED_32_ProcPoDolgObyaz</t>
+          <t>OKVED_R_VSvyaziSOplTrudRab</t>
         </is>
       </c>
     </row>
     <row r="1352">
       <c r="A1352" t="inlineStr">
         <is>
-          <t>OKVED_32_NalogNaPri</t>
+          <t>OKVED_R_ProcPoDolgObyaz</t>
         </is>
       </c>
     </row>
     <row r="1353">
       <c r="A1353" t="inlineStr">
         <is>
-          <t>OKVED_33_NalogNaPri</t>
+          <t>OKVED_R_NalogNaPri</t>
         </is>
       </c>
     </row>
     <row r="1354">
       <c r="A1354" t="inlineStr">
         <is>
-          <t>OKVED_36_ProcPoDolgObyaz</t>
+          <t>OKVED_93_PostavPoSyrMatRabUsl</t>
         </is>
       </c>
     </row>
     <row r="1355">
       <c r="A1355" t="inlineStr">
         <is>
-          <t>OKVED_38_NalogNaPri</t>
+          <t>OKVED_93_VSvyaziSOplTrudRab</t>
         </is>
       </c>
     </row>
     <row r="1356">
       <c r="A1356" t="inlineStr">
         <is>
-          <t>OKVED_49_ProcPoDolgObyaz</t>
+          <t>OKVED_93_ProcPoDolgObyaz</t>
         </is>
       </c>
     </row>
     <row r="1357">
       <c r="A1357" t="inlineStr">
         <is>
-          <t>OKVED_56_ProcPoDolgObyaz</t>
+          <t>OKVED_93_NalogNaPri</t>
         </is>
       </c>
     </row>
     <row r="1358">
       <c r="A1358" t="inlineStr">
         <is>
-          <t>OKVED_56_NalogNaPri</t>
+          <t>OKVED_96_ProcPoDolgObyaz</t>
         </is>
       </c>
     </row>
     <row r="1359">
       <c r="A1359" t="inlineStr">
         <is>
-          <t>OKVED_J_ProcPoDolgObyaz</t>
+          <t>OKVED_96_NalogNaPri</t>
         </is>
       </c>
     </row>
     <row r="1360">
       <c r="A1360" t="inlineStr">
         <is>
-          <t>OKVED_J_NalogNaPri</t>
+          <t>OKVED_01_OtProdVneObAktKromeFinVlozh</t>
         </is>
       </c>
     </row>
     <row r="1361">
       <c r="A1361" t="inlineStr">
         <is>
-          <t>OKVED_63_ProcPoDolgObyaz</t>
+          <t>OKVED_01_OtProdAkcOrgDolUch</t>
         </is>
       </c>
     </row>
     <row r="1362">
       <c r="A1362" t="inlineStr">
         <is>
-          <t>OKVED_63_NalogNaPri</t>
+          <t>OKVED_01_DivProcDolgFinVlozh</t>
         </is>
       </c>
     </row>
     <row r="1363">
       <c r="A1363" t="inlineStr">
         <is>
-          <t>OKVED_M_ProcPoDolgObyaz</t>
+          <t>OKVED_B_OtProdAkcOrgDolUch</t>
         </is>
       </c>
     </row>
     <row r="1364">
       <c r="A1364" t="inlineStr">
         <is>
-          <t>OKVED_69_ProcPoDolgObyaz</t>
+          <t>OKVED_07_OtProdAkcOrgDolUch</t>
         </is>
       </c>
     </row>
     <row r="1365">
       <c r="A1365" t="inlineStr">
         <is>
-          <t>OKVED_69_NalogNaPri</t>
+          <t>OKVED_C_OtProdAkcOrgDolUch</t>
         </is>
       </c>
     </row>
     <row r="1366">
       <c r="A1366" t="inlineStr">
         <is>
-          <t>OKVED_71_ProcPoDolgObyaz</t>
+          <t>OKVED_10_OtProdAkcOrgDolUch</t>
         </is>
       </c>
     </row>
     <row r="1367">
       <c r="A1367" t="inlineStr">
         <is>
-          <t>OKVED_71_NalogNaPri</t>
+          <t>OKVED_11_OtProdVneObAktKromeFinVlozh</t>
         </is>
       </c>
     </row>
     <row r="1368">
       <c r="A1368" t="inlineStr">
         <is>
-          <t>OKVED_74_ProcPoDolgObyaz</t>
+          <t>OKVED_11_OtProdAkcOrgDolUch</t>
         </is>
       </c>
     </row>
     <row r="1369">
       <c r="A1369" t="inlineStr">
         <is>
-          <t>OKVED_77_ProcPoDolgObyaz</t>
+          <t>OKVED_11_OtProdFinVlozh</t>
         </is>
       </c>
     </row>
     <row r="1370">
       <c r="A1370" t="inlineStr">
         <is>
-          <t>OKVED_79_NalogNaPri</t>
+          <t>OKVED_35_OtProdAkcOrgDolUch</t>
         </is>
       </c>
     </row>
     <row r="1371">
       <c r="A1371" t="inlineStr">
         <is>
-          <t>OKVED_81_NalogNaPri</t>
+          <t>OKVED_35_OtProdAkcOrgDolUch</t>
         </is>
       </c>
     </row>
     <row r="1372">
       <c r="A1372" t="inlineStr">
         <is>
-          <t>OKVED_O_PostavPoSyrMatRabUsl</t>
+          <t>OKVED_E_OtProdAkcOrgDolUch</t>
         </is>
       </c>
     </row>
     <row r="1373">
       <c r="A1373" t="inlineStr">
         <is>
-          <t>OKVED_O_VSvyaziSOplTrudRab</t>
+          <t>OKVED_E_OtProdFinVlozh</t>
         </is>
       </c>
     </row>
     <row r="1374">
       <c r="A1374" t="inlineStr">
         <is>
-          <t>OKVED_O_ProcPoDolgObyaz</t>
+          <t>OKVED_E_DivProcDolgFinVlozh</t>
         </is>
       </c>
     </row>
     <row r="1375">
       <c r="A1375" t="inlineStr">
         <is>
-          <t>OKVED_84_PostavPoSyrMatRabUsl</t>
+          <t>OKVED_36_OtProdAkcOrgDolUch</t>
         </is>
       </c>
     </row>
     <row r="1376">
       <c r="A1376" t="inlineStr">
         <is>
-          <t>OKVED_84_VSvyaziSOplTrudRab</t>
+          <t>OKVED_36_OtProdFinVlozh</t>
         </is>
       </c>
     </row>
     <row r="1377">
       <c r="A1377" t="inlineStr">
         <is>
-          <t>OKVED_84_ProcPoDolgObyaz</t>
+          <t>OKVED_36_DivProcDolgFinVlozh</t>
         </is>
       </c>
     </row>
     <row r="1378">
       <c r="A1378" t="inlineStr">
         <is>
-          <t>OKVED_85_ProcPoDolgObyaz</t>
+          <t>OKVED_38_OtProdVneObAktKromeFinVlozh</t>
         </is>
       </c>
     </row>
     <row r="1379">
       <c r="A1379" t="inlineStr">
         <is>
-          <t>OKVED_85_NalogNaPri</t>
+          <t>OKVED_38_OtProdAkcOrgDolUch</t>
         </is>
       </c>
     </row>
     <row r="1380">
       <c r="A1380" t="inlineStr">
         <is>
-          <t>OKVED_85_ProcPoDolgObyaz</t>
+          <t>OKVED_38_OtProdFinVlozh</t>
         </is>
       </c>
     </row>
     <row r="1381">
       <c r="A1381" t="inlineStr">
         <is>
-          <t>OKVED_85_NalogNaPri</t>
+          <t>OKVED_38_DivProcDolgFinVlozh</t>
         </is>
       </c>
     </row>
     <row r="1382">
       <c r="A1382" t="inlineStr">
         <is>
-          <t>OKVED_Q_ProcPoDolgObyaz</t>
+          <t>OKVED_F_OtProdVneObAktKromeFinVlozh</t>
         </is>
       </c>
     </row>
     <row r="1383">
       <c r="A1383" t="inlineStr">
         <is>
-          <t>OKVED_Q_NalogNaPri</t>
+          <t>OKVED_F_OtProdAkcOrgDolUch</t>
         </is>
       </c>
     </row>
     <row r="1384">
       <c r="A1384" t="inlineStr">
         <is>
-          <t>OKVED_R_PostavPoSyrMatRabUsl</t>
+          <t>OKVED_41_OtProdVneObAktKromeFinVlozh</t>
         </is>
       </c>
     </row>
     <row r="1385">
       <c r="A1385" t="inlineStr">
         <is>
-          <t>OKVED_R_VSvyaziSOplTrudRab</t>
+          <t>OKVED_41_OtProdAkcOrgDolUch</t>
         </is>
       </c>
     </row>
     <row r="1386">
       <c r="A1386" t="inlineStr">
         <is>
-          <t>OKVED_R_ProcPoDolgObyaz</t>
+          <t>OKVED_43_OtProdVneObAktKromeFinVlozh</t>
         </is>
       </c>
     </row>
     <row r="1387">
       <c r="A1387" t="inlineStr">
         <is>
-          <t>OKVED_R_NalogNaPri</t>
+          <t>OKVED_43_OtProdAkcOrgDolUch</t>
         </is>
       </c>
     </row>
     <row r="1388">
       <c r="A1388" t="inlineStr">
         <is>
-          <t>OKVED_93_PostavPoSyrMatRabUsl</t>
+          <t>OKVED_43_OtProdFinVlozh</t>
         </is>
       </c>
     </row>
     <row r="1389">
       <c r="A1389" t="inlineStr">
         <is>
-          <t>OKVED_93_VSvyaziSOplTrudRab</t>
+          <t>OKVED_G_OtProdAkcOrgDolUch</t>
         </is>
       </c>
     </row>
     <row r="1390">
       <c r="A1390" t="inlineStr">
         <is>
-          <t>OKVED_93_ProcPoDolgObyaz</t>
+          <t>OKVED_46_OtProdAkcOrgDolUch</t>
         </is>
       </c>
     </row>
     <row r="1391">
       <c r="A1391" t="inlineStr">
         <is>
-          <t>OKVED_93_NalogNaPri</t>
+          <t>OKVED_47_OtProdAkcOrgDolUch</t>
         </is>
       </c>
     </row>
     <row r="1392">
       <c r="A1392" t="inlineStr">
         <is>
-          <t>OKVED_96_ProcPoDolgObyaz</t>
+          <t>OKVED_H_OtProdAkcOrgDolUch</t>
         </is>
       </c>
     </row>
     <row r="1393">
       <c r="A1393" t="inlineStr">
         <is>
-          <t>OKVED_96_NalogNaPri</t>
+          <t>OKVED_49_OtProdVneObAktKromeFinVlozh</t>
         </is>
       </c>
     </row>
     <row r="1394">
       <c r="A1394" t="inlineStr">
         <is>
-          <t>OKVED_01_OtProdVneObAktKromeFinVlozh</t>
+          <t>OKVED_49_OtProdAkcOrgDolUch</t>
         </is>
       </c>
     </row>
     <row r="1395">
       <c r="A1395" t="inlineStr">
         <is>
-          <t>OKVED_01_OtProdAkcOrgDolUch</t>
+          <t>OKVED_49_DivProcDolgFinVlozh</t>
         </is>
       </c>
     </row>
     <row r="1396">
       <c r="A1396" t="inlineStr">
         <is>
-          <t>OKVED_01_DivProcDolgFinVlozh</t>
+          <t>OKVED_52_OtProdAkcOrgDolUch</t>
         </is>
       </c>
     </row>
     <row r="1397">
       <c r="A1397" t="inlineStr">
         <is>
-          <t>OKVED_01_PrPostDeyt</t>
+          <t>OKVED_I_OtProdVneObAktKromeFinVlozh</t>
         </is>
       </c>
     </row>
     <row r="1398">
       <c r="A1398" t="inlineStr">
         <is>
-          <t>OKVED_B_OtProdAkcOrgDolUch</t>
+          <t>OKVED_I_OtProdAkcOrgDolUch</t>
         </is>
       </c>
     </row>
     <row r="1399">
       <c r="A1399" t="inlineStr">
         <is>
-          <t>OKVED_B_PrPostDeyt</t>
+          <t>OKVED_55_OtProdVneObAktKromeFinVlozh</t>
         </is>
       </c>
     </row>
     <row r="1400">
       <c r="A1400" t="inlineStr">
         <is>
-          <t>OKVED_07_OtProdAkcOrgDolUch</t>
+          <t>OKVED_55_OtProdAkcOrgDolUch</t>
         </is>
       </c>
     </row>
     <row r="1401">
       <c r="A1401" t="inlineStr">
         <is>
-          <t>OKVED_07_PrPostDeyt</t>
+          <t>OKVED_K_OtProdVneObAktKromeFinVlozh</t>
         </is>
       </c>
     </row>
     <row r="1402">
       <c r="A1402" t="inlineStr">
         <is>
-          <t>OKVED_C_OtProdAkcOrgDolUch</t>
+          <t>OKVED_K_OtProdAkcOrgDolUch</t>
         </is>
       </c>
     </row>
     <row r="1403">
       <c r="A1403" t="inlineStr">
         <is>
-          <t>OKVED_10_OtProdAkcOrgDolUch</t>
+          <t>OKVED_64_OtProdVneObAktKromeFinVlozh</t>
         </is>
       </c>
     </row>
     <row r="1404">
       <c r="A1404" t="inlineStr">
         <is>
-          <t>OKVED_11_OtProdVneObAktKromeFinVlozh</t>
+          <t>OKVED_64_OtProdAkcOrgDolUch</t>
         </is>
       </c>
     </row>
     <row r="1405">
       <c r="A1405" t="inlineStr">
         <is>
-          <t>OKVED_11_OtProdAkcOrgDolUch</t>
+          <t>OKVED_L_OtProdAkcOrgDolUch</t>
         </is>
       </c>
     </row>
     <row r="1406">
       <c r="A1406" t="inlineStr">
         <is>
-          <t>OKVED_11_OtProdFinVlozh</t>
+          <t>OKVED_M_OtProdVneObAktKromeFinVlozh</t>
         </is>
       </c>
     </row>
     <row r="1407">
       <c r="A1407" t="inlineStr">
         <is>
-          <t>OKVED_11_PrPostDeyt</t>
+          <t>OKVED_M_OtProdAkcOrgDolUch</t>
         </is>
       </c>
     </row>
     <row r="1408">
       <c r="A1408" t="inlineStr">
         <is>
-          <t>OKVED_35_OtProdAkcOrgDolUch</t>
+          <t>OKVED_70_OtProdVneObAktKromeFinVlozh</t>
         </is>
       </c>
     </row>
     <row r="1409">
       <c r="A1409" t="inlineStr">
         <is>
-          <t>OKVED_35_PrPostDeyt</t>
+          <t>OKVED_70_OtProdAkcOrgDolUch</t>
         </is>
       </c>
     </row>
     <row r="1410">
       <c r="A1410" t="inlineStr">
         <is>
-          <t>OKVED_35_OtProdAkcOrgDolUch</t>
+          <t>OKVED_71_OtProdVneObAktKromeFinVlozh</t>
         </is>
       </c>
     </row>
     <row r="1411">
       <c r="A1411" t="inlineStr">
         <is>
-          <t>OKVED_35_PrPostDeyt</t>
+          <t>OKVED_71_OtProdAkcOrgDolUch</t>
         </is>
       </c>
     </row>
     <row r="1412">
       <c r="A1412" t="inlineStr">
         <is>
-          <t>OKVED_E_OtProdAkcOrgDolUch</t>
+          <t>OKVED_71_DivProcDolgFinVlozh</t>
         </is>
       </c>
     </row>
     <row r="1413">
       <c r="A1413" t="inlineStr">
         <is>
-          <t>OKVED_E_OtProdFinVlozh</t>
+          <t>OKVED_N_OtProdAkcOrgDolUch</t>
         </is>
       </c>
     </row>
     <row r="1414">
       <c r="A1414" t="inlineStr">
         <is>
-          <t>OKVED_E_DivProcDolgFinVlozh</t>
+          <t>OKVED_N_OtProdFinVlozh</t>
         </is>
       </c>
     </row>
     <row r="1415">
       <c r="A1415" t="inlineStr">
         <is>
-          <t>OKVED_36_OtProdAkcOrgDolUch</t>
+          <t>OKVED_77_OtProdAkcOrgDolUch</t>
         </is>
       </c>
     </row>
     <row r="1416">
       <c r="A1416" t="inlineStr">
         <is>
-          <t>OKVED_36_OtProdFinVlozh</t>
+          <t>OKVED_77_OtProdFinVlozh</t>
         </is>
       </c>
     </row>
     <row r="1417">
       <c r="A1417" t="inlineStr">
         <is>
-          <t>OKVED_36_DivProcDolgFinVlozh</t>
+          <t>OKVED_S_OtProdVneObAktKromeFinVlozh</t>
         </is>
       </c>
     </row>
     <row r="1418">
       <c r="A1418" t="inlineStr">
         <is>
-          <t>OKVED_38_OtProdVneObAktKromeFinVlozh</t>
+          <t>OKVED_S_OtProdAkcOrgDolUch</t>
         </is>
       </c>
     </row>
     <row r="1419">
       <c r="A1419" t="inlineStr">
         <is>
-          <t>OKVED_38_OtProdAkcOrgDolUch</t>
+          <t>OKVED_S_DivProcDolgFinVlozh</t>
         </is>
       </c>
     </row>
     <row r="1420">
       <c r="A1420" t="inlineStr">
         <is>
-          <t>OKVED_38_OtProdFinVlozh</t>
+          <t>OKVED_94_OtProdVneObAktKromeFinVlozh</t>
         </is>
       </c>
     </row>
     <row r="1421">
       <c r="A1421" t="inlineStr">
         <is>
-          <t>OKVED_38_DivProcDolgFinVlozh</t>
+          <t>OKVED_94_OtProdAkcOrgDolUch</t>
         </is>
       </c>
     </row>
     <row r="1422">
       <c r="A1422" t="inlineStr">
         <is>
-          <t>OKVED_F_OtProdVneObAktKromeFinVlozh</t>
+          <t>OKVED_94_DivProcDolgFinVlozh</t>
         </is>
       </c>
     </row>
     <row r="1423">
       <c r="A1423" t="inlineStr">
         <is>
-          <t>OKVED_F_OtProdAkcOrgDolUch</t>
+          <t>OKVED_01_DolUch</t>
         </is>
       </c>
     </row>
     <row r="1424">
       <c r="A1424" t="inlineStr">
         <is>
-          <t>OKVED_41_OtProdVneObAktKromeFinVlozh</t>
+          <t>OKVED_01_PrCenBum</t>
         </is>
       </c>
     </row>
     <row r="1425">
       <c r="A1425" t="inlineStr">
         <is>
-          <t>OKVED_41_OtProdAkcOrgDolUch</t>
+          <t>OKVED_B_DolUch</t>
         </is>
       </c>
     </row>
     <row r="1426">
       <c r="A1426" t="inlineStr">
         <is>
-          <t>OKVED_43_OtProdVneObAktKromeFinVlozh</t>
+          <t>OKVED_B_ProcDolgObyazVklInvAkt</t>
         </is>
       </c>
     </row>
     <row r="1427">
       <c r="A1427" t="inlineStr">
         <is>
-          <t>OKVED_43_OtProdAkcOrgDolUch</t>
+          <t>OKVED_C_DolUch</t>
         </is>
       </c>
     </row>
     <row r="1428">
       <c r="A1428" t="inlineStr">
         <is>
-          <t>OKVED_43_OtProdFinVlozh</t>
+          <t>OKVED_C_ProcDolgObyazVklInvAkt</t>
         </is>
       </c>
     </row>
     <row r="1429">
       <c r="A1429" t="inlineStr">
         <is>
-          <t>OKVED_43_PrPostDeyt</t>
+          <t>OKVED_10_DolUch</t>
         </is>
       </c>
     </row>
     <row r="1430">
       <c r="A1430" t="inlineStr">
         <is>
-          <t>OKVED_G_OtProdAkcOrgDolUch</t>
+          <t>OKVED_10_ProcDolgObyazVklInvAkt</t>
         </is>
       </c>
     </row>
     <row r="1431">
       <c r="A1431" t="inlineStr">
         <is>
-          <t>OKVED_G_PrPostDeyt</t>
+          <t>OKVED_11_DolUch</t>
         </is>
       </c>
     </row>
     <row r="1432">
       <c r="A1432" t="inlineStr">
         <is>
-          <t>OKVED_46_OtProdAkcOrgDolUch</t>
+          <t>OKVED_11_PrCenBum</t>
         </is>
       </c>
     </row>
     <row r="1433">
       <c r="A1433" t="inlineStr">
         <is>
-          <t>OKVED_46_PrPostDeyt</t>
+          <t>OKVED_11_ProcDolgObyazVklInvAkt</t>
         </is>
       </c>
     </row>
     <row r="1434">
       <c r="A1434" t="inlineStr">
         <is>
-          <t>OKVED_47_OtProdAkcOrgDolUch</t>
+          <t>OKVED_33_DolUch</t>
         </is>
       </c>
     </row>
     <row r="1435">
       <c r="A1435" t="inlineStr">
         <is>
-          <t>OKVED_47_PrPostDeyt</t>
+          <t>OKVED_33_ProcDolgObyazVklInvAkt</t>
         </is>
       </c>
     </row>
     <row r="1436">
       <c r="A1436" t="inlineStr">
         <is>
-          <t>OKVED_H_OtProdAkcOrgDolUch</t>
+          <t>OKVED_E_DolUch</t>
         </is>
       </c>
     </row>
     <row r="1437">
       <c r="A1437" t="inlineStr">
         <is>
-          <t>OKVED_H_PrPostDeyt</t>
+          <t>OKVED_E_PrCenBum</t>
         </is>
       </c>
     </row>
     <row r="1438">
       <c r="A1438" t="inlineStr">
         <is>
-          <t>OKVED_49_OtProdVneObAktKromeFinVlozh</t>
+          <t>OKVED_E_ProcDolgObyazVklInvAkt</t>
         </is>
       </c>
     </row>
     <row r="1439">
       <c r="A1439" t="inlineStr">
         <is>
-          <t>OKVED_49_OtProdAkcOrgDolUch</t>
+          <t>OKVED_36_DolUch</t>
         </is>
       </c>
     </row>
     <row r="1440">
       <c r="A1440" t="inlineStr">
         <is>
-          <t>OKVED_49_DivProcDolgFinVlozh</t>
+          <t>OKVED_36_PrCenBum</t>
         </is>
       </c>
     </row>
     <row r="1441">
       <c r="A1441" t="inlineStr">
         <is>
-          <t>OKVED_49_PrPostDeyt</t>
+          <t>OKVED_36_ProcDolgObyazVklInvAkt</t>
         </is>
       </c>
     </row>
     <row r="1442">
       <c r="A1442" t="inlineStr">
         <is>
-          <t>OKVED_52_OtProdAkcOrgDolUch</t>
+          <t>OKVED_F_DolUch</t>
         </is>
       </c>
     </row>
     <row r="1443">
       <c r="A1443" t="inlineStr">
         <is>
-          <t>OKVED_52_PrPostDeyt</t>
+          <t>OKVED_F_ProcDolgObyazVklInvAkt</t>
         </is>
       </c>
     </row>
     <row r="1444">
       <c r="A1444" t="inlineStr">
         <is>
-          <t>OKVED_I_OtProdVneObAktKromeFinVlozh</t>
+          <t>OKVED_41_DolUch</t>
         </is>
       </c>
     </row>
     <row r="1445">
       <c r="A1445" t="inlineStr">
         <is>
-          <t>OKVED_I_OtProdAkcOrgDolUch</t>
+          <t>OKVED_41_ProcDolgObyazVklInvAkt</t>
         </is>
       </c>
     </row>
     <row r="1446">
       <c r="A1446" t="inlineStr">
         <is>
-          <t>OKVED_55_OtProdVneObAktKromeFinVlozh</t>
+          <t>OKVED_42_DolUch</t>
         </is>
       </c>
     </row>
     <row r="1447">
       <c r="A1447" t="inlineStr">
         <is>
-          <t>OKVED_55_OtProdAkcOrgDolUch</t>
+          <t>OKVED_42_ProcDolgObyazVklInvAkt</t>
         </is>
       </c>
     </row>
     <row r="1448">
       <c r="A1448" t="inlineStr">
         <is>
-          <t>OKVED_K_OtProdVneObAktKromeFinVlozh</t>
+          <t>OKVED_43_DolUch</t>
         </is>
       </c>
     </row>
     <row r="1449">
       <c r="A1449" t="inlineStr">
         <is>
-          <t>OKVED_K_OtProdAkcOrgDolUch</t>
+          <t>OKVED_43_PrCenBum</t>
         </is>
       </c>
     </row>
     <row r="1450">
       <c r="A1450" t="inlineStr">
         <is>
-          <t>OKVED_K_PrPostDeyt</t>
+          <t>OKVED_43_ProcDolgObyazVklInvAkt</t>
         </is>
       </c>
     </row>
     <row r="1451">
       <c r="A1451" t="inlineStr">
         <is>
-          <t>OKVED_64_OtProdVneObAktKromeFinVlozh</t>
+          <t>OKVED_47_DolUch</t>
         </is>
       </c>
     </row>
     <row r="1452">
       <c r="A1452" t="inlineStr">
         <is>
-          <t>OKVED_64_OtProdAkcOrgDolUch</t>
+          <t>OKVED_H_DolUch</t>
         </is>
       </c>
     </row>
     <row r="1453">
       <c r="A1453" t="inlineStr">
         <is>
-          <t>OKVED_64_PrPostDeyt</t>
+          <t>OKVED_H_ProcDolgObyazVklInvAkt</t>
         </is>
       </c>
     </row>
     <row r="1454">
       <c r="A1454" t="inlineStr">
         <is>
-          <t>OKVED_L_OtProdAkcOrgDolUch</t>
+          <t>OKVED_49_DolUch</t>
         </is>
       </c>
     </row>
     <row r="1455">
       <c r="A1455" t="inlineStr">
         <is>
-          <t>OKVED_M_OtProdVneObAktKromeFinVlozh</t>
+          <t>OKVED_49_ProcDolgObyazVklInvAkt</t>
         </is>
       </c>
     </row>
     <row r="1456">
       <c r="A1456" t="inlineStr">
         <is>
-          <t>OKVED_M_OtProdAkcOrgDolUch</t>
+          <t>OKVED_50_DolUch</t>
         </is>
       </c>
     </row>
     <row r="1457">
       <c r="A1457" t="inlineStr">
         <is>
-          <t>OKVED_M_PrPostDeyt</t>
+          <t>OKVED_50_PrCenBum</t>
         </is>
       </c>
     </row>
     <row r="1458">
       <c r="A1458" t="inlineStr">
         <is>
-          <t>OKVED_70_OtProdVneObAktKromeFinVlozh</t>
+          <t>OKVED_50_ProcDolgObyazVklInvAkt</t>
         </is>
       </c>
     </row>
     <row r="1459">
       <c r="A1459" t="inlineStr">
         <is>
-          <t>OKVED_70_OtProdAkcOrgDolUch</t>
+          <t>OKVED_52_DolUch</t>
         </is>
       </c>
     </row>
     <row r="1460">
       <c r="A1460" t="inlineStr">
         <is>
-          <t>OKVED_70_PrPostDeyt</t>
+          <t>OKVED_52_ProcDolgObyazVklInvAkt</t>
         </is>
       </c>
     </row>
     <row r="1461">
       <c r="A1461" t="inlineStr">
         <is>
-          <t>OKVED_71_OtProdVneObAktKromeFinVlozh</t>
+          <t>OKVED_I_ProcDolgObyazVklInvAkt</t>
         </is>
       </c>
     </row>
     <row r="1462">
       <c r="A1462" t="inlineStr">
         <is>
-          <t>OKVED_71_OtProdAkcOrgDolUch</t>
+          <t>OKVED_55_ProcDolgObyazVklInvAkt</t>
         </is>
       </c>
     </row>
     <row r="1463">
       <c r="A1463" t="inlineStr">
         <is>
-          <t>OKVED_71_DivProcDolgFinVlozh</t>
+          <t>OKVED_K_DolUch</t>
         </is>
       </c>
     </row>
     <row r="1464">
       <c r="A1464" t="inlineStr">
         <is>
-          <t>OKVED_71_PrPostDeyt</t>
+          <t>OKVED_K_ProcDolgObyazVklInvAkt</t>
         </is>
       </c>
     </row>
     <row r="1465">
       <c r="A1465" t="inlineStr">
         <is>
-          <t>OKVED_N_OtProdAkcOrgDolUch</t>
+          <t>OKVED_M_DolUch</t>
         </is>
       </c>
     </row>
     <row r="1466">
       <c r="A1466" t="inlineStr">
         <is>
-          <t>OKVED_N_OtProdFinVlozh</t>
+          <t>OKVED_71_DolUch</t>
         </is>
       </c>
     </row>
     <row r="1467">
       <c r="A1467" t="inlineStr">
         <is>
-          <t>OKVED_77_OtProdAkcOrgDolUch</t>
+          <t>OKVED_N_DolUch</t>
         </is>
       </c>
     </row>
     <row r="1468">
       <c r="A1468" t="inlineStr">
         <is>
-          <t>OKVED_77_OtProdFinVlozh</t>
+          <t>OKVED_N_PrCenBum</t>
         </is>
       </c>
     </row>
     <row r="1469">
       <c r="A1469" t="inlineStr">
         <is>
-          <t>OKVED_77_PrPostDeyt</t>
+          <t>OKVED_79_DolUch</t>
         </is>
       </c>
     </row>
     <row r="1470">
       <c r="A1470" t="inlineStr">
         <is>
-          <t>OKVED_S_OtProdVneObAktKromeFinVlozh</t>
+          <t>OKVED_79_PrCenBum</t>
         </is>
       </c>
     </row>
     <row r="1471">
       <c r="A1471" t="inlineStr">
         <is>
-          <t>OKVED_S_OtProdAkcOrgDolUch</t>
+          <t>OKVED_S_Modern</t>
         </is>
       </c>
     </row>
     <row r="1472">
       <c r="A1472" t="inlineStr">
         <is>
-          <t>OKVED_S_DivProcDolgFinVlozh</t>
+          <t>OKVED_S_DolUch</t>
         </is>
       </c>
     </row>
     <row r="1473">
       <c r="A1473" t="inlineStr">
         <is>
-          <t>OKVED_94_OtProdVneObAktKromeFinVlozh</t>
+          <t>OKVED_S_ProcDolgObyazVklInvAkt</t>
         </is>
       </c>
     </row>
     <row r="1474">
       <c r="A1474" t="inlineStr">
         <is>
-          <t>OKVED_94_OtProdAkcOrgDolUch</t>
+          <t>OKVED_94_Modern</t>
         </is>
       </c>
     </row>
     <row r="1475">
       <c r="A1475" t="inlineStr">
         <is>
-          <t>OKVED_94_DivProcDolgFinVlozh</t>
+          <t>OKVED_94_DolUch</t>
         </is>
       </c>
     </row>
     <row r="1476">
       <c r="A1476" t="inlineStr">
         <is>
-          <t>OKVED_01_DolUch</t>
+          <t>OKVED_94_ProcDolgObyazVklInvAkt</t>
         </is>
       </c>
     </row>
     <row r="1477">
       <c r="A1477" t="inlineStr">
         <is>
-          <t>OKVED_01_PrCenBum</t>
+          <t>OKVED_01_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1478">
       <c r="A1478" t="inlineStr">
         <is>
-          <t>OKVED_B_DolUch</t>
+          <t>OKVED_01_DrPost</t>
         </is>
       </c>
     </row>
     <row r="1479">
       <c r="A1479" t="inlineStr">
         <is>
-          <t>OKVED_B_ProcDolgObyazVklInvAkt</t>
+          <t>OKVED_B_PostDeyt</t>
         </is>
       </c>
     </row>
     <row r="1480">
       <c r="A1480" t="inlineStr">
         <is>
-          <t>OKVED_C_DolUch</t>
+          <t>OKVED_B_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1481">
       <c r="A1481" t="inlineStr">
         <is>
-          <t>OKVED_C_ProcDolgObyazVklInvAkt</t>
+          <t>OKVED_07_PostDeyt</t>
         </is>
       </c>
     </row>
     <row r="1482">
       <c r="A1482" t="inlineStr">
         <is>
-          <t>OKVED_10_DolUch</t>
+          <t>OKVED_07_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1483">
       <c r="A1483" t="inlineStr">
         <is>
-          <t>OKVED_10_ProcDolgObyazVklInvAkt</t>
+          <t>OKVED_C_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1484">
       <c r="A1484" t="inlineStr">
         <is>
-          <t>OKVED_11_DolUch</t>
+          <t>OKVED_10_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1485">
       <c r="A1485" t="inlineStr">
         <is>
-          <t>OKVED_11_PrCenBum</t>
+          <t>OKVED_32_PlCredit</t>
         </is>
       </c>
     </row>
     <row r="1486">
       <c r="A1486" t="inlineStr">
         <is>
-          <t>OKVED_11_ProcDolgObyazVklInvAkt</t>
+          <t>OKVED_32_PostDeyt</t>
         </is>
       </c>
     </row>
     <row r="1487">
       <c r="A1487" t="inlineStr">
         <is>
-          <t>OKVED_33_DolUch</t>
+          <t>OKVED_32_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1488">
       <c r="A1488" t="inlineStr">
         <is>
-          <t>OKVED_33_ProcDolgObyazVklInvAkt</t>
+          <t>OKVED_33_PostDeyt</t>
         </is>
       </c>
     </row>
     <row r="1489">
       <c r="A1489" t="inlineStr">
         <is>
-          <t>OKVED_E_DolUch</t>
+          <t>OKVED_33_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1490">
       <c r="A1490" t="inlineStr">
         <is>
-          <t>OKVED_E_PrCenBum</t>
+          <t>OKVED_33_DrPost</t>
         </is>
       </c>
     </row>
     <row r="1491">
       <c r="A1491" t="inlineStr">
         <is>
-          <t>OKVED_E_ProcDolgObyazVklInvAkt</t>
+          <t>OKVED_35_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1492">
       <c r="A1492" t="inlineStr">
         <is>
-          <t>OKVED_36_DolUch</t>
+          <t>OKVED_35_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1493">
       <c r="A1493" t="inlineStr">
         <is>
-          <t>OKVED_36_PrCenBum</t>
+          <t>OKVED_38_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1494">
       <c r="A1494" t="inlineStr">
         <is>
-          <t>OKVED_36_ProcDolgObyazVklInvAkt</t>
+          <t>OKVED_38_DrPost</t>
         </is>
       </c>
     </row>
     <row r="1495">
       <c r="A1495" t="inlineStr">
         <is>
-          <t>OKVED_F_DolUch</t>
+          <t>OKVED_F_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1496">
       <c r="A1496" t="inlineStr">
         <is>
-          <t>OKVED_F_ProcDolgObyazVklInvAkt</t>
+          <t>OKVED_41_PostDeyt</t>
         </is>
       </c>
     </row>
     <row r="1497">
       <c r="A1497" t="inlineStr">
         <is>
-          <t>OKVED_41_DolUch</t>
+          <t>OKVED_41_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1498">
       <c r="A1498" t="inlineStr">
         <is>
-          <t>OKVED_41_ProcDolgObyazVklInvAkt</t>
+          <t>OKVED_42_PostDeyt</t>
         </is>
       </c>
     </row>
     <row r="1499">
       <c r="A1499" t="inlineStr">
         <is>
-          <t>OKVED_42_DolUch</t>
+          <t>OKVED_42_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1500">
       <c r="A1500" t="inlineStr">
         <is>
-          <t>OKVED_42_ProcDolgObyazVklInvAkt</t>
+          <t>OKVED_42_DrPost</t>
         </is>
       </c>
     </row>
     <row r="1501">
       <c r="A1501" t="inlineStr">
         <is>
-          <t>OKVED_43_DolUch</t>
+          <t>OKVED_43_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1502">
       <c r="A1502" t="inlineStr">
         <is>
-          <t>OKVED_43_PrCenBum</t>
+          <t>OKVED_43_DrPost</t>
         </is>
       </c>
     </row>
     <row r="1503">
       <c r="A1503" t="inlineStr">
         <is>
-          <t>OKVED_43_ProcDolgObyazVklInvAkt</t>
+          <t>OKVED_G_PostDeyt</t>
         </is>
       </c>
     </row>
     <row r="1504">
       <c r="A1504" t="inlineStr">
         <is>
-          <t>OKVED_47_DolUch</t>
+          <t>OKVED_G_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1505">
       <c r="A1505" t="inlineStr">
         <is>
-          <t>OKVED_H_DolUch</t>
+          <t>OKVED_46_PostDeyt</t>
         </is>
       </c>
     </row>
     <row r="1506">
       <c r="A1506" t="inlineStr">
         <is>
-          <t>OKVED_H_ProcDolgObyazVklInvAkt</t>
+          <t>OKVED_46_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1507">
       <c r="A1507" t="inlineStr">
         <is>
-          <t>OKVED_49_DolUch</t>
+          <t>OKVED_47_PostDeyt</t>
         </is>
       </c>
     </row>
     <row r="1508">
       <c r="A1508" t="inlineStr">
         <is>
-          <t>OKVED_49_ProcDolgObyazVklInvAkt</t>
+          <t>OKVED_47_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1509">
       <c r="A1509" t="inlineStr">
         <is>
-          <t>OKVED_50_DolUch</t>
+          <t>OKVED_H_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1510">
       <c r="A1510" t="inlineStr">
         <is>
-          <t>OKVED_50_PrCenBum</t>
+          <t>OKVED_50_PostDeyt</t>
         </is>
       </c>
     </row>
     <row r="1511">
       <c r="A1511" t="inlineStr">
         <is>
-          <t>OKVED_50_ProcDolgObyazVklInvAkt</t>
+          <t>OKVED_50_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1512">
       <c r="A1512" t="inlineStr">
         <is>
-          <t>OKVED_52_DolUch</t>
+          <t>OKVED_50_DrPost</t>
         </is>
       </c>
     </row>
     <row r="1513">
       <c r="A1513" t="inlineStr">
         <is>
-          <t>OKVED_52_ProcDolgObyazVklInvAkt</t>
+          <t>OKVED_51_PostDeyt</t>
         </is>
       </c>
     </row>
     <row r="1514">
       <c r="A1514" t="inlineStr">
         <is>
-          <t>OKVED_I_ProcDolgObyazVklInvAkt</t>
+          <t>OKVED_51_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1515">
       <c r="A1515" t="inlineStr">
         <is>
-          <t>OKVED_55_ProcDolgObyazVklInvAkt</t>
+          <t>OKVED_51_DrPost</t>
         </is>
       </c>
     </row>
     <row r="1516">
       <c r="A1516" t="inlineStr">
         <is>
-          <t>OKVED_K_DolUch</t>
+          <t>OKVED_52_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1517">
       <c r="A1517" t="inlineStr">
         <is>
-          <t>OKVED_K_ProcDolgObyazVklInvAkt</t>
+          <t>OKVED_I_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1518">
       <c r="A1518" t="inlineStr">
         <is>
-          <t>OKVED_M_DolUch</t>
+          <t>OKVED_I_DrPost</t>
         </is>
       </c>
     </row>
     <row r="1519">
       <c r="A1519" t="inlineStr">
         <is>
-          <t>OKVED_71_DolUch</t>
+          <t>OKVED_55_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1520">
       <c r="A1520" t="inlineStr">
         <is>
-          <t>OKVED_N_DolUch</t>
+          <t>OKVED_55_DrPost</t>
         </is>
       </c>
     </row>
     <row r="1521">
       <c r="A1521" t="inlineStr">
         <is>
-          <t>OKVED_N_PrCenBum</t>
+          <t>OKVED_K_PostDeyt</t>
         </is>
       </c>
     </row>
     <row r="1522">
       <c r="A1522" t="inlineStr">
         <is>
-          <t>OKVED_79_DolUch</t>
+          <t>OKVED_K_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1523">
       <c r="A1523" t="inlineStr">
         <is>
-          <t>OKVED_79_PrCenBum</t>
+          <t>OKVED_K_DrPost</t>
         </is>
       </c>
     </row>
     <row r="1524">
       <c r="A1524" t="inlineStr">
         <is>
-          <t>OKVED_S_Modern</t>
+          <t>OKVED_64_PostDeyt</t>
         </is>
       </c>
     </row>
     <row r="1525">
       <c r="A1525" t="inlineStr">
         <is>
-          <t>OKVED_S_DolUch</t>
+          <t>OKVED_64_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1526">
       <c r="A1526" t="inlineStr">
         <is>
-          <t>OKVED_S_ProcDolgObyazVklInvAkt</t>
+          <t>OKVED_64_DrPost</t>
         </is>
       </c>
     </row>
     <row r="1527">
       <c r="A1527" t="inlineStr">
         <is>
-          <t>OKVED_94_Modern</t>
+          <t>OKVED_L_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1528">
       <c r="A1528" t="inlineStr">
         <is>
-          <t>OKVED_94_DolUch</t>
+          <t>OKVED_68_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1529">
       <c r="A1529" t="inlineStr">
         <is>
-          <t>OKVED_94_ProcDolgObyazVklInvAkt</t>
+          <t>OKVED_70_PlCredit</t>
         </is>
       </c>
     </row>
     <row r="1530">
       <c r="A1530" t="inlineStr">
         <is>
-          <t>OKVED_01_PostDeyt1</t>
+          <t>OKVED_70_PostDeyt</t>
         </is>
       </c>
     </row>
     <row r="1531">
       <c r="A1531" t="inlineStr">
         <is>
-          <t>OKVED_01_DrPost</t>
+          <t>OKVED_71_PostDeyt</t>
         </is>
       </c>
     </row>
     <row r="1532">
       <c r="A1532" t="inlineStr">
         <is>
-          <t>OKVED_B_PostDeyt</t>
+          <t>OKVED_74_PostDeyt</t>
         </is>
       </c>
     </row>
     <row r="1533">
       <c r="A1533" t="inlineStr">
         <is>
-          <t>OKVED_B_PostDeyt1</t>
+          <t>OKVED_74_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1534">
       <c r="A1534" t="inlineStr">
         <is>
-          <t>OKVED_07_PostDeyt</t>
+          <t>OKVED_74_DrPost</t>
         </is>
       </c>
     </row>
     <row r="1535">
       <c r="A1535" t="inlineStr">
         <is>
-          <t>OKVED_07_PostDeyt1</t>
+          <t>OKVED_N_PostDeyt</t>
         </is>
       </c>
     </row>
     <row r="1536">
       <c r="A1536" t="inlineStr">
         <is>
-          <t>OKVED_C_PostDeyt1</t>
+          <t>OKVED_N_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1537">
       <c r="A1537" t="inlineStr">
         <is>
-          <t>OKVED_10_PostDeyt1</t>
+          <t>OKVED_79_PostDeyt</t>
         </is>
       </c>
     </row>
     <row r="1538">
       <c r="A1538" t="inlineStr">
         <is>
-          <t>OKVED_32_PlCredit</t>
+          <t>OKVED_79_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1539">
       <c r="A1539" t="inlineStr">
         <is>
-          <t>OKVED_32_PostDeyt</t>
+          <t>OKVED_79_DrPost</t>
         </is>
       </c>
     </row>
     <row r="1540">
       <c r="A1540" t="inlineStr">
         <is>
-          <t>OKVED_32_PostDeyt1</t>
+          <t>OKVED_81_PlCredit</t>
         </is>
       </c>
     </row>
     <row r="1541">
       <c r="A1541" t="inlineStr">
         <is>
-          <t>OKVED_33_PostDeyt</t>
+          <t>OKVED_81_PostDeyt</t>
         </is>
       </c>
     </row>
     <row r="1542">
       <c r="A1542" t="inlineStr">
         <is>
-          <t>OKVED_33_PostDeyt1</t>
+          <t>OKVED_81_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1543">
       <c r="A1543" t="inlineStr">
         <is>
-          <t>OKVED_33_DrPost</t>
+          <t>OKVED_S_PlCredit</t>
         </is>
       </c>
     </row>
     <row r="1544">
       <c r="A1544" t="inlineStr">
         <is>
-          <t>OKVED_35_PostDeyt1</t>
+          <t>OKVED_S_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1545">
       <c r="A1545" t="inlineStr">
         <is>
-          <t>OKVED_35_PostDeyt1</t>
+          <t>OKVED_94_PlCredit</t>
         </is>
       </c>
     </row>
     <row r="1546">
       <c r="A1546" t="inlineStr">
         <is>
-          <t>OKVED_38_PostDeyt1</t>
+          <t>OKVED_94_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1547">
       <c r="A1547" t="inlineStr">
         <is>
-          <t>OKVED_38_DrPost</t>
+          <t>OKVED_01_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1548">
       <c r="A1548" t="inlineStr">
         <is>
-          <t>OKVED_F_PostDeyt1</t>
+          <t>OKVED_01_PlPoFin2</t>
         </is>
       </c>
     </row>
     <row r="1549">
       <c r="A1549" t="inlineStr">
         <is>
-          <t>OKVED_41_PostDeyt</t>
+          <t>OKVED_B_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1550">
       <c r="A1550" t="inlineStr">
         <is>
-          <t>OKVED_41_PostDeyt1</t>
+          <t>OKVED_07_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1551">
       <c r="A1551" t="inlineStr">
         <is>
-          <t>OKVED_42_PostDeyt</t>
+          <t>OKVED_33_PlPoFin</t>
         </is>
       </c>
     </row>
     <row r="1552">
       <c r="A1552" t="inlineStr">
         <is>
-          <t>OKVED_42_PostDeyt1</t>
+          <t>OKVED_33_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1553">
       <c r="A1553" t="inlineStr">
         <is>
-          <t>OKVED_42_DrPost</t>
+          <t>OKVED_33_PlPoFin2</t>
         </is>
       </c>
     </row>
     <row r="1554">
       <c r="A1554" t="inlineStr">
         <is>
-          <t>OKVED_43_PostDeyt1</t>
+          <t>OKVED_33_PlPoFin3</t>
         </is>
       </c>
     </row>
     <row r="1555">
       <c r="A1555" t="inlineStr">
         <is>
-          <t>OKVED_43_DrPost</t>
+          <t>OKVED_35_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1556">
       <c r="A1556" t="inlineStr">
         <is>
-          <t>OKVED_G_PostDeyt</t>
+          <t>OKVED_35_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1557">
       <c r="A1557" t="inlineStr">
         <is>
-          <t>OKVED_G_PostDeyt1</t>
+          <t>OKVED_E_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1558">
       <c r="A1558" t="inlineStr">
         <is>
-          <t>OKVED_46_PostDeyt</t>
+          <t>OKVED_E_PlPoFin2</t>
         </is>
       </c>
     </row>
     <row r="1559">
       <c r="A1559" t="inlineStr">
         <is>
-          <t>OKVED_46_PostDeyt1</t>
+          <t>OKVED_38_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1560">
       <c r="A1560" t="inlineStr">
         <is>
-          <t>OKVED_47_PostDeyt</t>
+          <t>OKVED_38_PlPoFin2</t>
         </is>
       </c>
     </row>
     <row r="1561">
       <c r="A1561" t="inlineStr">
         <is>
-          <t>OKVED_47_PostDeyt1</t>
+          <t>OKVED_F_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1562">
       <c r="A1562" t="inlineStr">
         <is>
-          <t>OKVED_H_PostDeyt1</t>
+          <t>OKVED_41_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1563">
       <c r="A1563" t="inlineStr">
         <is>
-          <t>OKVED_50_PostDeyt</t>
+          <t>OKVED_43_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1564">
       <c r="A1564" t="inlineStr">
         <is>
-          <t>OKVED_50_PostDeyt1</t>
+          <t>OKVED_43_PlPoFin2</t>
         </is>
       </c>
     </row>
     <row r="1565">
       <c r="A1565" t="inlineStr">
         <is>
-          <t>OKVED_50_DrPost</t>
+          <t>OKVED_G_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1566">
       <c r="A1566" t="inlineStr">
         <is>
-          <t>OKVED_51_PostDeyt</t>
+          <t>OKVED_46_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1567">
       <c r="A1567" t="inlineStr">
         <is>
-          <t>OKVED_51_PostDeyt1</t>
+          <t>OKVED_47_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1568">
       <c r="A1568" t="inlineStr">
         <is>
-          <t>OKVED_51_DrPost</t>
+          <t>OKVED_H_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1569">
       <c r="A1569" t="inlineStr">
         <is>
-          <t>OKVED_52_PostDeyt1</t>
+          <t>OKVED_49_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1570">
       <c r="A1570" t="inlineStr">
         <is>
-          <t>OKVED_I_PostDeyt1</t>
+          <t>OKVED_49_PlPoFin2</t>
         </is>
       </c>
     </row>
     <row r="1571">
       <c r="A1571" t="inlineStr">
         <is>
-          <t>OKVED_I_DrPost</t>
+          <t>OKVED_50_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1572">
       <c r="A1572" t="inlineStr">
         <is>
-          <t>OKVED_55_PostDeyt1</t>
+          <t>OKVED_52_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1573">
       <c r="A1573" t="inlineStr">
         <is>
-          <t>OKVED_55_DrPost</t>
+          <t>OKVED_I_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1574">
       <c r="A1574" t="inlineStr">
         <is>
-          <t>OKVED_K_PostDeyt</t>
+          <t>OKVED_I_PlPoFin2</t>
         </is>
       </c>
     </row>
     <row r="1575">
       <c r="A1575" t="inlineStr">
         <is>
-          <t>OKVED_K_PostDeyt1</t>
+          <t>OKVED_55_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1576">
       <c r="A1576" t="inlineStr">
         <is>
-          <t>OKVED_K_DrPost</t>
+          <t>OKVED_55_PlPoFin2</t>
         </is>
       </c>
     </row>
     <row r="1577">
       <c r="A1577" t="inlineStr">
         <is>
-          <t>OKVED_64_PostDeyt</t>
+          <t>OKVED_K_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1578">
       <c r="A1578" t="inlineStr">
         <is>
-          <t>OKVED_64_PostDeyt1</t>
+          <t>OKVED_64_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1579">
       <c r="A1579" t="inlineStr">
         <is>
-          <t>OKVED_64_DrPost</t>
+          <t>OKVED_68_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1580">
       <c r="A1580" t="inlineStr">
         <is>
-          <t>OKVED_L_PostDeyt1</t>
+          <t>OKVED_M_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1581">
       <c r="A1581" t="inlineStr">
         <is>
-          <t>OKVED_68_PostDeyt1</t>
+          <t>OKVED_70_PlPoFin</t>
         </is>
       </c>
     </row>
     <row r="1582">
       <c r="A1582" t="inlineStr">
         <is>
-          <t>OKVED_70_PlCredit</t>
+          <t>OKVED_70_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1583">
       <c r="A1583" t="inlineStr">
         <is>
-          <t>OKVED_70_PostDeyt</t>
+          <t>OKVED_70_PlPoFin2</t>
         </is>
       </c>
     </row>
     <row r="1584">
       <c r="A1584" t="inlineStr">
         <is>
-          <t>OKVED_71_PostDeyt</t>
+          <t>OKVED_70_PlPoFin3</t>
         </is>
       </c>
     </row>
     <row r="1585">
       <c r="A1585" t="inlineStr">
         <is>
-          <t>OKVED_74_PostDeyt</t>
+          <t>OKVED_71_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1586">
       <c r="A1586" t="inlineStr">
         <is>
-          <t>OKVED_74_PostDeyt1</t>
+          <t>OKVED_74_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1587">
       <c r="A1587" t="inlineStr">
         <is>
-          <t>OKVED_74_DrPost</t>
+          <t>OKVED_74_PlPoFin2</t>
         </is>
       </c>
     </row>
     <row r="1588">
       <c r="A1588" t="inlineStr">
         <is>
-          <t>OKVED_N_PostDeyt</t>
+          <t>OKVED_74_PlPoFin3</t>
         </is>
       </c>
     </row>
     <row r="1589">
       <c r="A1589" t="inlineStr">
         <is>
-          <t>OKVED_N_PostDeyt1</t>
+          <t>OKVED_74_SaldoDenPot</t>
         </is>
       </c>
     </row>
     <row r="1590">
       <c r="A1590" t="inlineStr">
         <is>
-          <t>OKVED_79_PostDeyt</t>
+          <t>OKVED_79_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1591">
       <c r="A1591" t="inlineStr">
         <is>
-          <t>OKVED_79_PostDeyt1</t>
+          <t>OKVED_79_PlPoFin2</t>
         </is>
       </c>
     </row>
     <row r="1592">
       <c r="A1592" t="inlineStr">
         <is>
-          <t>OKVED_79_DrPost</t>
+          <t>OKVED_81_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1593">
       <c r="A1593" t="inlineStr">
         <is>
-          <t>OKVED_81_PlCredit</t>
+          <t>OKVED_81_PlPoFin2</t>
         </is>
       </c>
     </row>
     <row r="1594">
       <c r="A1594" t="inlineStr">
         <is>
-          <t>OKVED_81_PostDeyt</t>
+          <t>OKVED_81_PlPoFin3</t>
         </is>
       </c>
     </row>
     <row r="1595">
       <c r="A1595" t="inlineStr">
         <is>
-          <t>OKVED_81_PostDeyt1</t>
+          <t>OKVED_81_SaldoDenPot</t>
         </is>
       </c>
     </row>
     <row r="1596">
       <c r="A1596" t="inlineStr">
         <is>
-          <t>OKVED_S_PlCredit</t>
+          <t>OKVED_S_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1597">
       <c r="A1597" t="inlineStr">
         <is>
-          <t>OKVED_S_PostDeyt1</t>
+          <t>OKVED_S_PlPoFin2</t>
         </is>
       </c>
     </row>
     <row r="1598">
       <c r="A1598" t="inlineStr">
         <is>
-          <t>OKVED_94_PlCredit</t>
+          <t>OKVED_S_PlPoFin3</t>
         </is>
       </c>
     </row>
     <row r="1599">
       <c r="A1599" t="inlineStr">
         <is>
-          <t>OKVED_94_PostDeyt1</t>
+          <t>OKVED_94_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1600">
       <c r="A1600" t="inlineStr">
         <is>
-          <t>OKVED_01_PlPoFin1</t>
+          <t>OKVED_94_PlPoFin2</t>
         </is>
       </c>
     </row>
     <row r="1601">
       <c r="A1601" t="inlineStr">
         <is>
-          <t>OKVED_01_PlPoFin2</t>
+          <t>OKVED_94_PlPoFin3</t>
         </is>
       </c>
     </row>
     <row r="1602">
       <c r="A1602" t="inlineStr">
         <is>
-          <t>OKVED_B_PlPoFin1</t>
+          <t>OKVED_01_Velch</t>
         </is>
       </c>
     </row>
     <row r="1603">
       <c r="A1603" t="inlineStr">
         <is>
-          <t>OKVED_07_PlPoFin1</t>
+          <t>OKVED_11_Velch</t>
         </is>
       </c>
     </row>
     <row r="1604">
       <c r="A1604" t="inlineStr">
         <is>
-          <t>OKVED_33_PlPoFin</t>
+          <t>OKVED_32_Velch</t>
         </is>
       </c>
     </row>
     <row r="1605">
       <c r="A1605" t="inlineStr">
         <is>
-          <t>OKVED_33_PlPoFin1</t>
+          <t>OKVED_33_Velch</t>
         </is>
       </c>
     </row>
     <row r="1606">
       <c r="A1606" t="inlineStr">
         <is>
-          <t>OKVED_33_PlPoFin2</t>
+          <t>OKVED_E_Velch</t>
         </is>
       </c>
     </row>
     <row r="1607">
       <c r="A1607" t="inlineStr">
         <is>
-          <t>OKVED_33_PlPoFin3</t>
+          <t>OKVED_38_Velch</t>
         </is>
       </c>
     </row>
     <row r="1608">
       <c r="A1608" t="inlineStr">
         <is>
-          <t>OKVED_35_PlPoFin1</t>
+          <t>OKVED_F_Velch</t>
         </is>
       </c>
     </row>
     <row r="1609">
       <c r="A1609" t="inlineStr">
         <is>
-          <t>OKVED_35_PlPoFin1</t>
+          <t>OKVED_41_Velch</t>
         </is>
       </c>
     </row>
     <row r="1610">
       <c r="A1610" t="inlineStr">
         <is>
-          <t>OKVED_E_PlPoFin1</t>
+          <t>OKVED_42_Velch</t>
         </is>
       </c>
     </row>
     <row r="1611">
       <c r="A1611" t="inlineStr">
         <is>
-          <t>OKVED_E_PlPoFin2</t>
+          <t>OKVED_43_Velch</t>
         </is>
       </c>
     </row>
     <row r="1612">
       <c r="A1612" t="inlineStr">
         <is>
-          <t>OKVED_38_PlPoFin1</t>
+          <t>OKVED_47_Velch</t>
         </is>
       </c>
     </row>
     <row r="1613">
       <c r="A1613" t="inlineStr">
         <is>
-          <t>OKVED_38_PlPoFin2</t>
+          <t>OKVED_49_Velch</t>
         </is>
       </c>
     </row>
     <row r="1614">
       <c r="A1614" t="inlineStr">
         <is>
-          <t>OKVED_F_PlPoFin1</t>
+          <t>OKVED_I_Velch</t>
         </is>
       </c>
     </row>
     <row r="1615">
       <c r="A1615" t="inlineStr">
         <is>
-          <t>OKVED_41_PlPoFin1</t>
+          <t>OKVED_56_Velch</t>
         </is>
       </c>
     </row>
     <row r="1616">
       <c r="A1616" t="inlineStr">
         <is>
-          <t>OKVED_43_PlPoFin1</t>
+          <t>OKVED_J_Velch</t>
         </is>
       </c>
     </row>
     <row r="1617">
       <c r="A1617" t="inlineStr">
         <is>
-          <t>OKVED_43_PlPoFin2</t>
+          <t>OKVED_63_Velch</t>
         </is>
       </c>
     </row>
     <row r="1618">
       <c r="A1618" t="inlineStr">
         <is>
-          <t>OKVED_G_PlPoFin1</t>
+          <t>OKVED_L_Velch</t>
         </is>
       </c>
     </row>
     <row r="1619">
       <c r="A1619" t="inlineStr">
         <is>
-          <t>OKVED_46_PlPoFin1</t>
+          <t>OKVED_68_Velch</t>
         </is>
       </c>
     </row>
     <row r="1620">
       <c r="A1620" t="inlineStr">
         <is>
-          <t>OKVED_47_PlPoFin1</t>
+          <t>OKVED_M_Velch</t>
         </is>
       </c>
     </row>
     <row r="1621">
       <c r="A1621" t="inlineStr">
         <is>
-          <t>OKVED_H_PlPoFin1</t>
+          <t>OKVED_69_Velch</t>
         </is>
       </c>
     </row>
     <row r="1622">
       <c r="A1622" t="inlineStr">
         <is>
-          <t>OKVED_49_PlPoFin1</t>
+          <t>OKVED_70_Velch</t>
         </is>
       </c>
     </row>
     <row r="1623">
       <c r="A1623" t="inlineStr">
         <is>
-          <t>OKVED_49_PlPoFin2</t>
+          <t>OKVED_71_Velch</t>
         </is>
       </c>
     </row>
     <row r="1624">
       <c r="A1624" t="inlineStr">
         <is>
-          <t>OKVED_50_PlPoFin1</t>
+          <t>OKVED_N_Velch</t>
         </is>
       </c>
     </row>
     <row r="1625">
       <c r="A1625" t="inlineStr">
         <is>
-          <t>OKVED_52_PlPoFin1</t>
+          <t>OKVED_77_Velch</t>
         </is>
       </c>
     </row>
     <row r="1626">
       <c r="A1626" t="inlineStr">
         <is>
-          <t>OKVED_I_PlPoFin1</t>
+          <t>OKVED_79_Velch</t>
         </is>
       </c>
     </row>
     <row r="1627">
       <c r="A1627" t="inlineStr">
         <is>
-          <t>OKVED_I_PlPoFin2</t>
+          <t>OKVED_81_Velch</t>
         </is>
       </c>
     </row>
     <row r="1628">
       <c r="A1628" t="inlineStr">
         <is>
-          <t>OKVED_55_PlPoFin1</t>
+          <t>OKVED_82_Velch</t>
         </is>
       </c>
     </row>
     <row r="1629">
       <c r="A1629" t="inlineStr">
         <is>
-          <t>OKVED_55_PlPoFin2</t>
+          <t>OKVED_O_Velch</t>
         </is>
       </c>
     </row>
     <row r="1630">
       <c r="A1630" t="inlineStr">
         <is>
-          <t>OKVED_K_PlPoFin1</t>
+          <t>OKVED_84_Velch</t>
         </is>
       </c>
     </row>
     <row r="1631">
       <c r="A1631" t="inlineStr">
         <is>
-          <t>OKVED_64_PlPoFin1</t>
+          <t>OKVED_85_Velch</t>
         </is>
       </c>
     </row>
     <row r="1632">
       <c r="A1632" t="inlineStr">
         <is>
-          <t>OKVED_68_PlPoFin1</t>
+          <t>OKVED_85_Velch</t>
         </is>
       </c>
     </row>
     <row r="1633">
       <c r="A1633" t="inlineStr">
         <is>
-          <t>OKVED_M_PlPoFin1</t>
+          <t>OKVED_88_Velch</t>
         </is>
       </c>
     </row>
     <row r="1634">
       <c r="A1634" t="inlineStr">
         <is>
-          <t>OKVED_70_PlPoFin</t>
+          <t>OKVED_R_Velch</t>
         </is>
       </c>
     </row>
     <row r="1635">
       <c r="A1635" t="inlineStr">
         <is>
-          <t>OKVED_70_PlPoFin1</t>
+          <t>OKVED_93_Velch</t>
         </is>
       </c>
     </row>
     <row r="1636">
       <c r="A1636" t="inlineStr">
         <is>
-          <t>OKVED_70_PlPoFin2</t>
+          <t>OKVED_S_Velch</t>
         </is>
       </c>
     </row>
     <row r="1637">
       <c r="A1637" t="inlineStr">
         <is>
-          <t>OKVED_70_PlPoFin3</t>
+          <t>OKVED_94_Velch</t>
         </is>
       </c>
     </row>
     <row r="1638">
       <c r="A1638" t="inlineStr">
         <is>
-          <t>OKVED_71_PlPoFin1</t>
+          <t>OKVED_96_Velch</t>
         </is>
       </c>
     </row>
     <row r="1639">
       <c r="A1639" t="inlineStr">
         <is>
-          <t>OKVED_74_PlPoFin1</t>
+          <t>OKVED_43_UstKap</t>
         </is>
       </c>
     </row>
     <row r="1640">
       <c r="A1640" t="inlineStr">
         <is>
-          <t>OKVED_74_PlPoFin2</t>
+          <t>OKVED_43_ChiAkt</t>
         </is>
       </c>
     </row>
     <row r="1641">
       <c r="A1641" t="inlineStr">
         <is>
-          <t>OKVED_74_PlPoFin3</t>
+          <t>OKVED_J_UstKap</t>
         </is>
       </c>
     </row>
     <row r="1642">
       <c r="A1642" t="inlineStr">
         <is>
-          <t>OKVED_74_SaldoDenPot</t>
+          <t>OKVED_J_Pri(ubOtPro</t>
         </is>
       </c>
     </row>
     <row r="1643">
       <c r="A1643" t="inlineStr">
         <is>
-          <t>OKVED_79_PlPoFin1</t>
+          <t>OKVED_J_ChiPri(ubOtcPer</t>
         </is>
       </c>
     </row>
     <row r="1644">
       <c r="A1644" t="inlineStr">
         <is>
-          <t>OKVED_79_PlPoFin2</t>
+          <t>OKVED_J_PriUby(-DoNalKChiAktV%</t>
         </is>
       </c>
     </row>
     <row r="1645">
       <c r="A1645" t="inlineStr">
         <is>
-          <t>OKVED_81_PlPoFin1</t>
+          <t>OKVED_63_UstKap</t>
         </is>
       </c>
     </row>
     <row r="1646">
       <c r="A1646" t="inlineStr">
         <is>
-          <t>OKVED_81_PlPoFin2</t>
+          <t>OKVED_63_Pri(ubOtPro</t>
         </is>
       </c>
     </row>
     <row r="1647">
       <c r="A1647" t="inlineStr">
         <is>
-          <t>OKVED_81_PlPoFin3</t>
+          <t>OKVED_63_ChiPri(ubOtcPer</t>
         </is>
       </c>
     </row>
     <row r="1648">
       <c r="A1648" t="inlineStr">
         <is>
-          <t>OKVED_81_SaldoDenPot</t>
+          <t>OKVED_63_PriUby(-DoNalKChiAktV%</t>
         </is>
       </c>
     </row>
     <row r="1649">
       <c r="A1649" t="inlineStr">
         <is>
-          <t>OKVED_S_PlPoFin1</t>
+          <t>OKVED_69_UstKap</t>
         </is>
       </c>
     </row>
     <row r="1650">
       <c r="A1650" t="inlineStr">
         <is>
-          <t>OKVED_S_PlPoFin2</t>
+          <t>OKVED_69_ChiAkt</t>
         </is>
       </c>
     </row>
     <row r="1651">
       <c r="A1651" t="inlineStr">
         <is>
-          <t>OKVED_S_PlPoFin3</t>
+          <t>OKVED_O_UstKap</t>
         </is>
       </c>
     </row>
     <row r="1652">
       <c r="A1652" t="inlineStr">
         <is>
-          <t>OKVED_94_PlPoFin1</t>
+          <t>OKVED_84_UstKap</t>
         </is>
       </c>
     </row>
     <row r="1653">
       <c r="A1653" t="inlineStr">
         <is>
-          <t>OKVED_94_PlPoFin2</t>
+          <t>OKVED_85_UstKap</t>
         </is>
       </c>
     </row>
     <row r="1654">
       <c r="A1654" t="inlineStr">
         <is>
-          <t>OKVED_94_PlPoFin3</t>
+          <t>OKVED_Q_UstKap</t>
         </is>
       </c>
     </row>
     <row r="1655">
       <c r="A1655" t="inlineStr">
         <is>
-          <t>OKVED_01_Velch</t>
+          <t>OKVED_Q_Pri(ubOtPro</t>
         </is>
       </c>
     </row>
     <row r="1656">
       <c r="A1656" t="inlineStr">
         <is>
-          <t>OKVED_11_Velch</t>
+          <t>OKVED_Q_ChiPri(ubOtcPer</t>
         </is>
       </c>
     </row>
     <row r="1657">
       <c r="A1657" t="inlineStr">
         <is>
-          <t>OKVED_32_Velch</t>
+          <t>OKVED_Q_PriUby(-DoNalKChiAktV%</t>
         </is>
       </c>
     </row>
     <row r="1658">
       <c r="A1658" t="inlineStr">
         <is>
-          <t>OKVED_33_Velch</t>
+          <t>OKVED_88_UstKap</t>
         </is>
       </c>
     </row>
     <row r="1659">
       <c r="A1659" t="inlineStr">
         <is>
-          <t>OKVED_E_Velch</t>
+          <t>OKVED_88_Pri(ubOtPro</t>
         </is>
       </c>
     </row>
     <row r="1660">
       <c r="A1660" t="inlineStr">
         <is>
-          <t>OKVED_38_Velch</t>
+          <t>OKVED_88_ChiPri(ubOtcPer</t>
         </is>
       </c>
     </row>
     <row r="1661">
       <c r="A1661" t="inlineStr">
-        <is>
-          <t>OKVED_F_Velch</t>
-        </is>
-      </c>
-    </row>
-    <row r="1662">
-      <c r="A1662" t="inlineStr">
-        <is>
-          <t>OKVED_41_Velch</t>
-        </is>
-      </c>
-    </row>
-    <row r="1663">
-      <c r="A1663" t="inlineStr">
-        <is>
-          <t>OKVED_42_Velch</t>
-        </is>
-      </c>
-    </row>
-    <row r="1664">
-      <c r="A1664" t="inlineStr">
-        <is>
-          <t>OKVED_43_Velch</t>
-        </is>
-      </c>
-    </row>
-    <row r="1665">
-      <c r="A1665" t="inlineStr">
-        <is>
-          <t>OKVED_47_Velch</t>
-        </is>
-      </c>
-    </row>
-    <row r="1666">
-      <c r="A1666" t="inlineStr">
-        <is>
-          <t>OKVED_49_Velch</t>
-        </is>
-      </c>
-    </row>
-    <row r="1667">
-      <c r="A1667" t="inlineStr">
-        <is>
-          <t>OKVED_I_Velch</t>
-        </is>
-      </c>
-    </row>
-    <row r="1668">
-      <c r="A1668" t="inlineStr">
-        <is>
-          <t>OKVED_56_Velch</t>
-        </is>
-      </c>
-    </row>
-    <row r="1669">
-      <c r="A1669" t="inlineStr">
-        <is>
-          <t>OKVED_J_Velch</t>
-        </is>
-      </c>
-    </row>
-    <row r="1670">
-      <c r="A1670" t="inlineStr">
-        <is>
-          <t>OKVED_63_Velch</t>
-        </is>
-      </c>
-    </row>
-    <row r="1671">
-      <c r="A1671" t="inlineStr">
-        <is>
-          <t>OKVED_L_Velch</t>
-        </is>
-      </c>
-    </row>
-    <row r="1672">
-      <c r="A1672" t="inlineStr">
-        <is>
-          <t>OKVED_68_Velch</t>
-        </is>
-      </c>
-    </row>
-    <row r="1673">
-      <c r="A1673" t="inlineStr">
-        <is>
-          <t>OKVED_M_Velch</t>
-        </is>
-      </c>
-    </row>
-    <row r="1674">
-      <c r="A1674" t="inlineStr">
-        <is>
-          <t>OKVED_69_Velch</t>
-        </is>
-      </c>
-    </row>
-    <row r="1675">
-      <c r="A1675" t="inlineStr">
-        <is>
-          <t>OKVED_70_Velch</t>
-        </is>
-      </c>
-    </row>
-    <row r="1676">
-      <c r="A1676" t="inlineStr">
-        <is>
-          <t>OKVED_71_Velch</t>
-        </is>
-      </c>
-    </row>
-    <row r="1677">
-      <c r="A1677" t="inlineStr">
-        <is>
-          <t>OKVED_N_Velch</t>
-        </is>
-      </c>
-    </row>
-    <row r="1678">
-      <c r="A1678" t="inlineStr">
-        <is>
-          <t>OKVED_77_Velch</t>
-        </is>
-      </c>
-    </row>
-    <row r="1679">
-      <c r="A1679" t="inlineStr">
-        <is>
-          <t>OKVED_79_Velch</t>
-        </is>
-      </c>
-    </row>
-    <row r="1680">
-      <c r="A1680" t="inlineStr">
-        <is>
-          <t>OKVED_81_Velch</t>
-        </is>
-      </c>
-    </row>
-    <row r="1681">
-      <c r="A1681" t="inlineStr">
-        <is>
-          <t>OKVED_82_Velch</t>
-        </is>
-      </c>
-    </row>
-    <row r="1682">
-      <c r="A1682" t="inlineStr">
-        <is>
-          <t>OKVED_O_Velch</t>
-        </is>
-      </c>
-    </row>
-    <row r="1683">
-      <c r="A1683" t="inlineStr">
-        <is>
-          <t>OKVED_84_Velch</t>
-        </is>
-      </c>
-    </row>
-    <row r="1684">
-      <c r="A1684" t="inlineStr">
-        <is>
-          <t>OKVED_85_Velch</t>
-        </is>
-      </c>
-    </row>
-    <row r="1685">
-      <c r="A1685" t="inlineStr">
-        <is>
-          <t>OKVED_85_Velch</t>
-        </is>
-      </c>
-    </row>
-    <row r="1686">
-      <c r="A1686" t="inlineStr">
-        <is>
-          <t>OKVED_88_Velch</t>
-        </is>
-      </c>
-    </row>
-    <row r="1687">
-      <c r="A1687" t="inlineStr">
-        <is>
-          <t>OKVED_R_Velch</t>
-        </is>
-      </c>
-    </row>
-    <row r="1688">
-      <c r="A1688" t="inlineStr">
-        <is>
-          <t>OKVED_93_Velch</t>
-        </is>
-      </c>
-    </row>
-    <row r="1689">
-      <c r="A1689" t="inlineStr">
-        <is>
-          <t>OKVED_S_Velch</t>
-        </is>
-      </c>
-    </row>
-    <row r="1690">
-      <c r="A1690" t="inlineStr">
-        <is>
-          <t>OKVED_94_Velch</t>
-        </is>
-      </c>
-    </row>
-    <row r="1691">
-      <c r="A1691" t="inlineStr">
-        <is>
-          <t>OKVED_96_Velch</t>
-        </is>
-      </c>
-    </row>
-    <row r="1692">
-      <c r="A1692" t="inlineStr">
-        <is>
-          <t>OKVED_43_UstKap</t>
-        </is>
-      </c>
-    </row>
-    <row r="1693">
-      <c r="A1693" t="inlineStr">
-        <is>
-          <t>OKVED_43_ChiAkt</t>
-        </is>
-      </c>
-    </row>
-    <row r="1694">
-      <c r="A1694" t="inlineStr">
-        <is>
-          <t>OKVED_J_UstKap</t>
-        </is>
-      </c>
-    </row>
-    <row r="1695">
-      <c r="A1695" t="inlineStr">
-        <is>
-          <t>OKVED_J_Pri(ubOtPro</t>
-        </is>
-      </c>
-    </row>
-    <row r="1696">
-      <c r="A1696" t="inlineStr">
-        <is>
-          <t>OKVED_J_ChiPri(ubOtcPer</t>
-        </is>
-      </c>
-    </row>
-    <row r="1697">
-      <c r="A1697" t="inlineStr">
-        <is>
-          <t>OKVED_J_PriUby(-DoNalKChiAktV%</t>
-        </is>
-      </c>
-    </row>
-    <row r="1698">
-      <c r="A1698" t="inlineStr">
-        <is>
-          <t>OKVED_63_UstKap</t>
-        </is>
-      </c>
-    </row>
-    <row r="1699">
-      <c r="A1699" t="inlineStr">
-        <is>
-          <t>OKVED_63_Pri(ubOtPro</t>
-        </is>
-      </c>
-    </row>
-    <row r="1700">
-      <c r="A1700" t="inlineStr">
-        <is>
-          <t>OKVED_63_ChiPri(ubOtcPer</t>
-        </is>
-      </c>
-    </row>
-    <row r="1701">
-      <c r="A1701" t="inlineStr">
-        <is>
-          <t>OKVED_63_PriUby(-DoNalKChiAktV%</t>
-        </is>
-      </c>
-    </row>
-    <row r="1702">
-      <c r="A1702" t="inlineStr">
-        <is>
-          <t>OKVED_69_UstKap</t>
-        </is>
-      </c>
-    </row>
-    <row r="1703">
-      <c r="A1703" t="inlineStr">
-        <is>
-          <t>OKVED_69_ChiAkt</t>
-        </is>
-      </c>
-    </row>
-    <row r="1704">
-      <c r="A1704" t="inlineStr">
-        <is>
-          <t>OKVED_O_UstKap</t>
-        </is>
-      </c>
-    </row>
-    <row r="1705">
-      <c r="A1705" t="inlineStr">
-        <is>
-          <t>OKVED_84_UstKap</t>
-        </is>
-      </c>
-    </row>
-    <row r="1706">
-      <c r="A1706" t="inlineStr">
-        <is>
-          <t>OKVED_85_UstKap</t>
-        </is>
-      </c>
-    </row>
-    <row r="1707">
-      <c r="A1707" t="inlineStr">
-        <is>
-          <t>OKVED_Q_UstKap</t>
-        </is>
-      </c>
-    </row>
-    <row r="1708">
-      <c r="A1708" t="inlineStr">
-        <is>
-          <t>OKVED_Q_Pri(ubOtPro</t>
-        </is>
-      </c>
-    </row>
-    <row r="1709">
-      <c r="A1709" t="inlineStr">
-        <is>
-          <t>OKVED_Q_ChiPri(ubOtcPer</t>
-        </is>
-      </c>
-    </row>
-    <row r="1710">
-      <c r="A1710" t="inlineStr">
-        <is>
-          <t>OKVED_Q_PriUby(-DoNalKChiAktV%</t>
-        </is>
-      </c>
-    </row>
-    <row r="1711">
-      <c r="A1711" t="inlineStr">
-        <is>
-          <t>OKVED_88_UstKap</t>
-        </is>
-      </c>
-    </row>
-    <row r="1712">
-      <c r="A1712" t="inlineStr">
-        <is>
-          <t>OKVED_88_Pri(ubOtPro</t>
-        </is>
-      </c>
-    </row>
-    <row r="1713">
-      <c r="A1713" t="inlineStr">
-        <is>
-          <t>OKVED_88_ChiPri(ubOtcPer</t>
-        </is>
-      </c>
-    </row>
-    <row r="1714">
-      <c r="A1714" t="inlineStr">
         <is>
           <t>OKVED_88_PriUby(-DoNalKChiAktV%</t>
         </is>

</xml_diff>

<commit_message>
Skip phantom gridSpan-duplicated cells in column matching
python-docx's row.cells repeats the same physical <w:tc> at every
grid position a merged (gridSpan>1) cell covers. _compute_section_mapping
iterated header_row.cells/year_row.cells directly, so a merged cell
was visited twice, advancing the "consumed" counter used to
disambiguate repeated header text (see _resolve_indicator) an extra
time. That misassigned the second sibling's indicator to the first
(merged) cell and left the real second cell's indicator marked as an
already-seen duplicate, dropping its tag entirely -- see table 19's
"в % к общей задолженности" columns (Дебиторская/Кредиторская).

Skip a cell when it's the same <w:tc> as the previous iteration's
cell before doing any matching, in both the has_years and non-year
branches.
</commit_message>
<xml_diff>
--- a/output/unfilled_tags.xlsx
+++ b/output/unfilled_tags.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1880"/>
+  <dimension ref="A1:A1881"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10331,14 +10331,14 @@
     <row r="1417">
       <c r="A1417" t="inlineStr">
         <is>
-          <t>OKVED_10_KoeTekLikDo&lt;10V%KObsZadKre</t>
+          <t>OKVED_10_KoeTekLikDo&lt;10KreZad</t>
         </is>
       </c>
     </row>
     <row r="1418">
       <c r="A1418" t="inlineStr">
         <is>
-          <t>OKVED_10_KoeTekLikDo&lt;10KreZad</t>
+          <t>OKVED_10_KoeTekLikDo&lt;10V%KObsZadKre</t>
         </is>
       </c>
     </row>
@@ -10366,7 +10366,7 @@
     <row r="1422">
       <c r="A1422" t="inlineStr">
         <is>
-          <t>OKVED_38_KoeTekLikDo&lt;10V%KObsZadKre</t>
+          <t>OKVED_38_KoeTekLikDo&lt;10V%KObsZad</t>
         </is>
       </c>
     </row>
@@ -10380,315 +10380,315 @@
     <row r="1424">
       <c r="A1424" t="inlineStr">
         <is>
-          <t>OKVED_70_KoeTekLikDo&lt;10KreZad</t>
+          <t>OKVED_38_KoeTekLikDo&lt;10V%KObsZadKre</t>
         </is>
       </c>
     </row>
     <row r="1425">
       <c r="A1425" t="inlineStr">
         <is>
-          <t>OKVED_70_KoeTekLikDo&lt;10V%KObsZadKre</t>
+          <t>OKVED_70_KoeTekLikDo&lt;10KreZad</t>
         </is>
       </c>
     </row>
     <row r="1426">
       <c r="A1426" t="inlineStr">
         <is>
-          <t>OKVED_R_KoeTekLikDo&lt;10KreZad</t>
+          <t>OKVED_70_KoeTekLikDo&lt;10V%KObsZadKre</t>
         </is>
       </c>
     </row>
     <row r="1427">
       <c r="A1427" t="inlineStr">
         <is>
-          <t>OKVED_R_KoeTekLikDo&lt;10V%KObsZadKre</t>
+          <t>OKVED_R_KoeTekLikDo&lt;10KreZad</t>
         </is>
       </c>
     </row>
     <row r="1428">
       <c r="A1428" t="inlineStr">
         <is>
-          <t>OKVED_93_KoeTekLikDo&lt;10KreZad</t>
+          <t>OKVED_R_KoeTekLikDo&lt;10V%KObsZadKre</t>
         </is>
       </c>
     </row>
     <row r="1429">
       <c r="A1429" t="inlineStr">
         <is>
-          <t>OKVED_93_KoeTekLikDo&lt;10V%KObsZadKre</t>
+          <t>OKVED_93_KoeTekLikDo&lt;10KreZad</t>
         </is>
       </c>
     </row>
     <row r="1430">
       <c r="A1430" t="inlineStr">
         <is>
-          <t>OKVED_94_KoeTekLikDo&lt;10KreZad</t>
+          <t>OKVED_93_KoeTekLikDo&lt;10V%KObsZadKre</t>
         </is>
       </c>
     </row>
     <row r="1431">
       <c r="A1431" t="inlineStr">
         <is>
-          <t>OKVED_94_KoeTekLikDo&lt;10V%KObsZadKre</t>
+          <t>OKVED_94_KoeTekLikDo&lt;10KreZad</t>
         </is>
       </c>
     </row>
     <row r="1432">
       <c r="A1432" t="inlineStr">
         <is>
-          <t>OKVED_96_KoeTekLikDo&lt;10DenSreIDenEkv</t>
+          <t>OKVED_94_KoeTekLikDo&lt;10V%KObsZadKre</t>
         </is>
       </c>
     </row>
     <row r="1433">
       <c r="A1433" t="inlineStr">
         <is>
-          <t>OKVED_96_KoeTekLikDo&lt;10V%KoVsDenSreDenEkv</t>
+          <t>OKVED_96_KoeTekLikDo&lt;10DenSreIDenEkv</t>
         </is>
       </c>
     </row>
     <row r="1434">
       <c r="A1434" t="inlineStr">
         <is>
-          <t>OKVED_42_KoeTekLikOt&gt;=20KolOrg(ed</t>
+          <t>OKVED_96_KoeTekLikDo&lt;10V%KoVsDenSreDenEkv</t>
         </is>
       </c>
     </row>
     <row r="1435">
       <c r="A1435" t="inlineStr">
         <is>
-          <t>OKVED_42_KoeTekLikOt&gt;=20V%KObsKol</t>
+          <t>OKVED_42_KoeTekLikOt&gt;=20KolOrg(ed</t>
         </is>
       </c>
     </row>
     <row r="1436">
       <c r="A1436" t="inlineStr">
         <is>
-          <t>OKVED_42_KoeTekLikOt&gt;=20DebZad</t>
+          <t>OKVED_42_KoeTekLikOt&gt;=20V%KObsKol</t>
         </is>
       </c>
     </row>
     <row r="1437">
       <c r="A1437" t="inlineStr">
         <is>
-          <t>OKVED_42_KoeTekLikOt&gt;=20V%KObsZad</t>
+          <t>OKVED_42_KoeTekLikOt&gt;=20DebZad</t>
         </is>
       </c>
     </row>
     <row r="1438">
       <c r="A1438" t="inlineStr">
         <is>
-          <t>OKVED_42_KoeTekLikOt&gt;=20KreZad</t>
+          <t>OKVED_42_KoeTekLikOt&gt;=20V%KObsZad</t>
         </is>
       </c>
     </row>
     <row r="1439">
       <c r="A1439" t="inlineStr">
         <is>
-          <t>OKVED_42_KoeTekLikOt&gt;=20V%KObsZadKre</t>
+          <t>OKVED_42_KoeTekLikOt&gt;=20KreZad</t>
         </is>
       </c>
     </row>
     <row r="1440">
       <c r="A1440" t="inlineStr">
         <is>
-          <t>OKVED_42_KoeTekLikOt&gt;=20DenSreIDenEkv</t>
+          <t>OKVED_42_KoeTekLikOt&gt;=20V%KObsZadKre</t>
         </is>
       </c>
     </row>
     <row r="1441">
       <c r="A1441" t="inlineStr">
         <is>
-          <t>OKVED_42_KoeTekLikOt&gt;=20V%KoVsDenSreDenEkv</t>
+          <t>OKVED_42_KoeTekLikOt&gt;=20DenSreIDenEkv</t>
         </is>
       </c>
     </row>
     <row r="1442">
       <c r="A1442" t="inlineStr">
         <is>
-          <t>OKVED_69_KoeTekLikOt&gt;=20DebZad</t>
+          <t>OKVED_42_KoeTekLikOt&gt;=20V%KoVsDenSreDenEkv</t>
         </is>
       </c>
     </row>
     <row r="1443">
       <c r="A1443" t="inlineStr">
         <is>
-          <t>OKVED_69_KoeTekLikOt&gt;=20V%KObsZad</t>
+          <t>OKVED_69_KoeTekLikOt&gt;=20DebZad</t>
         </is>
       </c>
     </row>
     <row r="1444">
       <c r="A1444" t="inlineStr">
         <is>
-          <t>OKVED_01_ArendPlDeVsego</t>
+          <t>OKVED_69_KoeTekLikOt&gt;=20V%KObsZad</t>
         </is>
       </c>
     </row>
     <row r="1445">
       <c r="A1445" t="inlineStr">
         <is>
-          <t>OKVED_32_ArendPlDeVsego</t>
+          <t>OKVED_01_ArendPlDeVsego</t>
         </is>
       </c>
     </row>
     <row r="1446">
       <c r="A1446" t="inlineStr">
         <is>
-          <t>OKVED_E_ArendPlDeVsego</t>
+          <t>OKVED_32_ArendPlDeVsego</t>
         </is>
       </c>
     </row>
     <row r="1447">
       <c r="A1447" t="inlineStr">
         <is>
-          <t>OKVED_36_ArendPlDeVsego</t>
+          <t>OKVED_E_ArendPlDeVsego</t>
         </is>
       </c>
     </row>
     <row r="1448">
       <c r="A1448" t="inlineStr">
         <is>
-          <t>OKVED_38_ArendPlDeVsego</t>
+          <t>OKVED_36_ArendPlDeVsego</t>
         </is>
       </c>
     </row>
     <row r="1449">
       <c r="A1449" t="inlineStr">
         <is>
-          <t>OKVED_41_ArendPlDeVsego</t>
+          <t>OKVED_38_ArendPlDeVsego</t>
         </is>
       </c>
     </row>
     <row r="1450">
       <c r="A1450" t="inlineStr">
         <is>
-          <t>OKVED_43_ArendPlDeVsego</t>
+          <t>OKVED_41_ArendPlDeVsego</t>
         </is>
       </c>
     </row>
     <row r="1451">
       <c r="A1451" t="inlineStr">
         <is>
-          <t>OKVED_49_ArendPlDeVsego</t>
+          <t>OKVED_43_ArendPlDeVsego</t>
         </is>
       </c>
     </row>
     <row r="1452">
       <c r="A1452" t="inlineStr">
         <is>
-          <t>OKVED_50_ArendPlDeVsego</t>
+          <t>OKVED_49_ArendPlDeVsego</t>
         </is>
       </c>
     </row>
     <row r="1453">
       <c r="A1453" t="inlineStr">
         <is>
-          <t>OKVED_I_ArendPlDeVsego</t>
+          <t>OKVED_50_ArendPlDeVsego</t>
         </is>
       </c>
     </row>
     <row r="1454">
       <c r="A1454" t="inlineStr">
         <is>
-          <t>OKVED_55_ArendPlDeVsego</t>
+          <t>OKVED_I_ArendPlDeVsego</t>
         </is>
       </c>
     </row>
     <row r="1455">
       <c r="A1455" t="inlineStr">
         <is>
-          <t>OKVED_56_ArendPlDeVsego</t>
+          <t>OKVED_55_ArendPlDeVsego</t>
         </is>
       </c>
     </row>
     <row r="1456">
       <c r="A1456" t="inlineStr">
         <is>
-          <t>OKVED_J_OtProdDeVsego</t>
+          <t>OKVED_56_ArendPlDeVsego</t>
         </is>
       </c>
     </row>
     <row r="1457">
       <c r="A1457" t="inlineStr">
         <is>
-          <t>OKVED_J_ArendPlDeVsego</t>
+          <t>OKVED_J_OtProdDeVsego</t>
         </is>
       </c>
     </row>
     <row r="1458">
       <c r="A1458" t="inlineStr">
         <is>
-          <t>OKVED_63_OtProdDeVsego</t>
+          <t>OKVED_J_ArendPlDeVsego</t>
         </is>
       </c>
     </row>
     <row r="1459">
       <c r="A1459" t="inlineStr">
         <is>
-          <t>OKVED_63_ArendPlDeVsego</t>
+          <t>OKVED_63_OtProdDeVsego</t>
         </is>
       </c>
     </row>
     <row r="1460">
       <c r="A1460" t="inlineStr">
         <is>
-          <t>OKVED_K_ArendPlDeVsego</t>
+          <t>OKVED_63_ArendPlDeVsego</t>
         </is>
       </c>
     </row>
     <row r="1461">
       <c r="A1461" t="inlineStr">
         <is>
-          <t>OKVED_64_ArendPlDeVsego</t>
+          <t>OKVED_K_ArendPlDeVsego</t>
         </is>
       </c>
     </row>
     <row r="1462">
       <c r="A1462" t="inlineStr">
         <is>
-          <t>OKVED_69_ArendPlDeVsego</t>
+          <t>OKVED_64_ArendPlDeVsego</t>
         </is>
       </c>
     </row>
     <row r="1463">
       <c r="A1463" t="inlineStr">
         <is>
-          <t>OKVED_79_ArendPlDeVsego</t>
+          <t>OKVED_69_ArendPlDeVsego</t>
         </is>
       </c>
     </row>
     <row r="1464">
       <c r="A1464" t="inlineStr">
         <is>
-          <t>OKVED_81_ArendPlDeVsego</t>
+          <t>OKVED_79_ArendPlDeVsego</t>
         </is>
       </c>
     </row>
     <row r="1465">
       <c r="A1465" t="inlineStr">
         <is>
-          <t>OKVED_82_ArendPlDeVsego</t>
+          <t>OKVED_81_ArendPlDeVsego</t>
         </is>
       </c>
     </row>
     <row r="1466">
       <c r="A1466" t="inlineStr">
         <is>
-          <t>OKVED_O_ArendPlDeVsego</t>
+          <t>OKVED_82_ArendPlDeVsego</t>
         </is>
       </c>
     </row>
     <row r="1467">
       <c r="A1467" t="inlineStr">
         <is>
-          <t>OKVED_84_ArendPlDeVsego</t>
+          <t>OKVED_O_ArendPlDeVsego</t>
         </is>
       </c>
     </row>
     <row r="1468">
       <c r="A1468" t="inlineStr">
         <is>
-          <t>OKVED_85_ArendPlDeVsego</t>
+          <t>OKVED_84_ArendPlDeVsego</t>
         </is>
       </c>
     </row>
@@ -10702,539 +10702,539 @@
     <row r="1470">
       <c r="A1470" t="inlineStr">
         <is>
-          <t>OKVED_Q_OtProdDeVsego</t>
+          <t>OKVED_85_ArendPlDeVsego</t>
         </is>
       </c>
     </row>
     <row r="1471">
       <c r="A1471" t="inlineStr">
         <is>
-          <t>OKVED_Q_ArendPlDeVsego</t>
+          <t>OKVED_Q_OtProdDeVsego</t>
         </is>
       </c>
     </row>
     <row r="1472">
       <c r="A1472" t="inlineStr">
         <is>
-          <t>OKVED_88_OtProdDeVsego</t>
+          <t>OKVED_Q_ArendPlDeVsego</t>
         </is>
       </c>
     </row>
     <row r="1473">
       <c r="A1473" t="inlineStr">
         <is>
-          <t>OKVED_88_ArendPlDeVsego</t>
+          <t>OKVED_88_OtProdDeVsego</t>
         </is>
       </c>
     </row>
     <row r="1474">
       <c r="A1474" t="inlineStr">
         <is>
-          <t>OKVED_R_OtProdDeVsego</t>
+          <t>OKVED_88_ArendPlDeVsego</t>
         </is>
       </c>
     </row>
     <row r="1475">
       <c r="A1475" t="inlineStr">
         <is>
-          <t>OKVED_R_ArendPlDeVsego</t>
+          <t>OKVED_R_OtProdDeVsego</t>
         </is>
       </c>
     </row>
     <row r="1476">
       <c r="A1476" t="inlineStr">
         <is>
-          <t>OKVED_93_OtProdDeVsego</t>
+          <t>OKVED_R_ArendPlDeVsego</t>
         </is>
       </c>
     </row>
     <row r="1477">
       <c r="A1477" t="inlineStr">
         <is>
-          <t>OKVED_93_ArendPlDeVsego</t>
+          <t>OKVED_93_OtProdDeVsego</t>
         </is>
       </c>
     </row>
     <row r="1478">
       <c r="A1478" t="inlineStr">
         <is>
-          <t>OKVED_S_ArendPlDeVsego</t>
+          <t>OKVED_93_ArendPlDeVsego</t>
         </is>
       </c>
     </row>
     <row r="1479">
       <c r="A1479" t="inlineStr">
         <is>
-          <t>OKVED_94_ArendPlDeVsego</t>
+          <t>OKVED_S_ArendPlDeVsego</t>
         </is>
       </c>
     </row>
     <row r="1480">
       <c r="A1480" t="inlineStr">
         <is>
-          <t>OKVED_96_ArendPlDeVsego</t>
+          <t>OKVED_94_ArendPlDeVsego</t>
         </is>
       </c>
     </row>
     <row r="1481">
       <c r="A1481" t="inlineStr">
         <is>
-          <t>OKVED_11_ProcPoDolgObyaz</t>
+          <t>OKVED_96_ArendPlDeVsego</t>
         </is>
       </c>
     </row>
     <row r="1482">
       <c r="A1482" t="inlineStr">
         <is>
-          <t>OKVED_32_ProcPoDolgObyaz</t>
+          <t>OKVED_11_ProcPoDolgObyaz</t>
         </is>
       </c>
     </row>
     <row r="1483">
       <c r="A1483" t="inlineStr">
         <is>
-          <t>OKVED_32_NalogNaPri</t>
+          <t>OKVED_32_ProcPoDolgObyaz</t>
         </is>
       </c>
     </row>
     <row r="1484">
       <c r="A1484" t="inlineStr">
         <is>
-          <t>OKVED_33_NalogNaPri</t>
+          <t>OKVED_32_NalogNaPri</t>
         </is>
       </c>
     </row>
     <row r="1485">
       <c r="A1485" t="inlineStr">
         <is>
-          <t>OKVED_36_ProcPoDolgObyaz</t>
+          <t>OKVED_33_NalogNaPri</t>
         </is>
       </c>
     </row>
     <row r="1486">
       <c r="A1486" t="inlineStr">
         <is>
-          <t>OKVED_38_NalogNaPri</t>
+          <t>OKVED_36_ProcPoDolgObyaz</t>
         </is>
       </c>
     </row>
     <row r="1487">
       <c r="A1487" t="inlineStr">
         <is>
-          <t>OKVED_49_ProcPoDolgObyaz</t>
+          <t>OKVED_38_NalogNaPri</t>
         </is>
       </c>
     </row>
     <row r="1488">
       <c r="A1488" t="inlineStr">
         <is>
-          <t>OKVED_56_ProcPoDolgObyaz</t>
+          <t>OKVED_49_ProcPoDolgObyaz</t>
         </is>
       </c>
     </row>
     <row r="1489">
       <c r="A1489" t="inlineStr">
         <is>
-          <t>OKVED_56_NalogNaPri</t>
+          <t>OKVED_56_ProcPoDolgObyaz</t>
         </is>
       </c>
     </row>
     <row r="1490">
       <c r="A1490" t="inlineStr">
         <is>
-          <t>OKVED_J_ProcPoDolgObyaz</t>
+          <t>OKVED_56_NalogNaPri</t>
         </is>
       </c>
     </row>
     <row r="1491">
       <c r="A1491" t="inlineStr">
         <is>
-          <t>OKVED_J_NalogNaPri</t>
+          <t>OKVED_J_ProcPoDolgObyaz</t>
         </is>
       </c>
     </row>
     <row r="1492">
       <c r="A1492" t="inlineStr">
         <is>
-          <t>OKVED_63_ProcPoDolgObyaz</t>
+          <t>OKVED_J_NalogNaPri</t>
         </is>
       </c>
     </row>
     <row r="1493">
       <c r="A1493" t="inlineStr">
         <is>
-          <t>OKVED_63_NalogNaPri</t>
+          <t>OKVED_63_ProcPoDolgObyaz</t>
         </is>
       </c>
     </row>
     <row r="1494">
       <c r="A1494" t="inlineStr">
         <is>
-          <t>OKVED_M_ProcPoDolgObyaz</t>
+          <t>OKVED_63_NalogNaPri</t>
         </is>
       </c>
     </row>
     <row r="1495">
       <c r="A1495" t="inlineStr">
         <is>
-          <t>OKVED_69_ProcPoDolgObyaz</t>
+          <t>OKVED_M_ProcPoDolgObyaz</t>
         </is>
       </c>
     </row>
     <row r="1496">
       <c r="A1496" t="inlineStr">
         <is>
-          <t>OKVED_69_NalogNaPri</t>
+          <t>OKVED_69_ProcPoDolgObyaz</t>
         </is>
       </c>
     </row>
     <row r="1497">
       <c r="A1497" t="inlineStr">
         <is>
-          <t>OKVED_70_ProcPoDolgObyaz</t>
+          <t>OKVED_69_NalogNaPri</t>
         </is>
       </c>
     </row>
     <row r="1498">
       <c r="A1498" t="inlineStr">
         <is>
-          <t>OKVED_71_ProcPoDolgObyaz</t>
+          <t>OKVED_70_ProcPoDolgObyaz</t>
         </is>
       </c>
     </row>
     <row r="1499">
       <c r="A1499" t="inlineStr">
         <is>
-          <t>OKVED_71_NalogNaPri</t>
+          <t>OKVED_71_ProcPoDolgObyaz</t>
         </is>
       </c>
     </row>
     <row r="1500">
       <c r="A1500" t="inlineStr">
         <is>
-          <t>OKVED_74_ProcPoDolgObyaz</t>
+          <t>OKVED_71_NalogNaPri</t>
         </is>
       </c>
     </row>
     <row r="1501">
       <c r="A1501" t="inlineStr">
         <is>
-          <t>OKVED_77_ProcPoDolgObyaz</t>
+          <t>OKVED_74_ProcPoDolgObyaz</t>
         </is>
       </c>
     </row>
     <row r="1502">
       <c r="A1502" t="inlineStr">
         <is>
-          <t>OKVED_79_NalogNaPri</t>
+          <t>OKVED_77_ProcPoDolgObyaz</t>
         </is>
       </c>
     </row>
     <row r="1503">
       <c r="A1503" t="inlineStr">
         <is>
-          <t>OKVED_81_NalogNaPri</t>
+          <t>OKVED_79_NalogNaPri</t>
         </is>
       </c>
     </row>
     <row r="1504">
       <c r="A1504" t="inlineStr">
         <is>
-          <t>OKVED_82_ProcPoDolgObyaz</t>
+          <t>OKVED_81_NalogNaPri</t>
         </is>
       </c>
     </row>
     <row r="1505">
       <c r="A1505" t="inlineStr">
         <is>
-          <t>OKVED_O_PostavPoSyrMatRabUsl</t>
+          <t>OKVED_82_ProcPoDolgObyaz</t>
         </is>
       </c>
     </row>
     <row r="1506">
       <c r="A1506" t="inlineStr">
         <is>
-          <t>OKVED_O_VSvyaziSOplTrudRab</t>
+          <t>OKVED_O_PostavPoSyrMatRabUsl</t>
         </is>
       </c>
     </row>
     <row r="1507">
       <c r="A1507" t="inlineStr">
         <is>
-          <t>OKVED_O_ProcPoDolgObyaz</t>
+          <t>OKVED_O_VSvyaziSOplTrudRab</t>
         </is>
       </c>
     </row>
     <row r="1508">
       <c r="A1508" t="inlineStr">
         <is>
-          <t>OKVED_84_PostavPoSyrMatRabUsl</t>
+          <t>OKVED_O_ProcPoDolgObyaz</t>
         </is>
       </c>
     </row>
     <row r="1509">
       <c r="A1509" t="inlineStr">
         <is>
-          <t>OKVED_84_VSvyaziSOplTrudRab</t>
+          <t>OKVED_84_PostavPoSyrMatRabUsl</t>
         </is>
       </c>
     </row>
     <row r="1510">
       <c r="A1510" t="inlineStr">
         <is>
-          <t>OKVED_84_ProcPoDolgObyaz</t>
+          <t>OKVED_84_VSvyaziSOplTrudRab</t>
         </is>
       </c>
     </row>
     <row r="1511">
       <c r="A1511" t="inlineStr">
         <is>
-          <t>OKVED_85_ProcPoDolgObyaz</t>
+          <t>OKVED_84_ProcPoDolgObyaz</t>
         </is>
       </c>
     </row>
     <row r="1512">
       <c r="A1512" t="inlineStr">
         <is>
-          <t>OKVED_85_NalogNaPri</t>
+          <t>OKVED_85_ProcPoDolgObyaz</t>
         </is>
       </c>
     </row>
     <row r="1513">
       <c r="A1513" t="inlineStr">
         <is>
-          <t>OKVED_85_ProcPoDolgObyaz</t>
+          <t>OKVED_85_NalogNaPri</t>
         </is>
       </c>
     </row>
     <row r="1514">
       <c r="A1514" t="inlineStr">
         <is>
-          <t>OKVED_85_NalogNaPri</t>
+          <t>OKVED_85_ProcPoDolgObyaz</t>
         </is>
       </c>
     </row>
     <row r="1515">
       <c r="A1515" t="inlineStr">
         <is>
-          <t>OKVED_Q_ProcPoDolgObyaz</t>
+          <t>OKVED_85_NalogNaPri</t>
         </is>
       </c>
     </row>
     <row r="1516">
       <c r="A1516" t="inlineStr">
         <is>
-          <t>OKVED_Q_NalogNaPri</t>
+          <t>OKVED_Q_ProcPoDolgObyaz</t>
         </is>
       </c>
     </row>
     <row r="1517">
       <c r="A1517" t="inlineStr">
         <is>
-          <t>OKVED_86_PlatPoTekDeVsego</t>
+          <t>OKVED_Q_NalogNaPri</t>
         </is>
       </c>
     </row>
     <row r="1518">
       <c r="A1518" t="inlineStr">
         <is>
-          <t>OKVED_86_PostavPoSyrMatRabUsl</t>
+          <t>OKVED_86_PlatPoTekDeVsego</t>
         </is>
       </c>
     </row>
     <row r="1519">
       <c r="A1519" t="inlineStr">
         <is>
-          <t>OKVED_86_VSvyaziSOplTrudRab</t>
+          <t>OKVED_86_PostavPoSyrMatRabUsl</t>
         </is>
       </c>
     </row>
     <row r="1520">
       <c r="A1520" t="inlineStr">
         <is>
-          <t>OKVED_86_ProcPoDolgObyaz</t>
+          <t>OKVED_86_VSvyaziSOplTrudRab</t>
         </is>
       </c>
     </row>
     <row r="1521">
       <c r="A1521" t="inlineStr">
         <is>
-          <t>OKVED_86_NalogNaPri</t>
+          <t>OKVED_86_ProcPoDolgObyaz</t>
         </is>
       </c>
     </row>
     <row r="1522">
       <c r="A1522" t="inlineStr">
         <is>
-          <t>OKVED_86_SaldoDenPotTekOper</t>
+          <t>OKVED_86_NalogNaPri</t>
         </is>
       </c>
     </row>
     <row r="1523">
       <c r="A1523" t="inlineStr">
         <is>
-          <t>OKVED_R_PostavPoSyrMatRabUsl</t>
+          <t>OKVED_86_SaldoDenPotTekOper</t>
         </is>
       </c>
     </row>
     <row r="1524">
       <c r="A1524" t="inlineStr">
         <is>
-          <t>OKVED_R_VSvyaziSOplTrudRab</t>
+          <t>OKVED_R_PostavPoSyrMatRabUsl</t>
         </is>
       </c>
     </row>
     <row r="1525">
       <c r="A1525" t="inlineStr">
         <is>
-          <t>OKVED_R_ProcPoDolgObyaz</t>
+          <t>OKVED_R_VSvyaziSOplTrudRab</t>
         </is>
       </c>
     </row>
     <row r="1526">
       <c r="A1526" t="inlineStr">
         <is>
-          <t>OKVED_R_NalogNaPri</t>
+          <t>OKVED_R_ProcPoDolgObyaz</t>
         </is>
       </c>
     </row>
     <row r="1527">
       <c r="A1527" t="inlineStr">
         <is>
-          <t>OKVED_93_PostavPoSyrMatRabUsl</t>
+          <t>OKVED_R_NalogNaPri</t>
         </is>
       </c>
     </row>
     <row r="1528">
       <c r="A1528" t="inlineStr">
         <is>
-          <t>OKVED_93_VSvyaziSOplTrudRab</t>
+          <t>OKVED_93_PostavPoSyrMatRabUsl</t>
         </is>
       </c>
     </row>
     <row r="1529">
       <c r="A1529" t="inlineStr">
         <is>
-          <t>OKVED_93_ProcPoDolgObyaz</t>
+          <t>OKVED_93_VSvyaziSOplTrudRab</t>
         </is>
       </c>
     </row>
     <row r="1530">
       <c r="A1530" t="inlineStr">
         <is>
-          <t>OKVED_93_NalogNaPri</t>
+          <t>OKVED_93_ProcPoDolgObyaz</t>
         </is>
       </c>
     </row>
     <row r="1531">
       <c r="A1531" t="inlineStr">
         <is>
-          <t>OKVED_96_ProcPoDolgObyaz</t>
+          <t>OKVED_93_NalogNaPri</t>
         </is>
       </c>
     </row>
     <row r="1532">
       <c r="A1532" t="inlineStr">
         <is>
-          <t>OKVED_96_NalogNaPri</t>
+          <t>OKVED_96_ProcPoDolgObyaz</t>
         </is>
       </c>
     </row>
     <row r="1533">
       <c r="A1533" t="inlineStr">
         <is>
-          <t>OKVED_01_OtProdVneObAktKromeFinVlozh</t>
+          <t>OKVED_96_NalogNaPri</t>
         </is>
       </c>
     </row>
     <row r="1534">
       <c r="A1534" t="inlineStr">
         <is>
-          <t>OKVED_01_OtProdAkcOrgDolUch</t>
+          <t>OKVED_01_OtProdVneObAktKromeFinVlozh</t>
         </is>
       </c>
     </row>
     <row r="1535">
       <c r="A1535" t="inlineStr">
         <is>
-          <t>OKVED_01_DivProcDolgFinVlozh</t>
+          <t>OKVED_01_OtProdAkcOrgDolUch</t>
         </is>
       </c>
     </row>
     <row r="1536">
       <c r="A1536" t="inlineStr">
         <is>
-          <t>OKVED_B_OtProdAkcOrgDolUch</t>
+          <t>OKVED_01_DivProcDolgFinVlozh</t>
         </is>
       </c>
     </row>
     <row r="1537">
       <c r="A1537" t="inlineStr">
         <is>
-          <t>OKVED_07_OtProdAkcOrgDolUch</t>
+          <t>OKVED_B_OtProdAkcOrgDolUch</t>
         </is>
       </c>
     </row>
     <row r="1538">
       <c r="A1538" t="inlineStr">
         <is>
-          <t>OKVED_C_OtProdAkcOrgDolUch</t>
+          <t>OKVED_07_OtProdAkcOrgDolUch</t>
         </is>
       </c>
     </row>
     <row r="1539">
       <c r="A1539" t="inlineStr">
         <is>
-          <t>OKVED_10_OtProdAkcOrgDolUch</t>
+          <t>OKVED_C_OtProdAkcOrgDolUch</t>
         </is>
       </c>
     </row>
     <row r="1540">
       <c r="A1540" t="inlineStr">
         <is>
-          <t>OKVED_11_OtProdVneObAktKromeFinVlozh</t>
+          <t>OKVED_10_OtProdAkcOrgDolUch</t>
         </is>
       </c>
     </row>
     <row r="1541">
       <c r="A1541" t="inlineStr">
         <is>
-          <t>OKVED_11_OtProdAkcOrgDolUch</t>
+          <t>OKVED_11_OtProdVneObAktKromeFinVlozh</t>
         </is>
       </c>
     </row>
     <row r="1542">
       <c r="A1542" t="inlineStr">
         <is>
-          <t>OKVED_11_OtProdFinVlozh</t>
+          <t>OKVED_11_OtProdAkcOrgDolUch</t>
         </is>
       </c>
     </row>
     <row r="1543">
       <c r="A1543" t="inlineStr">
         <is>
-          <t>OKVED_33_OtProdVneObAktKromeFinVlozh</t>
+          <t>OKVED_11_OtProdFinVlozh</t>
         </is>
       </c>
     </row>
     <row r="1544">
       <c r="A1544" t="inlineStr">
         <is>
-          <t>OKVED_33_OtProdAkcOrgDolUch</t>
+          <t>OKVED_33_OtProdVneObAktKromeFinVlozh</t>
         </is>
       </c>
     </row>
     <row r="1545">
       <c r="A1545" t="inlineStr">
         <is>
-          <t>OKVED_33_DivProcDolgFinVlozh</t>
+          <t>OKVED_33_OtProdAkcOrgDolUch</t>
         </is>
       </c>
     </row>
     <row r="1546">
       <c r="A1546" t="inlineStr">
         <is>
-          <t>OKVED_35_OtProdAkcOrgDolUch</t>
+          <t>OKVED_33_DivProcDolgFinVlozh</t>
         </is>
       </c>
     </row>
@@ -11248,1008 +11248,1008 @@
     <row r="1548">
       <c r="A1548" t="inlineStr">
         <is>
-          <t>OKVED_E_OtProdAkcOrgDolUch</t>
+          <t>OKVED_35_OtProdAkcOrgDolUch</t>
         </is>
       </c>
     </row>
     <row r="1549">
       <c r="A1549" t="inlineStr">
         <is>
-          <t>OKVED_E_OtProdFinVlozh</t>
+          <t>OKVED_E_OtProdAkcOrgDolUch</t>
         </is>
       </c>
     </row>
     <row r="1550">
       <c r="A1550" t="inlineStr">
         <is>
-          <t>OKVED_E_DivProcDolgFinVlozh</t>
+          <t>OKVED_E_OtProdFinVlozh</t>
         </is>
       </c>
     </row>
     <row r="1551">
       <c r="A1551" t="inlineStr">
         <is>
-          <t>OKVED_36_OtProdAkcOrgDolUch</t>
+          <t>OKVED_E_DivProcDolgFinVlozh</t>
         </is>
       </c>
     </row>
     <row r="1552">
       <c r="A1552" t="inlineStr">
         <is>
-          <t>OKVED_36_OtProdFinVlozh</t>
+          <t>OKVED_36_OtProdAkcOrgDolUch</t>
         </is>
       </c>
     </row>
     <row r="1553">
       <c r="A1553" t="inlineStr">
         <is>
-          <t>OKVED_36_DivProcDolgFinVlozh</t>
+          <t>OKVED_36_OtProdFinVlozh</t>
         </is>
       </c>
     </row>
     <row r="1554">
       <c r="A1554" t="inlineStr">
         <is>
-          <t>OKVED_38_OtProdVneObAktKromeFinVlozh</t>
+          <t>OKVED_36_DivProcDolgFinVlozh</t>
         </is>
       </c>
     </row>
     <row r="1555">
       <c r="A1555" t="inlineStr">
         <is>
-          <t>OKVED_38_OtProdAkcOrgDolUch</t>
+          <t>OKVED_38_OtProdVneObAktKromeFinVlozh</t>
         </is>
       </c>
     </row>
     <row r="1556">
       <c r="A1556" t="inlineStr">
         <is>
-          <t>OKVED_38_OtProdFinVlozh</t>
+          <t>OKVED_38_OtProdAkcOrgDolUch</t>
         </is>
       </c>
     </row>
     <row r="1557">
       <c r="A1557" t="inlineStr">
         <is>
-          <t>OKVED_38_DivProcDolgFinVlozh</t>
+          <t>OKVED_38_OtProdFinVlozh</t>
         </is>
       </c>
     </row>
     <row r="1558">
       <c r="A1558" t="inlineStr">
         <is>
-          <t>OKVED_F_OtProdVneObAktKromeFinVlozh</t>
+          <t>OKVED_38_DivProcDolgFinVlozh</t>
         </is>
       </c>
     </row>
     <row r="1559">
       <c r="A1559" t="inlineStr">
         <is>
-          <t>OKVED_F_OtProdAkcOrgDolUch</t>
+          <t>OKVED_F_OtProdVneObAktKromeFinVlozh</t>
         </is>
       </c>
     </row>
     <row r="1560">
       <c r="A1560" t="inlineStr">
         <is>
-          <t>OKVED_41_OtProdVneObAktKromeFinVlozh</t>
+          <t>OKVED_F_OtProdAkcOrgDolUch</t>
         </is>
       </c>
     </row>
     <row r="1561">
       <c r="A1561" t="inlineStr">
         <is>
-          <t>OKVED_41_OtProdAkcOrgDolUch</t>
+          <t>OKVED_41_OtProdVneObAktKromeFinVlozh</t>
         </is>
       </c>
     </row>
     <row r="1562">
       <c r="A1562" t="inlineStr">
         <is>
-          <t>OKVED_42_OtProdVneObAktKromeFinVlozh</t>
+          <t>OKVED_41_OtProdAkcOrgDolUch</t>
         </is>
       </c>
     </row>
     <row r="1563">
       <c r="A1563" t="inlineStr">
         <is>
-          <t>OKVED_42_OtProdAkcOrgDolUch</t>
+          <t>OKVED_42_OtProdVneObAktKromeFinVlozh</t>
         </is>
       </c>
     </row>
     <row r="1564">
       <c r="A1564" t="inlineStr">
         <is>
-          <t>OKVED_43_OtProdVneObAktKromeFinVlozh</t>
+          <t>OKVED_42_OtProdAkcOrgDolUch</t>
         </is>
       </c>
     </row>
     <row r="1565">
       <c r="A1565" t="inlineStr">
         <is>
-          <t>OKVED_43_OtProdAkcOrgDolUch</t>
+          <t>OKVED_43_OtProdVneObAktKromeFinVlozh</t>
         </is>
       </c>
     </row>
     <row r="1566">
       <c r="A1566" t="inlineStr">
         <is>
-          <t>OKVED_43_OtProdFinVlozh</t>
+          <t>OKVED_43_OtProdAkcOrgDolUch</t>
         </is>
       </c>
     </row>
     <row r="1567">
       <c r="A1567" t="inlineStr">
         <is>
-          <t>OKVED_G_OtProdAkcOrgDolUch</t>
+          <t>OKVED_43_OtProdFinVlozh</t>
         </is>
       </c>
     </row>
     <row r="1568">
       <c r="A1568" t="inlineStr">
         <is>
-          <t>OKVED_46_OtProdAkcOrgDolUch</t>
+          <t>OKVED_G_OtProdAkcOrgDolUch</t>
         </is>
       </c>
     </row>
     <row r="1569">
       <c r="A1569" t="inlineStr">
         <is>
-          <t>OKVED_47_OtProdAkcOrgDolUch</t>
+          <t>OKVED_46_OtProdAkcOrgDolUch</t>
         </is>
       </c>
     </row>
     <row r="1570">
       <c r="A1570" t="inlineStr">
         <is>
-          <t>OKVED_H_OtProdAkcOrgDolUch</t>
+          <t>OKVED_47_OtProdAkcOrgDolUch</t>
         </is>
       </c>
     </row>
     <row r="1571">
       <c r="A1571" t="inlineStr">
         <is>
-          <t>OKVED_49_OtProdVneObAktKromeFinVlozh</t>
+          <t>OKVED_H_OtProdAkcOrgDolUch</t>
         </is>
       </c>
     </row>
     <row r="1572">
       <c r="A1572" t="inlineStr">
         <is>
-          <t>OKVED_49_OtProdAkcOrgDolUch</t>
+          <t>OKVED_49_OtProdVneObAktKromeFinVlozh</t>
         </is>
       </c>
     </row>
     <row r="1573">
       <c r="A1573" t="inlineStr">
         <is>
-          <t>OKVED_49_DivProcDolgFinVlozh</t>
+          <t>OKVED_49_OtProdAkcOrgDolUch</t>
         </is>
       </c>
     </row>
     <row r="1574">
       <c r="A1574" t="inlineStr">
         <is>
-          <t>OKVED_51_OtProdVneObAktKromeFinVlozh</t>
+          <t>OKVED_49_DivProcDolgFinVlozh</t>
         </is>
       </c>
     </row>
     <row r="1575">
       <c r="A1575" t="inlineStr">
         <is>
-          <t>OKVED_51_OtProdAkcOrgDolUch</t>
+          <t>OKVED_51_OtProdVneObAktKromeFinVlozh</t>
         </is>
       </c>
     </row>
     <row r="1576">
       <c r="A1576" t="inlineStr">
         <is>
-          <t>OKVED_52_OtProdAkcOrgDolUch</t>
+          <t>OKVED_51_OtProdAkcOrgDolUch</t>
         </is>
       </c>
     </row>
     <row r="1577">
       <c r="A1577" t="inlineStr">
         <is>
-          <t>OKVED_I_OtProdVneObAktKromeFinVlozh</t>
+          <t>OKVED_52_OtProdAkcOrgDolUch</t>
         </is>
       </c>
     </row>
     <row r="1578">
       <c r="A1578" t="inlineStr">
         <is>
-          <t>OKVED_I_OtProdAkcOrgDolUch</t>
+          <t>OKVED_I_OtProdVneObAktKromeFinVlozh</t>
         </is>
       </c>
     </row>
     <row r="1579">
       <c r="A1579" t="inlineStr">
         <is>
-          <t>OKVED_55_OtProdVneObAktKromeFinVlozh</t>
+          <t>OKVED_I_OtProdAkcOrgDolUch</t>
         </is>
       </c>
     </row>
     <row r="1580">
       <c r="A1580" t="inlineStr">
         <is>
-          <t>OKVED_55_OtProdAkcOrgDolUch</t>
+          <t>OKVED_55_OtProdVneObAktKromeFinVlozh</t>
         </is>
       </c>
     </row>
     <row r="1581">
       <c r="A1581" t="inlineStr">
         <is>
-          <t>OKVED_K_OtProdVneObAktKromeFinVlozh</t>
+          <t>OKVED_55_OtProdAkcOrgDolUch</t>
         </is>
       </c>
     </row>
     <row r="1582">
       <c r="A1582" t="inlineStr">
         <is>
-          <t>OKVED_K_OtProdAkcOrgDolUch</t>
+          <t>OKVED_K_OtProdVneObAktKromeFinVlozh</t>
         </is>
       </c>
     </row>
     <row r="1583">
       <c r="A1583" t="inlineStr">
         <is>
-          <t>OKVED_64_OtProdVneObAktKromeFinVlozh</t>
+          <t>OKVED_K_OtProdAkcOrgDolUch</t>
         </is>
       </c>
     </row>
     <row r="1584">
       <c r="A1584" t="inlineStr">
         <is>
-          <t>OKVED_64_OtProdAkcOrgDolUch</t>
+          <t>OKVED_64_OtProdVneObAktKromeFinVlozh</t>
         </is>
       </c>
     </row>
     <row r="1585">
       <c r="A1585" t="inlineStr">
         <is>
-          <t>OKVED_L_OtProdAkcOrgDolUch</t>
+          <t>OKVED_64_OtProdAkcOrgDolUch</t>
         </is>
       </c>
     </row>
     <row r="1586">
       <c r="A1586" t="inlineStr">
         <is>
-          <t>OKVED_68_OtProdAkcOrgDolUch</t>
+          <t>OKVED_L_OtProdAkcOrgDolUch</t>
         </is>
       </c>
     </row>
     <row r="1587">
       <c r="A1587" t="inlineStr">
         <is>
-          <t>OKVED_M_OtProdVneObAktKromeFinVlozh</t>
+          <t>OKVED_68_OtProdAkcOrgDolUch</t>
         </is>
       </c>
     </row>
     <row r="1588">
       <c r="A1588" t="inlineStr">
         <is>
-          <t>OKVED_M_OtProdAkcOrgDolUch</t>
+          <t>OKVED_M_OtProdVneObAktKromeFinVlozh</t>
         </is>
       </c>
     </row>
     <row r="1589">
       <c r="A1589" t="inlineStr">
         <is>
-          <t>OKVED_70_OtProdVneObAktKromeFinVlozh</t>
+          <t>OKVED_M_OtProdAkcOrgDolUch</t>
         </is>
       </c>
     </row>
     <row r="1590">
       <c r="A1590" t="inlineStr">
         <is>
-          <t>OKVED_70_OtProdAkcOrgDolUch</t>
+          <t>OKVED_70_OtProdVneObAktKromeFinVlozh</t>
         </is>
       </c>
     </row>
     <row r="1591">
       <c r="A1591" t="inlineStr">
         <is>
-          <t>OKVED_71_OtProdVneObAktKromeFinVlozh</t>
+          <t>OKVED_70_OtProdAkcOrgDolUch</t>
         </is>
       </c>
     </row>
     <row r="1592">
       <c r="A1592" t="inlineStr">
         <is>
-          <t>OKVED_71_OtProdAkcOrgDolUch</t>
+          <t>OKVED_71_OtProdVneObAktKromeFinVlozh</t>
         </is>
       </c>
     </row>
     <row r="1593">
       <c r="A1593" t="inlineStr">
         <is>
-          <t>OKVED_71_DivProcDolgFinVlozh</t>
+          <t>OKVED_71_OtProdAkcOrgDolUch</t>
         </is>
       </c>
     </row>
     <row r="1594">
       <c r="A1594" t="inlineStr">
         <is>
-          <t>OKVED_N_OtProdAkcOrgDolUch</t>
+          <t>OKVED_71_DivProcDolgFinVlozh</t>
         </is>
       </c>
     </row>
     <row r="1595">
       <c r="A1595" t="inlineStr">
         <is>
-          <t>OKVED_N_OtProdFinVlozh</t>
+          <t>OKVED_N_OtProdAkcOrgDolUch</t>
         </is>
       </c>
     </row>
     <row r="1596">
       <c r="A1596" t="inlineStr">
         <is>
-          <t>OKVED_77_OtProdAkcOrgDolUch</t>
+          <t>OKVED_N_OtProdFinVlozh</t>
         </is>
       </c>
     </row>
     <row r="1597">
       <c r="A1597" t="inlineStr">
         <is>
-          <t>OKVED_77_OtProdFinVlozh</t>
+          <t>OKVED_77_OtProdAkcOrgDolUch</t>
         </is>
       </c>
     </row>
     <row r="1598">
       <c r="A1598" t="inlineStr">
         <is>
-          <t>OKVED_79_OtProdAkcOrgDolUch</t>
+          <t>OKVED_77_OtProdFinVlozh</t>
         </is>
       </c>
     </row>
     <row r="1599">
       <c r="A1599" t="inlineStr">
         <is>
-          <t>OKVED_79_OtProdFinVlozh</t>
+          <t>OKVED_79_OtProdAkcOrgDolUch</t>
         </is>
       </c>
     </row>
     <row r="1600">
       <c r="A1600" t="inlineStr">
         <is>
-          <t>OKVED_79_DivProcDolgFinVlozh</t>
+          <t>OKVED_79_OtProdFinVlozh</t>
         </is>
       </c>
     </row>
     <row r="1601">
       <c r="A1601" t="inlineStr">
         <is>
-          <t>OKVED_S_OtProdVneObAktKromeFinVlozh</t>
+          <t>OKVED_79_DivProcDolgFinVlozh</t>
         </is>
       </c>
     </row>
     <row r="1602">
       <c r="A1602" t="inlineStr">
         <is>
-          <t>OKVED_S_OtProdAkcOrgDolUch</t>
+          <t>OKVED_S_OtProdVneObAktKromeFinVlozh</t>
         </is>
       </c>
     </row>
     <row r="1603">
       <c r="A1603" t="inlineStr">
         <is>
-          <t>OKVED_S_DivProcDolgFinVlozh</t>
+          <t>OKVED_S_OtProdAkcOrgDolUch</t>
         </is>
       </c>
     </row>
     <row r="1604">
       <c r="A1604" t="inlineStr">
         <is>
-          <t>OKVED_94_OtProdVneObAktKromeFinVlozh</t>
+          <t>OKVED_S_DivProcDolgFinVlozh</t>
         </is>
       </c>
     </row>
     <row r="1605">
       <c r="A1605" t="inlineStr">
         <is>
-          <t>OKVED_94_OtProdAkcOrgDolUch</t>
+          <t>OKVED_94_OtProdVneObAktKromeFinVlozh</t>
         </is>
       </c>
     </row>
     <row r="1606">
       <c r="A1606" t="inlineStr">
         <is>
-          <t>OKVED_94_DivProcDolgFinVlozh</t>
+          <t>OKVED_94_OtProdAkcOrgDolUch</t>
         </is>
       </c>
     </row>
     <row r="1607">
       <c r="A1607" t="inlineStr">
         <is>
-          <t>OKVED_01_DolUch</t>
+          <t>OKVED_94_DivProcDolgFinVlozh</t>
         </is>
       </c>
     </row>
     <row r="1608">
       <c r="A1608" t="inlineStr">
         <is>
-          <t>OKVED_01_PrCenBum</t>
+          <t>OKVED_01_DolUch</t>
         </is>
       </c>
     </row>
     <row r="1609">
       <c r="A1609" t="inlineStr">
         <is>
-          <t>OKVED_B_DolUch</t>
+          <t>OKVED_01_PrCenBum</t>
         </is>
       </c>
     </row>
     <row r="1610">
       <c r="A1610" t="inlineStr">
         <is>
-          <t>OKVED_B_ProcDolgObyazVklInvAkt</t>
+          <t>OKVED_B_DolUch</t>
         </is>
       </c>
     </row>
     <row r="1611">
       <c r="A1611" t="inlineStr">
         <is>
-          <t>OKVED_07_DolUch</t>
+          <t>OKVED_B_ProcDolgObyazVklInvAkt</t>
         </is>
       </c>
     </row>
     <row r="1612">
       <c r="A1612" t="inlineStr">
         <is>
-          <t>OKVED_07_ProcDolgObyazVklInvAkt</t>
+          <t>OKVED_07_DolUch</t>
         </is>
       </c>
     </row>
     <row r="1613">
       <c r="A1613" t="inlineStr">
         <is>
-          <t>OKVED_C_DolUch</t>
+          <t>OKVED_07_ProcDolgObyazVklInvAkt</t>
         </is>
       </c>
     </row>
     <row r="1614">
       <c r="A1614" t="inlineStr">
         <is>
-          <t>OKVED_C_ProcDolgObyazVklInvAkt</t>
+          <t>OKVED_C_DolUch</t>
         </is>
       </c>
     </row>
     <row r="1615">
       <c r="A1615" t="inlineStr">
         <is>
-          <t>OKVED_10_DolUch</t>
+          <t>OKVED_C_ProcDolgObyazVklInvAkt</t>
         </is>
       </c>
     </row>
     <row r="1616">
       <c r="A1616" t="inlineStr">
         <is>
-          <t>OKVED_10_ProcDolgObyazVklInvAkt</t>
+          <t>OKVED_10_DolUch</t>
         </is>
       </c>
     </row>
     <row r="1617">
       <c r="A1617" t="inlineStr">
         <is>
-          <t>OKVED_11_DolUch</t>
+          <t>OKVED_10_ProcDolgObyazVklInvAkt</t>
         </is>
       </c>
     </row>
     <row r="1618">
       <c r="A1618" t="inlineStr">
         <is>
-          <t>OKVED_11_PrCenBum</t>
+          <t>OKVED_11_DolUch</t>
         </is>
       </c>
     </row>
     <row r="1619">
       <c r="A1619" t="inlineStr">
         <is>
-          <t>OKVED_11_ProcDolgObyazVklInvAkt</t>
+          <t>OKVED_11_PrCenBum</t>
         </is>
       </c>
     </row>
     <row r="1620">
       <c r="A1620" t="inlineStr">
         <is>
-          <t>OKVED_33_DolUch</t>
+          <t>OKVED_11_ProcDolgObyazVklInvAkt</t>
         </is>
       </c>
     </row>
     <row r="1621">
       <c r="A1621" t="inlineStr">
         <is>
-          <t>OKVED_33_ProcDolgObyazVklInvAkt</t>
+          <t>OKVED_33_DolUch</t>
         </is>
       </c>
     </row>
     <row r="1622">
       <c r="A1622" t="inlineStr">
         <is>
-          <t>OKVED_E_DolUch</t>
+          <t>OKVED_33_ProcDolgObyazVklInvAkt</t>
         </is>
       </c>
     </row>
     <row r="1623">
       <c r="A1623" t="inlineStr">
         <is>
-          <t>OKVED_E_PrCenBum</t>
+          <t>OKVED_E_DolUch</t>
         </is>
       </c>
     </row>
     <row r="1624">
       <c r="A1624" t="inlineStr">
         <is>
-          <t>OKVED_E_ProcDolgObyazVklInvAkt</t>
+          <t>OKVED_E_PrCenBum</t>
         </is>
       </c>
     </row>
     <row r="1625">
       <c r="A1625" t="inlineStr">
         <is>
-          <t>OKVED_36_DolUch</t>
+          <t>OKVED_E_ProcDolgObyazVklInvAkt</t>
         </is>
       </c>
     </row>
     <row r="1626">
       <c r="A1626" t="inlineStr">
         <is>
-          <t>OKVED_36_PrCenBum</t>
+          <t>OKVED_36_DolUch</t>
         </is>
       </c>
     </row>
     <row r="1627">
       <c r="A1627" t="inlineStr">
         <is>
-          <t>OKVED_36_ProcDolgObyazVklInvAkt</t>
+          <t>OKVED_36_PrCenBum</t>
         </is>
       </c>
     </row>
     <row r="1628">
       <c r="A1628" t="inlineStr">
         <is>
-          <t>OKVED_38_DolUch</t>
+          <t>OKVED_36_ProcDolgObyazVklInvAkt</t>
         </is>
       </c>
     </row>
     <row r="1629">
       <c r="A1629" t="inlineStr">
         <is>
-          <t>OKVED_38_PrCenBum</t>
+          <t>OKVED_38_DolUch</t>
         </is>
       </c>
     </row>
     <row r="1630">
       <c r="A1630" t="inlineStr">
         <is>
-          <t>OKVED_38_ProcDolgObyazVklInvAkt</t>
+          <t>OKVED_38_PrCenBum</t>
         </is>
       </c>
     </row>
     <row r="1631">
       <c r="A1631" t="inlineStr">
         <is>
-          <t>OKVED_F_DolUch</t>
+          <t>OKVED_38_ProcDolgObyazVklInvAkt</t>
         </is>
       </c>
     </row>
     <row r="1632">
       <c r="A1632" t="inlineStr">
         <is>
-          <t>OKVED_F_ProcDolgObyazVklInvAkt</t>
+          <t>OKVED_F_DolUch</t>
         </is>
       </c>
     </row>
     <row r="1633">
       <c r="A1633" t="inlineStr">
         <is>
-          <t>OKVED_41_DolUch</t>
+          <t>OKVED_F_ProcDolgObyazVklInvAkt</t>
         </is>
       </c>
     </row>
     <row r="1634">
       <c r="A1634" t="inlineStr">
         <is>
-          <t>OKVED_41_ProcDolgObyazVklInvAkt</t>
+          <t>OKVED_41_DolUch</t>
         </is>
       </c>
     </row>
     <row r="1635">
       <c r="A1635" t="inlineStr">
         <is>
-          <t>OKVED_42_DolUch</t>
+          <t>OKVED_41_ProcDolgObyazVklInvAkt</t>
         </is>
       </c>
     </row>
     <row r="1636">
       <c r="A1636" t="inlineStr">
         <is>
-          <t>OKVED_42_ProcDolgObyazVklInvAkt</t>
+          <t>OKVED_42_DolUch</t>
         </is>
       </c>
     </row>
     <row r="1637">
       <c r="A1637" t="inlineStr">
         <is>
-          <t>OKVED_43_DolUch</t>
+          <t>OKVED_42_ProcDolgObyazVklInvAkt</t>
         </is>
       </c>
     </row>
     <row r="1638">
       <c r="A1638" t="inlineStr">
         <is>
-          <t>OKVED_43_PrCenBum</t>
+          <t>OKVED_43_DolUch</t>
         </is>
       </c>
     </row>
     <row r="1639">
       <c r="A1639" t="inlineStr">
         <is>
-          <t>OKVED_43_ProcDolgObyazVklInvAkt</t>
+          <t>OKVED_43_PrCenBum</t>
         </is>
       </c>
     </row>
     <row r="1640">
       <c r="A1640" t="inlineStr">
         <is>
-          <t>OKVED_46_ProcDolgObyazVklInvAkt</t>
+          <t>OKVED_43_ProcDolgObyazVklInvAkt</t>
         </is>
       </c>
     </row>
     <row r="1641">
       <c r="A1641" t="inlineStr">
         <is>
-          <t>OKVED_47_DolUch</t>
+          <t>OKVED_46_ProcDolgObyazVklInvAkt</t>
         </is>
       </c>
     </row>
     <row r="1642">
       <c r="A1642" t="inlineStr">
         <is>
-          <t>OKVED_H_DolUch</t>
+          <t>OKVED_47_DolUch</t>
         </is>
       </c>
     </row>
     <row r="1643">
       <c r="A1643" t="inlineStr">
         <is>
-          <t>OKVED_H_ProcDolgObyazVklInvAkt</t>
+          <t>OKVED_H_DolUch</t>
         </is>
       </c>
     </row>
     <row r="1644">
       <c r="A1644" t="inlineStr">
         <is>
-          <t>OKVED_49_DolUch</t>
+          <t>OKVED_H_ProcDolgObyazVklInvAkt</t>
         </is>
       </c>
     </row>
     <row r="1645">
       <c r="A1645" t="inlineStr">
         <is>
-          <t>OKVED_49_ProcDolgObyazVklInvAkt</t>
+          <t>OKVED_49_DolUch</t>
         </is>
       </c>
     </row>
     <row r="1646">
       <c r="A1646" t="inlineStr">
         <is>
-          <t>OKVED_50_DolUch</t>
+          <t>OKVED_49_ProcDolgObyazVklInvAkt</t>
         </is>
       </c>
     </row>
     <row r="1647">
       <c r="A1647" t="inlineStr">
         <is>
-          <t>OKVED_50_PrCenBum</t>
+          <t>OKVED_50_DolUch</t>
         </is>
       </c>
     </row>
     <row r="1648">
       <c r="A1648" t="inlineStr">
         <is>
-          <t>OKVED_50_ProcDolgObyazVklInvAkt</t>
+          <t>OKVED_50_PrCenBum</t>
         </is>
       </c>
     </row>
     <row r="1649">
       <c r="A1649" t="inlineStr">
         <is>
-          <t>OKVED_51_DolUch</t>
+          <t>OKVED_50_ProcDolgObyazVklInvAkt</t>
         </is>
       </c>
     </row>
     <row r="1650">
       <c r="A1650" t="inlineStr">
         <is>
-          <t>OKVED_51_PrCenBum</t>
+          <t>OKVED_51_DolUch</t>
         </is>
       </c>
     </row>
     <row r="1651">
       <c r="A1651" t="inlineStr">
         <is>
-          <t>OKVED_51_ProcDolgObyazVklInvAkt</t>
+          <t>OKVED_51_PrCenBum</t>
         </is>
       </c>
     </row>
     <row r="1652">
       <c r="A1652" t="inlineStr">
         <is>
-          <t>OKVED_52_DolUch</t>
+          <t>OKVED_51_ProcDolgObyazVklInvAkt</t>
         </is>
       </c>
     </row>
     <row r="1653">
       <c r="A1653" t="inlineStr">
         <is>
-          <t>OKVED_52_ProcDolgObyazVklInvAkt</t>
+          <t>OKVED_52_DolUch</t>
         </is>
       </c>
     </row>
     <row r="1654">
       <c r="A1654" t="inlineStr">
         <is>
-          <t>OKVED_I_ProcDolgObyazVklInvAkt</t>
+          <t>OKVED_52_ProcDolgObyazVklInvAkt</t>
         </is>
       </c>
     </row>
     <row r="1655">
       <c r="A1655" t="inlineStr">
         <is>
-          <t>OKVED_55_ProcDolgObyazVklInvAkt</t>
+          <t>OKVED_I_ProcDolgObyazVklInvAkt</t>
         </is>
       </c>
     </row>
     <row r="1656">
       <c r="A1656" t="inlineStr">
         <is>
-          <t>OKVED_K_DolUch</t>
+          <t>OKVED_55_ProcDolgObyazVklInvAkt</t>
         </is>
       </c>
     </row>
     <row r="1657">
       <c r="A1657" t="inlineStr">
         <is>
-          <t>OKVED_K_ProcDolgObyazVklInvAkt</t>
+          <t>OKVED_K_DolUch</t>
         </is>
       </c>
     </row>
     <row r="1658">
       <c r="A1658" t="inlineStr">
         <is>
-          <t>OKVED_64_DolUch</t>
+          <t>OKVED_K_ProcDolgObyazVklInvAkt</t>
         </is>
       </c>
     </row>
     <row r="1659">
       <c r="A1659" t="inlineStr">
         <is>
-          <t>OKVED_64_ProcDolgObyazVklInvAkt</t>
+          <t>OKVED_64_DolUch</t>
         </is>
       </c>
     </row>
     <row r="1660">
       <c r="A1660" t="inlineStr">
         <is>
-          <t>OKVED_M_DolUch</t>
+          <t>OKVED_64_ProcDolgObyazVklInvAkt</t>
         </is>
       </c>
     </row>
     <row r="1661">
       <c r="A1661" t="inlineStr">
         <is>
-          <t>OKVED_70_DolUch</t>
+          <t>OKVED_M_DolUch</t>
         </is>
       </c>
     </row>
     <row r="1662">
       <c r="A1662" t="inlineStr">
         <is>
-          <t>OKVED_70_ProcDolgObyazVklInvAkt</t>
+          <t>OKVED_70_DolUch</t>
         </is>
       </c>
     </row>
     <row r="1663">
       <c r="A1663" t="inlineStr">
         <is>
-          <t>OKVED_71_DolUch</t>
+          <t>OKVED_70_ProcDolgObyazVklInvAkt</t>
         </is>
       </c>
     </row>
     <row r="1664">
       <c r="A1664" t="inlineStr">
         <is>
-          <t>OKVED_N_DolUch</t>
+          <t>OKVED_71_DolUch</t>
         </is>
       </c>
     </row>
     <row r="1665">
       <c r="A1665" t="inlineStr">
         <is>
-          <t>OKVED_N_PrCenBum</t>
+          <t>OKVED_N_DolUch</t>
         </is>
       </c>
     </row>
     <row r="1666">
       <c r="A1666" t="inlineStr">
         <is>
-          <t>OKVED_77_DolUch</t>
+          <t>OKVED_N_PrCenBum</t>
         </is>
       </c>
     </row>
     <row r="1667">
       <c r="A1667" t="inlineStr">
         <is>
-          <t>OKVED_77_PrCenBum</t>
+          <t>OKVED_77_DolUch</t>
         </is>
       </c>
     </row>
     <row r="1668">
       <c r="A1668" t="inlineStr">
         <is>
-          <t>OKVED_77_ProcDolgObyazVklInvAkt</t>
+          <t>OKVED_77_PrCenBum</t>
         </is>
       </c>
     </row>
     <row r="1669">
       <c r="A1669" t="inlineStr">
         <is>
-          <t>OKVED_79_DolUch</t>
+          <t>OKVED_77_ProcDolgObyazVklInvAkt</t>
         </is>
       </c>
     </row>
     <row r="1670">
       <c r="A1670" t="inlineStr">
         <is>
-          <t>OKVED_79_PrCenBum</t>
+          <t>OKVED_79_DolUch</t>
         </is>
       </c>
     </row>
     <row r="1671">
       <c r="A1671" t="inlineStr">
         <is>
-          <t>OKVED_S_Modern</t>
+          <t>OKVED_79_PrCenBum</t>
         </is>
       </c>
     </row>
     <row r="1672">
       <c r="A1672" t="inlineStr">
         <is>
-          <t>OKVED_S_DolUch</t>
+          <t>OKVED_S_Modern</t>
         </is>
       </c>
     </row>
     <row r="1673">
       <c r="A1673" t="inlineStr">
         <is>
-          <t>OKVED_S_ProcDolgObyazVklInvAkt</t>
+          <t>OKVED_S_DolUch</t>
         </is>
       </c>
     </row>
     <row r="1674">
       <c r="A1674" t="inlineStr">
         <is>
-          <t>OKVED_94_Modern</t>
+          <t>OKVED_S_ProcDolgObyazVklInvAkt</t>
         </is>
       </c>
     </row>
     <row r="1675">
       <c r="A1675" t="inlineStr">
         <is>
-          <t>OKVED_94_DolUch</t>
+          <t>OKVED_94_Modern</t>
         </is>
       </c>
     </row>
     <row r="1676">
       <c r="A1676" t="inlineStr">
         <is>
-          <t>OKVED_94_ProcDolgObyazVklInvAkt</t>
+          <t>OKVED_94_DolUch</t>
         </is>
       </c>
     </row>
     <row r="1677">
       <c r="A1677" t="inlineStr">
         <is>
-          <t>OKVED_01_PostDeyt1</t>
+          <t>OKVED_94_ProcDolgObyazVklInvAkt</t>
         </is>
       </c>
     </row>
     <row r="1678">
       <c r="A1678" t="inlineStr">
         <is>
-          <t>OKVED_01_DrPost</t>
+          <t>OKVED_01_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1679">
       <c r="A1679" t="inlineStr">
         <is>
-          <t>OKVED_B_PostDeyt</t>
+          <t>OKVED_01_DrPost</t>
         </is>
       </c>
     </row>
     <row r="1680">
       <c r="A1680" t="inlineStr">
         <is>
-          <t>OKVED_B_PostDeyt1</t>
+          <t>OKVED_B_PostDeyt</t>
         </is>
       </c>
     </row>
     <row r="1681">
       <c r="A1681" t="inlineStr">
         <is>
-          <t>OKVED_07_PostDeyt</t>
+          <t>OKVED_B_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1682">
       <c r="A1682" t="inlineStr">
         <is>
-          <t>OKVED_07_PostDeyt1</t>
+          <t>OKVED_07_PostDeyt</t>
         </is>
       </c>
     </row>
     <row r="1683">
       <c r="A1683" t="inlineStr">
         <is>
-          <t>OKVED_C_PostDeyt1</t>
+          <t>OKVED_07_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1684">
       <c r="A1684" t="inlineStr">
         <is>
-          <t>OKVED_10_PostDeyt1</t>
+          <t>OKVED_C_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1685">
       <c r="A1685" t="inlineStr">
         <is>
-          <t>OKVED_32_PlCredit</t>
+          <t>OKVED_10_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1686">
       <c r="A1686" t="inlineStr">
         <is>
-          <t>OKVED_32_PostDeyt</t>
+          <t>OKVED_32_PlCredit</t>
         </is>
       </c>
     </row>
     <row r="1687">
       <c r="A1687" t="inlineStr">
         <is>
-          <t>OKVED_32_PostDeyt1</t>
+          <t>OKVED_32_PostDeyt</t>
         </is>
       </c>
     </row>
     <row r="1688">
       <c r="A1688" t="inlineStr">
         <is>
-          <t>OKVED_33_PostDeyt</t>
+          <t>OKVED_32_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1689">
       <c r="A1689" t="inlineStr">
         <is>
-          <t>OKVED_33_PostDeyt1</t>
+          <t>OKVED_33_PostDeyt</t>
         </is>
       </c>
     </row>
     <row r="1690">
       <c r="A1690" t="inlineStr">
         <is>
-          <t>OKVED_33_DrPost</t>
+          <t>OKVED_33_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1691">
       <c r="A1691" t="inlineStr">
         <is>
-          <t>OKVED_35_PostDeyt1</t>
+          <t>OKVED_33_DrPost</t>
         </is>
       </c>
     </row>
@@ -12263,504 +12263,504 @@
     <row r="1693">
       <c r="A1693" t="inlineStr">
         <is>
-          <t>OKVED_E_PostDeyt1</t>
+          <t>OKVED_35_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1694">
       <c r="A1694" t="inlineStr">
         <is>
-          <t>OKVED_E_DrPost</t>
+          <t>OKVED_E_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1695">
       <c r="A1695" t="inlineStr">
         <is>
-          <t>OKVED_38_PostDeyt1</t>
+          <t>OKVED_E_DrPost</t>
         </is>
       </c>
     </row>
     <row r="1696">
       <c r="A1696" t="inlineStr">
         <is>
-          <t>OKVED_38_DrPost</t>
+          <t>OKVED_38_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1697">
       <c r="A1697" t="inlineStr">
         <is>
-          <t>OKVED_F_PostDeyt1</t>
+          <t>OKVED_38_DrPost</t>
         </is>
       </c>
     </row>
     <row r="1698">
       <c r="A1698" t="inlineStr">
         <is>
-          <t>OKVED_41_PostDeyt</t>
+          <t>OKVED_F_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1699">
       <c r="A1699" t="inlineStr">
         <is>
-          <t>OKVED_41_PostDeyt1</t>
+          <t>OKVED_41_PostDeyt</t>
         </is>
       </c>
     </row>
     <row r="1700">
       <c r="A1700" t="inlineStr">
         <is>
-          <t>OKVED_42_PostDeyt</t>
+          <t>OKVED_41_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1701">
       <c r="A1701" t="inlineStr">
         <is>
-          <t>OKVED_42_PostDeyt1</t>
+          <t>OKVED_42_PostDeyt</t>
         </is>
       </c>
     </row>
     <row r="1702">
       <c r="A1702" t="inlineStr">
         <is>
-          <t>OKVED_42_DrPost</t>
+          <t>OKVED_42_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1703">
       <c r="A1703" t="inlineStr">
         <is>
-          <t>OKVED_43_PostDeyt1</t>
+          <t>OKVED_42_DrPost</t>
         </is>
       </c>
     </row>
     <row r="1704">
       <c r="A1704" t="inlineStr">
         <is>
-          <t>OKVED_43_DrPost</t>
+          <t>OKVED_43_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1705">
       <c r="A1705" t="inlineStr">
         <is>
-          <t>OKVED_G_PostDeyt</t>
+          <t>OKVED_43_DrPost</t>
         </is>
       </c>
     </row>
     <row r="1706">
       <c r="A1706" t="inlineStr">
         <is>
-          <t>OKVED_G_PostDeyt1</t>
+          <t>OKVED_G_PostDeyt</t>
         </is>
       </c>
     </row>
     <row r="1707">
       <c r="A1707" t="inlineStr">
         <is>
-          <t>OKVED_46_PostDeyt</t>
+          <t>OKVED_G_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1708">
       <c r="A1708" t="inlineStr">
         <is>
-          <t>OKVED_46_PostDeyt1</t>
+          <t>OKVED_46_PostDeyt</t>
         </is>
       </c>
     </row>
     <row r="1709">
       <c r="A1709" t="inlineStr">
         <is>
-          <t>OKVED_47_PostDeyt</t>
+          <t>OKVED_46_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1710">
       <c r="A1710" t="inlineStr">
         <is>
-          <t>OKVED_47_PostDeyt1</t>
+          <t>OKVED_47_PostDeyt</t>
         </is>
       </c>
     </row>
     <row r="1711">
       <c r="A1711" t="inlineStr">
         <is>
-          <t>OKVED_H_PostDeyt1</t>
+          <t>OKVED_47_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1712">
       <c r="A1712" t="inlineStr">
         <is>
-          <t>OKVED_49_PostDeyt</t>
+          <t>OKVED_H_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1713">
       <c r="A1713" t="inlineStr">
         <is>
-          <t>OKVED_49_PostDeyt1</t>
+          <t>OKVED_49_PostDeyt</t>
         </is>
       </c>
     </row>
     <row r="1714">
       <c r="A1714" t="inlineStr">
         <is>
-          <t>OKVED_50_PostDeyt</t>
+          <t>OKVED_49_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1715">
       <c r="A1715" t="inlineStr">
         <is>
-          <t>OKVED_50_PostDeyt1</t>
+          <t>OKVED_50_PostDeyt</t>
         </is>
       </c>
     </row>
     <row r="1716">
       <c r="A1716" t="inlineStr">
         <is>
-          <t>OKVED_50_DrPost</t>
+          <t>OKVED_50_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1717">
       <c r="A1717" t="inlineStr">
         <is>
-          <t>OKVED_51_PostDeyt</t>
+          <t>OKVED_50_DrPost</t>
         </is>
       </c>
     </row>
     <row r="1718">
       <c r="A1718" t="inlineStr">
         <is>
-          <t>OKVED_51_PostDeyt1</t>
+          <t>OKVED_51_PostDeyt</t>
         </is>
       </c>
     </row>
     <row r="1719">
       <c r="A1719" t="inlineStr">
         <is>
-          <t>OKVED_51_DrPost</t>
+          <t>OKVED_51_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1720">
       <c r="A1720" t="inlineStr">
         <is>
-          <t>OKVED_52_PostDeyt1</t>
+          <t>OKVED_51_DrPost</t>
         </is>
       </c>
     </row>
     <row r="1721">
       <c r="A1721" t="inlineStr">
         <is>
-          <t>OKVED_I_PostDeyt1</t>
+          <t>OKVED_52_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1722">
       <c r="A1722" t="inlineStr">
         <is>
-          <t>OKVED_I_DrPost</t>
+          <t>OKVED_I_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1723">
       <c r="A1723" t="inlineStr">
         <is>
-          <t>OKVED_55_PostDeyt1</t>
+          <t>OKVED_I_DrPost</t>
         </is>
       </c>
     </row>
     <row r="1724">
       <c r="A1724" t="inlineStr">
         <is>
-          <t>OKVED_55_DrPost</t>
+          <t>OKVED_55_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1725">
       <c r="A1725" t="inlineStr">
         <is>
-          <t>OKVED_K_PostDeyt</t>
+          <t>OKVED_55_DrPost</t>
         </is>
       </c>
     </row>
     <row r="1726">
       <c r="A1726" t="inlineStr">
         <is>
-          <t>OKVED_K_PostDeyt1</t>
+          <t>OKVED_K_PostDeyt</t>
         </is>
       </c>
     </row>
     <row r="1727">
       <c r="A1727" t="inlineStr">
         <is>
-          <t>OKVED_K_DrPost</t>
+          <t>OKVED_K_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1728">
       <c r="A1728" t="inlineStr">
         <is>
-          <t>OKVED_64_PostDeyt</t>
+          <t>OKVED_K_DrPost</t>
         </is>
       </c>
     </row>
     <row r="1729">
       <c r="A1729" t="inlineStr">
         <is>
-          <t>OKVED_64_PostDeyt1</t>
+          <t>OKVED_64_PostDeyt</t>
         </is>
       </c>
     </row>
     <row r="1730">
       <c r="A1730" t="inlineStr">
         <is>
-          <t>OKVED_64_DrPost</t>
+          <t>OKVED_64_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1731">
       <c r="A1731" t="inlineStr">
         <is>
-          <t>OKVED_L_PostDeyt1</t>
+          <t>OKVED_64_DrPost</t>
         </is>
       </c>
     </row>
     <row r="1732">
       <c r="A1732" t="inlineStr">
         <is>
-          <t>OKVED_68_PostDeyt1</t>
+          <t>OKVED_L_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1733">
       <c r="A1733" t="inlineStr">
         <is>
-          <t>OKVED_M_PostDeyt</t>
+          <t>OKVED_68_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1734">
       <c r="A1734" t="inlineStr">
         <is>
-          <t>OKVED_70_PlCredit</t>
+          <t>OKVED_M_PostDeyt</t>
         </is>
       </c>
     </row>
     <row r="1735">
       <c r="A1735" t="inlineStr">
         <is>
-          <t>OKVED_70_PostDeyt</t>
+          <t>OKVED_70_PlCredit</t>
         </is>
       </c>
     </row>
     <row r="1736">
       <c r="A1736" t="inlineStr">
         <is>
-          <t>OKVED_71_PostDeyt</t>
+          <t>OKVED_70_PostDeyt</t>
         </is>
       </c>
     </row>
     <row r="1737">
       <c r="A1737" t="inlineStr">
         <is>
-          <t>OKVED_74_PostDeyt</t>
+          <t>OKVED_71_PostDeyt</t>
         </is>
       </c>
     </row>
     <row r="1738">
       <c r="A1738" t="inlineStr">
         <is>
-          <t>OKVED_74_PostDeyt1</t>
+          <t>OKVED_74_PostDeyt</t>
         </is>
       </c>
     </row>
     <row r="1739">
       <c r="A1739" t="inlineStr">
         <is>
-          <t>OKVED_74_DrPost</t>
+          <t>OKVED_74_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1740">
       <c r="A1740" t="inlineStr">
         <is>
-          <t>OKVED_N_PostDeyt</t>
+          <t>OKVED_74_DrPost</t>
         </is>
       </c>
     </row>
     <row r="1741">
       <c r="A1741" t="inlineStr">
         <is>
-          <t>OKVED_N_PostDeyt1</t>
+          <t>OKVED_N_PostDeyt</t>
         </is>
       </c>
     </row>
     <row r="1742">
       <c r="A1742" t="inlineStr">
         <is>
-          <t>OKVED_79_PostDeyt</t>
+          <t>OKVED_N_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1743">
       <c r="A1743" t="inlineStr">
         <is>
-          <t>OKVED_79_PostDeyt1</t>
+          <t>OKVED_79_PostDeyt</t>
         </is>
       </c>
     </row>
     <row r="1744">
       <c r="A1744" t="inlineStr">
         <is>
-          <t>OKVED_79_DrPost</t>
+          <t>OKVED_79_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1745">
       <c r="A1745" t="inlineStr">
         <is>
-          <t>OKVED_81_PlCredit</t>
+          <t>OKVED_79_DrPost</t>
         </is>
       </c>
     </row>
     <row r="1746">
       <c r="A1746" t="inlineStr">
         <is>
-          <t>OKVED_81_PostDeyt</t>
+          <t>OKVED_81_PlCredit</t>
         </is>
       </c>
     </row>
     <row r="1747">
       <c r="A1747" t="inlineStr">
         <is>
-          <t>OKVED_81_PostDeyt1</t>
+          <t>OKVED_81_PostDeyt</t>
         </is>
       </c>
     </row>
     <row r="1748">
       <c r="A1748" t="inlineStr">
         <is>
-          <t>OKVED_S_PlCredit</t>
+          <t>OKVED_81_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1749">
       <c r="A1749" t="inlineStr">
         <is>
-          <t>OKVED_S_PostDeyt1</t>
+          <t>OKVED_S_PlCredit</t>
         </is>
       </c>
     </row>
     <row r="1750">
       <c r="A1750" t="inlineStr">
         <is>
-          <t>OKVED_94_PlCredit</t>
+          <t>OKVED_S_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1751">
       <c r="A1751" t="inlineStr">
         <is>
-          <t>OKVED_94_PostDeyt1</t>
+          <t>OKVED_94_PlCredit</t>
         </is>
       </c>
     </row>
     <row r="1752">
       <c r="A1752" t="inlineStr">
         <is>
-          <t>OKVED_01_PlPoFin1</t>
+          <t>OKVED_94_PostDeyt1</t>
         </is>
       </c>
     </row>
     <row r="1753">
       <c r="A1753" t="inlineStr">
         <is>
-          <t>OKVED_01_PlPoFin2</t>
+          <t>OKVED_01_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1754">
       <c r="A1754" t="inlineStr">
         <is>
-          <t>OKVED_B_PlPoFin1</t>
+          <t>OKVED_01_PlPoFin2</t>
         </is>
       </c>
     </row>
     <row r="1755">
       <c r="A1755" t="inlineStr">
         <is>
-          <t>OKVED_07_PlPoFin1</t>
+          <t>OKVED_B_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1756">
       <c r="A1756" t="inlineStr">
         <is>
-          <t>OKVED_32_PlPoFin</t>
+          <t>OKVED_07_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1757">
       <c r="A1757" t="inlineStr">
         <is>
-          <t>OKVED_32_PlPoFin1</t>
+          <t>OKVED_32_PlPoFin</t>
         </is>
       </c>
     </row>
     <row r="1758">
       <c r="A1758" t="inlineStr">
         <is>
-          <t>OKVED_32_PlPoFin2</t>
+          <t>OKVED_32_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1759">
       <c r="A1759" t="inlineStr">
         <is>
-          <t>OKVED_32_PlPoFin3</t>
+          <t>OKVED_32_PlPoFin2</t>
         </is>
       </c>
     </row>
     <row r="1760">
       <c r="A1760" t="inlineStr">
         <is>
-          <t>OKVED_33_PlPoFin</t>
+          <t>OKVED_32_PlPoFin3</t>
         </is>
       </c>
     </row>
     <row r="1761">
       <c r="A1761" t="inlineStr">
         <is>
-          <t>OKVED_33_PlPoFin1</t>
+          <t>OKVED_33_PlPoFin</t>
         </is>
       </c>
     </row>
     <row r="1762">
       <c r="A1762" t="inlineStr">
         <is>
-          <t>OKVED_33_PlPoFin2</t>
+          <t>OKVED_33_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1763">
       <c r="A1763" t="inlineStr">
         <is>
-          <t>OKVED_33_PlPoFin3</t>
+          <t>OKVED_33_PlPoFin2</t>
         </is>
       </c>
     </row>
     <row r="1764">
       <c r="A1764" t="inlineStr">
         <is>
-          <t>OKVED_35_PlPoFin1</t>
+          <t>OKVED_33_PlPoFin3</t>
         </is>
       </c>
     </row>
@@ -12774,588 +12774,588 @@
     <row r="1766">
       <c r="A1766" t="inlineStr">
         <is>
-          <t>OKVED_E_PlPoFin1</t>
+          <t>OKVED_35_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1767">
       <c r="A1767" t="inlineStr">
         <is>
-          <t>OKVED_E_PlPoFin2</t>
+          <t>OKVED_E_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1768">
       <c r="A1768" t="inlineStr">
         <is>
-          <t>OKVED_38_PlPoFin1</t>
+          <t>OKVED_E_PlPoFin2</t>
         </is>
       </c>
     </row>
     <row r="1769">
       <c r="A1769" t="inlineStr">
         <is>
-          <t>OKVED_38_PlPoFin2</t>
+          <t>OKVED_38_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1770">
       <c r="A1770" t="inlineStr">
         <is>
-          <t>OKVED_F_PlPoFin1</t>
+          <t>OKVED_38_PlPoFin2</t>
         </is>
       </c>
     </row>
     <row r="1771">
       <c r="A1771" t="inlineStr">
         <is>
-          <t>OKVED_41_PlPoFin1</t>
+          <t>OKVED_F_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1772">
       <c r="A1772" t="inlineStr">
         <is>
-          <t>OKVED_42_PlPoFin1</t>
+          <t>OKVED_41_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1773">
       <c r="A1773" t="inlineStr">
         <is>
-          <t>OKVED_43_PlPoFin1</t>
+          <t>OKVED_42_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1774">
       <c r="A1774" t="inlineStr">
         <is>
-          <t>OKVED_43_PlPoFin2</t>
+          <t>OKVED_43_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1775">
       <c r="A1775" t="inlineStr">
         <is>
-          <t>OKVED_G_PlPoFin1</t>
+          <t>OKVED_43_PlPoFin2</t>
         </is>
       </c>
     </row>
     <row r="1776">
       <c r="A1776" t="inlineStr">
         <is>
-          <t>OKVED_46_PlPoFin1</t>
+          <t>OKVED_G_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1777">
       <c r="A1777" t="inlineStr">
         <is>
-          <t>OKVED_47_PlPoFin1</t>
+          <t>OKVED_46_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1778">
       <c r="A1778" t="inlineStr">
         <is>
-          <t>OKVED_H_PlPoFin1</t>
+          <t>OKVED_47_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1779">
       <c r="A1779" t="inlineStr">
         <is>
-          <t>OKVED_49_PlPoFin1</t>
+          <t>OKVED_H_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1780">
       <c r="A1780" t="inlineStr">
         <is>
-          <t>OKVED_49_PlPoFin2</t>
+          <t>OKVED_49_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1781">
       <c r="A1781" t="inlineStr">
         <is>
-          <t>OKVED_50_PlPoFin1</t>
+          <t>OKVED_49_PlPoFin2</t>
         </is>
       </c>
     </row>
     <row r="1782">
       <c r="A1782" t="inlineStr">
         <is>
-          <t>OKVED_51_PlPoFin1</t>
+          <t>OKVED_50_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1783">
       <c r="A1783" t="inlineStr">
         <is>
-          <t>OKVED_51_PlPoFin2</t>
+          <t>OKVED_51_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1784">
       <c r="A1784" t="inlineStr">
         <is>
-          <t>OKVED_52_PlPoFin1</t>
+          <t>OKVED_51_PlPoFin2</t>
         </is>
       </c>
     </row>
     <row r="1785">
       <c r="A1785" t="inlineStr">
         <is>
-          <t>OKVED_I_PlPoFin1</t>
+          <t>OKVED_52_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1786">
       <c r="A1786" t="inlineStr">
         <is>
-          <t>OKVED_I_PlPoFin2</t>
+          <t>OKVED_I_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1787">
       <c r="A1787" t="inlineStr">
         <is>
-          <t>OKVED_55_PlPoFin1</t>
+          <t>OKVED_I_PlPoFin2</t>
         </is>
       </c>
     </row>
     <row r="1788">
       <c r="A1788" t="inlineStr">
         <is>
-          <t>OKVED_55_PlPoFin2</t>
+          <t>OKVED_55_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1789">
       <c r="A1789" t="inlineStr">
         <is>
-          <t>OKVED_K_PlPoFin1</t>
+          <t>OKVED_55_PlPoFin2</t>
         </is>
       </c>
     </row>
     <row r="1790">
       <c r="A1790" t="inlineStr">
         <is>
-          <t>OKVED_64_PlPoFin1</t>
+          <t>OKVED_K_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1791">
       <c r="A1791" t="inlineStr">
         <is>
-          <t>OKVED_L_PlPoFin1</t>
+          <t>OKVED_64_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1792">
       <c r="A1792" t="inlineStr">
         <is>
-          <t>OKVED_68_PlPoFin1</t>
+          <t>OKVED_L_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1793">
       <c r="A1793" t="inlineStr">
         <is>
-          <t>OKVED_M_PlPoFin1</t>
+          <t>OKVED_68_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1794">
       <c r="A1794" t="inlineStr">
         <is>
-          <t>OKVED_70_PlPoFin</t>
+          <t>OKVED_M_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1795">
       <c r="A1795" t="inlineStr">
         <is>
-          <t>OKVED_70_PlPoFin1</t>
+          <t>OKVED_70_PlPoFin</t>
         </is>
       </c>
     </row>
     <row r="1796">
       <c r="A1796" t="inlineStr">
         <is>
-          <t>OKVED_70_PlPoFin2</t>
+          <t>OKVED_70_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1797">
       <c r="A1797" t="inlineStr">
         <is>
-          <t>OKVED_70_PlPoFin3</t>
+          <t>OKVED_70_PlPoFin2</t>
         </is>
       </c>
     </row>
     <row r="1798">
       <c r="A1798" t="inlineStr">
         <is>
-          <t>OKVED_71_PlPoFin1</t>
+          <t>OKVED_70_PlPoFin3</t>
         </is>
       </c>
     </row>
     <row r="1799">
       <c r="A1799" t="inlineStr">
         <is>
-          <t>OKVED_74_PlPoFin1</t>
+          <t>OKVED_71_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1800">
       <c r="A1800" t="inlineStr">
         <is>
-          <t>OKVED_74_PlPoFin2</t>
+          <t>OKVED_74_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1801">
       <c r="A1801" t="inlineStr">
         <is>
-          <t>OKVED_74_PlPoFin3</t>
+          <t>OKVED_74_PlPoFin2</t>
         </is>
       </c>
     </row>
     <row r="1802">
       <c r="A1802" t="inlineStr">
         <is>
-          <t>OKVED_74_SaldoDenPot</t>
+          <t>OKVED_74_PlPoFin3</t>
         </is>
       </c>
     </row>
     <row r="1803">
       <c r="A1803" t="inlineStr">
         <is>
-          <t>OKVED_N_PlPoFin1</t>
+          <t>OKVED_74_SaldoDenPot</t>
         </is>
       </c>
     </row>
     <row r="1804">
       <c r="A1804" t="inlineStr">
         <is>
-          <t>OKVED_N_PlPoFin2</t>
+          <t>OKVED_N_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1805">
       <c r="A1805" t="inlineStr">
         <is>
-          <t>OKVED_79_PlPoFin1</t>
+          <t>OKVED_N_PlPoFin2</t>
         </is>
       </c>
     </row>
     <row r="1806">
       <c r="A1806" t="inlineStr">
         <is>
-          <t>OKVED_79_PlPoFin2</t>
+          <t>OKVED_79_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1807">
       <c r="A1807" t="inlineStr">
         <is>
-          <t>OKVED_81_PlPoFin1</t>
+          <t>OKVED_79_PlPoFin2</t>
         </is>
       </c>
     </row>
     <row r="1808">
       <c r="A1808" t="inlineStr">
         <is>
-          <t>OKVED_81_PlPoFin2</t>
+          <t>OKVED_81_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1809">
       <c r="A1809" t="inlineStr">
         <is>
-          <t>OKVED_81_PlPoFin3</t>
+          <t>OKVED_81_PlPoFin2</t>
         </is>
       </c>
     </row>
     <row r="1810">
       <c r="A1810" t="inlineStr">
         <is>
-          <t>OKVED_81_SaldoDenPot</t>
+          <t>OKVED_81_PlPoFin3</t>
         </is>
       </c>
     </row>
     <row r="1811">
       <c r="A1811" t="inlineStr">
         <is>
-          <t>OKVED_S_PlPoFin1</t>
+          <t>OKVED_81_SaldoDenPot</t>
         </is>
       </c>
     </row>
     <row r="1812">
       <c r="A1812" t="inlineStr">
         <is>
-          <t>OKVED_S_PlPoFin2</t>
+          <t>OKVED_S_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1813">
       <c r="A1813" t="inlineStr">
         <is>
-          <t>OKVED_S_PlPoFin3</t>
+          <t>OKVED_S_PlPoFin2</t>
         </is>
       </c>
     </row>
     <row r="1814">
       <c r="A1814" t="inlineStr">
         <is>
-          <t>OKVED_94_PlPoFin1</t>
+          <t>OKVED_S_PlPoFin3</t>
         </is>
       </c>
     </row>
     <row r="1815">
       <c r="A1815" t="inlineStr">
         <is>
-          <t>OKVED_94_PlPoFin2</t>
+          <t>OKVED_94_PlPoFin1</t>
         </is>
       </c>
     </row>
     <row r="1816">
       <c r="A1816" t="inlineStr">
         <is>
-          <t>OKVED_94_PlPoFin3</t>
+          <t>OKVED_94_PlPoFin2</t>
         </is>
       </c>
     </row>
     <row r="1817">
       <c r="A1817" t="inlineStr">
         <is>
-          <t>OKVED_01_Velch</t>
+          <t>OKVED_94_PlPoFin3</t>
         </is>
       </c>
     </row>
     <row r="1818">
       <c r="A1818" t="inlineStr">
         <is>
-          <t>OKVED_11_Velch</t>
+          <t>OKVED_01_Velch</t>
         </is>
       </c>
     </row>
     <row r="1819">
       <c r="A1819" t="inlineStr">
         <is>
-          <t>OKVED_32_Velch</t>
+          <t>OKVED_11_Velch</t>
         </is>
       </c>
     </row>
     <row r="1820">
       <c r="A1820" t="inlineStr">
         <is>
-          <t>OKVED_33_Velch</t>
+          <t>OKVED_32_Velch</t>
         </is>
       </c>
     </row>
     <row r="1821">
       <c r="A1821" t="inlineStr">
         <is>
-          <t>OKVED_E_Velch</t>
+          <t>OKVED_33_Velch</t>
         </is>
       </c>
     </row>
     <row r="1822">
       <c r="A1822" t="inlineStr">
         <is>
-          <t>OKVED_36_Velch</t>
+          <t>OKVED_E_Velch</t>
         </is>
       </c>
     </row>
     <row r="1823">
       <c r="A1823" t="inlineStr">
         <is>
-          <t>OKVED_38_Velch</t>
+          <t>OKVED_36_Velch</t>
         </is>
       </c>
     </row>
     <row r="1824">
       <c r="A1824" t="inlineStr">
         <is>
-          <t>OKVED_F_Velch</t>
+          <t>OKVED_38_Velch</t>
         </is>
       </c>
     </row>
     <row r="1825">
       <c r="A1825" t="inlineStr">
         <is>
-          <t>OKVED_41_Velch</t>
+          <t>OKVED_F_Velch</t>
         </is>
       </c>
     </row>
     <row r="1826">
       <c r="A1826" t="inlineStr">
         <is>
-          <t>OKVED_42_Velch</t>
+          <t>OKVED_41_Velch</t>
         </is>
       </c>
     </row>
     <row r="1827">
       <c r="A1827" t="inlineStr">
         <is>
-          <t>OKVED_43_Velch</t>
+          <t>OKVED_42_Velch</t>
         </is>
       </c>
     </row>
     <row r="1828">
       <c r="A1828" t="inlineStr">
         <is>
-          <t>OKVED_47_Velch</t>
+          <t>OKVED_43_Velch</t>
         </is>
       </c>
     </row>
     <row r="1829">
       <c r="A1829" t="inlineStr">
         <is>
-          <t>OKVED_49_Velch</t>
+          <t>OKVED_47_Velch</t>
         </is>
       </c>
     </row>
     <row r="1830">
       <c r="A1830" t="inlineStr">
         <is>
-          <t>OKVED_I_Velch</t>
+          <t>OKVED_49_Velch</t>
         </is>
       </c>
     </row>
     <row r="1831">
       <c r="A1831" t="inlineStr">
         <is>
-          <t>OKVED_55_Velch</t>
+          <t>OKVED_I_Velch</t>
         </is>
       </c>
     </row>
     <row r="1832">
       <c r="A1832" t="inlineStr">
         <is>
-          <t>OKVED_56_Velch</t>
+          <t>OKVED_55_Velch</t>
         </is>
       </c>
     </row>
     <row r="1833">
       <c r="A1833" t="inlineStr">
         <is>
-          <t>OKVED_J_Velch</t>
+          <t>OKVED_56_Velch</t>
         </is>
       </c>
     </row>
     <row r="1834">
       <c r="A1834" t="inlineStr">
         <is>
-          <t>OKVED_63_Velch</t>
+          <t>OKVED_J_Velch</t>
         </is>
       </c>
     </row>
     <row r="1835">
       <c r="A1835" t="inlineStr">
         <is>
-          <t>OKVED_L_Velch</t>
+          <t>OKVED_63_Velch</t>
         </is>
       </c>
     </row>
     <row r="1836">
       <c r="A1836" t="inlineStr">
         <is>
-          <t>OKVED_68_Velch</t>
+          <t>OKVED_L_Velch</t>
         </is>
       </c>
     </row>
     <row r="1837">
       <c r="A1837" t="inlineStr">
         <is>
-          <t>OKVED_M_Velch</t>
+          <t>OKVED_68_Velch</t>
         </is>
       </c>
     </row>
     <row r="1838">
       <c r="A1838" t="inlineStr">
         <is>
-          <t>OKVED_69_Velch</t>
+          <t>OKVED_M_Velch</t>
         </is>
       </c>
     </row>
     <row r="1839">
       <c r="A1839" t="inlineStr">
         <is>
-          <t>OKVED_70_Velch</t>
+          <t>OKVED_69_Velch</t>
         </is>
       </c>
     </row>
     <row r="1840">
       <c r="A1840" t="inlineStr">
         <is>
-          <t>OKVED_71_Velch</t>
+          <t>OKVED_70_Velch</t>
         </is>
       </c>
     </row>
     <row r="1841">
       <c r="A1841" t="inlineStr">
         <is>
-          <t>OKVED_74_Velch</t>
+          <t>OKVED_71_Velch</t>
         </is>
       </c>
     </row>
     <row r="1842">
       <c r="A1842" t="inlineStr">
         <is>
-          <t>OKVED_N_Velch</t>
+          <t>OKVED_74_Velch</t>
         </is>
       </c>
     </row>
     <row r="1843">
       <c r="A1843" t="inlineStr">
         <is>
-          <t>OKVED_77_Velch</t>
+          <t>OKVED_N_Velch</t>
         </is>
       </c>
     </row>
     <row r="1844">
       <c r="A1844" t="inlineStr">
         <is>
-          <t>OKVED_79_Velch</t>
+          <t>OKVED_77_Velch</t>
         </is>
       </c>
     </row>
     <row r="1845">
       <c r="A1845" t="inlineStr">
         <is>
-          <t>OKVED_81_Velch</t>
+          <t>OKVED_79_Velch</t>
         </is>
       </c>
     </row>
     <row r="1846">
       <c r="A1846" t="inlineStr">
         <is>
-          <t>OKVED_82_Velch</t>
+          <t>OKVED_81_Velch</t>
         </is>
       </c>
     </row>
     <row r="1847">
       <c r="A1847" t="inlineStr">
         <is>
-          <t>OKVED_O_Velch</t>
+          <t>OKVED_82_Velch</t>
         </is>
       </c>
     </row>
     <row r="1848">
       <c r="A1848" t="inlineStr">
         <is>
-          <t>OKVED_84_Velch</t>
+          <t>OKVED_O_Velch</t>
         </is>
       </c>
     </row>
     <row r="1849">
       <c r="A1849" t="inlineStr">
         <is>
-          <t>OKVED_85_Velch</t>
+          <t>OKVED_84_Velch</t>
         </is>
       </c>
     </row>
@@ -13369,208 +13369,215 @@
     <row r="1851">
       <c r="A1851" t="inlineStr">
         <is>
-          <t>OKVED_Q_Velch</t>
+          <t>OKVED_85_Velch</t>
         </is>
       </c>
     </row>
     <row r="1852">
       <c r="A1852" t="inlineStr">
         <is>
-          <t>OKVED_88_Velch</t>
+          <t>OKVED_Q_Velch</t>
         </is>
       </c>
     </row>
     <row r="1853">
       <c r="A1853" t="inlineStr">
         <is>
-          <t>OKVED_R_Velch</t>
+          <t>OKVED_88_Velch</t>
         </is>
       </c>
     </row>
     <row r="1854">
       <c r="A1854" t="inlineStr">
         <is>
-          <t>OKVED_93_Velch</t>
+          <t>OKVED_R_Velch</t>
         </is>
       </c>
     </row>
     <row r="1855">
       <c r="A1855" t="inlineStr">
         <is>
-          <t>OKVED_S_Velch</t>
+          <t>OKVED_93_Velch</t>
         </is>
       </c>
     </row>
     <row r="1856">
       <c r="A1856" t="inlineStr">
         <is>
-          <t>OKVED_94_Velch</t>
+          <t>OKVED_S_Velch</t>
         </is>
       </c>
     </row>
     <row r="1857">
       <c r="A1857" t="inlineStr">
         <is>
-          <t>OKVED_96_Velch</t>
+          <t>OKVED_94_Velch</t>
         </is>
       </c>
     </row>
     <row r="1858">
       <c r="A1858" t="inlineStr">
         <is>
-          <t>OKVED_43_UstKap_23</t>
+          <t>OKVED_96_Velch</t>
         </is>
       </c>
     </row>
     <row r="1859">
       <c r="A1859" t="inlineStr">
         <is>
-          <t>OKVED_43_ChiAkt_23</t>
+          <t>OKVED_43_UstKap_23</t>
         </is>
       </c>
     </row>
     <row r="1860">
       <c r="A1860" t="inlineStr">
         <is>
-          <t>OKVED_J_UstKap_23</t>
+          <t>OKVED_43_ChiAkt_23</t>
         </is>
       </c>
     </row>
     <row r="1861">
       <c r="A1861" t="inlineStr">
         <is>
-          <t>OKVED_J_UstKap_24</t>
+          <t>OKVED_J_UstKap_23</t>
         </is>
       </c>
     </row>
     <row r="1862">
       <c r="A1862" t="inlineStr">
         <is>
-          <t>OKVED_63_UstKap_23</t>
+          <t>OKVED_J_UstKap_24</t>
         </is>
       </c>
     </row>
     <row r="1863">
       <c r="A1863" t="inlineStr">
         <is>
-          <t>OKVED_63_UstKap_24</t>
+          <t>OKVED_63_UstKap_23</t>
         </is>
       </c>
     </row>
     <row r="1864">
       <c r="A1864" t="inlineStr">
         <is>
-          <t>OKVED_69_UstKap_23</t>
+          <t>OKVED_63_UstKap_24</t>
         </is>
       </c>
     </row>
     <row r="1865">
       <c r="A1865" t="inlineStr">
         <is>
-          <t>OKVED_69_UstKap_24</t>
+          <t>OKVED_69_UstKap_23</t>
         </is>
       </c>
     </row>
     <row r="1866">
       <c r="A1866" t="inlineStr">
         <is>
-          <t>OKVED_69_ChiAkt_23</t>
+          <t>OKVED_69_UstKap_24</t>
         </is>
       </c>
     </row>
     <row r="1867">
       <c r="A1867" t="inlineStr">
         <is>
-          <t>OKVED_O_UstKap_23</t>
+          <t>OKVED_69_ChiAkt_23</t>
         </is>
       </c>
     </row>
     <row r="1868">
       <c r="A1868" t="inlineStr">
         <is>
-          <t>OKVED_O_UstKap_24</t>
+          <t>OKVED_O_UstKap_23</t>
         </is>
       </c>
     </row>
     <row r="1869">
       <c r="A1869" t="inlineStr">
         <is>
-          <t>OKVED_84_UstKap_23</t>
+          <t>OKVED_O_UstKap_24</t>
         </is>
       </c>
     </row>
     <row r="1870">
       <c r="A1870" t="inlineStr">
         <is>
-          <t>OKVED_84_UstKap_24</t>
+          <t>OKVED_84_UstKap_23</t>
         </is>
       </c>
     </row>
     <row r="1871">
       <c r="A1871" t="inlineStr">
         <is>
-          <t>OKVED_85_UstKap_23</t>
+          <t>OKVED_84_UstKap_24</t>
         </is>
       </c>
     </row>
     <row r="1872">
       <c r="A1872" t="inlineStr">
         <is>
-          <t>OKVED_85_UstKap_24</t>
+          <t>OKVED_85_UstKap_23</t>
         </is>
       </c>
     </row>
     <row r="1873">
       <c r="A1873" t="inlineStr">
         <is>
-          <t>OKVED_85_UstKap_23</t>
+          <t>OKVED_85_UstKap_24</t>
         </is>
       </c>
     </row>
     <row r="1874">
       <c r="A1874" t="inlineStr">
         <is>
-          <t>OKVED_85_UstKap_24</t>
+          <t>OKVED_85_UstKap_23</t>
         </is>
       </c>
     </row>
     <row r="1875">
       <c r="A1875" t="inlineStr">
         <is>
-          <t>OKVED_Q_UstKap_23</t>
+          <t>OKVED_85_UstKap_24</t>
         </is>
       </c>
     </row>
     <row r="1876">
       <c r="A1876" t="inlineStr">
         <is>
-          <t>OKVED_Q_UstKap_24</t>
+          <t>OKVED_Q_UstKap_23</t>
         </is>
       </c>
     </row>
     <row r="1877">
       <c r="A1877" t="inlineStr">
         <is>
-          <t>OKVED_88_UstKap_23</t>
+          <t>OKVED_Q_UstKap_24</t>
         </is>
       </c>
     </row>
     <row r="1878">
       <c r="A1878" t="inlineStr">
         <is>
-          <t>OKVED_88_UstKap_24</t>
+          <t>OKVED_88_UstKap_23</t>
         </is>
       </c>
     </row>
     <row r="1879">
       <c r="A1879" t="inlineStr">
         <is>
-          <t>OKVED_R_UstKap_24</t>
+          <t>OKVED_88_UstKap_24</t>
         </is>
       </c>
     </row>
     <row r="1880">
       <c r="A1880" t="inlineStr">
+        <is>
+          <t>OKVED_R_UstKap_24</t>
+        </is>
+      </c>
+    </row>
+    <row r="1881">
+      <c r="A1881" t="inlineStr">
         <is>
           <t>OKVED_93_UstKap_24</t>
         </is>

</xml_diff>

<commit_message>
Stop dropping non-year columns mixed into a year-paired header run
_compute_section_mapping's has_years branch decides per section whether
columns carry a year suffix, but some tables mix year-paired columns
(e.g. "Уставный капитал" with 2023/2024 sub-columns) with standalone
columns that have no year at all (e.g. "Себестоимость продаж", "Чистая
прибыль (убыток) отчетного периода" in the "Чистые активы" table,
section 21). Any column whose year-row cell didn't parse as a year was
skipped outright via `continue`, even though its own header text
matched a real indicator just fine -- it just doesn't get a year
suffix. Now such columns are matched the same way and tagged without a
year suffix instead of being silently dropped.

Verified against the known-good baseline: 0 lost/changed tags, 232 new
tags across the affected tables.
</commit_message>
<xml_diff>
--- a/output/unfilled_tags.xlsx
+++ b/output/unfilled_tags.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1946"/>
+  <dimension ref="A1:A1967"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13908,133 +13908,280 @@
     <row r="1928">
       <c r="A1928" t="inlineStr">
         <is>
-          <t>OKVED_63_UstKap_23</t>
+          <t>OKVED_J_SebPro</t>
         </is>
       </c>
     </row>
     <row r="1929">
       <c r="A1929" t="inlineStr">
         <is>
-          <t>OKVED_63_UstKap_24</t>
+          <t>OKVED_J_Pri(ubOtPro</t>
         </is>
       </c>
     </row>
     <row r="1930">
       <c r="A1930" t="inlineStr">
         <is>
-          <t>OKVED_69_UstKap_23</t>
+          <t>OKVED_J_ChiPri(ubOtcPer</t>
         </is>
       </c>
     </row>
     <row r="1931">
       <c r="A1931" t="inlineStr">
         <is>
-          <t>OKVED_69_UstKap_24</t>
+          <t>OKVED_J_PriUby(-DoNalKChiAktV%</t>
         </is>
       </c>
     </row>
     <row r="1932">
       <c r="A1932" t="inlineStr">
         <is>
-          <t>OKVED_69_ChiAkt_23</t>
+          <t>OKVED_63_UstKap_23</t>
         </is>
       </c>
     </row>
     <row r="1933">
       <c r="A1933" t="inlineStr">
         <is>
-          <t>OKVED_O_UstKap_23</t>
+          <t>OKVED_63_UstKap_24</t>
         </is>
       </c>
     </row>
     <row r="1934">
       <c r="A1934" t="inlineStr">
         <is>
-          <t>OKVED_O_UstKap_24</t>
+          <t>OKVED_63_SebPro</t>
         </is>
       </c>
     </row>
     <row r="1935">
       <c r="A1935" t="inlineStr">
         <is>
-          <t>OKVED_84_UstKap_23</t>
+          <t>OKVED_63_Pri(ubOtPro</t>
         </is>
       </c>
     </row>
     <row r="1936">
       <c r="A1936" t="inlineStr">
         <is>
-          <t>OKVED_84_UstKap_24</t>
+          <t>OKVED_63_ChiPri(ubOtcPer</t>
         </is>
       </c>
     </row>
     <row r="1937">
       <c r="A1937" t="inlineStr">
         <is>
-          <t>OKVED_85_UstKap_23</t>
+          <t>OKVED_63_PriUby(-DoNalKChiAktV%</t>
         </is>
       </c>
     </row>
     <row r="1938">
       <c r="A1938" t="inlineStr">
         <is>
-          <t>OKVED_85_UstKap_24</t>
+          <t>OKVED_K_SebPro</t>
         </is>
       </c>
     </row>
     <row r="1939">
       <c r="A1939" t="inlineStr">
         <is>
-          <t>OKVED_85_UstKap_23</t>
+          <t>OKVED_64_SebPro</t>
         </is>
       </c>
     </row>
     <row r="1940">
       <c r="A1940" t="inlineStr">
         <is>
-          <t>OKVED_85_UstKap_24</t>
+          <t>OKVED_69_UstKap_23</t>
         </is>
       </c>
     </row>
     <row r="1941">
       <c r="A1941" t="inlineStr">
         <is>
-          <t>OKVED_Q_UstKap_23</t>
+          <t>OKVED_69_UstKap_24</t>
         </is>
       </c>
     </row>
     <row r="1942">
       <c r="A1942" t="inlineStr">
         <is>
-          <t>OKVED_Q_UstKap_24</t>
+          <t>OKVED_69_ChiAkt_23</t>
         </is>
       </c>
     </row>
     <row r="1943">
       <c r="A1943" t="inlineStr">
         <is>
-          <t>OKVED_88_UstKap_23</t>
+          <t>OKVED_69_SebPro</t>
         </is>
       </c>
     </row>
     <row r="1944">
       <c r="A1944" t="inlineStr">
         <is>
-          <t>OKVED_88_UstKap_24</t>
+          <t>OKVED_O_UstKap_23</t>
         </is>
       </c>
     </row>
     <row r="1945">
       <c r="A1945" t="inlineStr">
         <is>
-          <t>OKVED_R_UstKap_24</t>
+          <t>OKVED_O_UstKap_24</t>
         </is>
       </c>
     </row>
     <row r="1946">
       <c r="A1946" t="inlineStr">
         <is>
+          <t>OKVED_84_UstKap_23</t>
+        </is>
+      </c>
+    </row>
+    <row r="1947">
+      <c r="A1947" t="inlineStr">
+        <is>
+          <t>OKVED_84_UstKap_24</t>
+        </is>
+      </c>
+    </row>
+    <row r="1948">
+      <c r="A1948" t="inlineStr">
+        <is>
+          <t>OKVED_85_UstKap_23</t>
+        </is>
+      </c>
+    </row>
+    <row r="1949">
+      <c r="A1949" t="inlineStr">
+        <is>
+          <t>OKVED_85_UstKap_24</t>
+        </is>
+      </c>
+    </row>
+    <row r="1950">
+      <c r="A1950" t="inlineStr">
+        <is>
+          <t>OKVED_85_UstKap_23</t>
+        </is>
+      </c>
+    </row>
+    <row r="1951">
+      <c r="A1951" t="inlineStr">
+        <is>
+          <t>OKVED_85_UstKap_24</t>
+        </is>
+      </c>
+    </row>
+    <row r="1952">
+      <c r="A1952" t="inlineStr">
+        <is>
+          <t>OKVED_Q_UstKap_23</t>
+        </is>
+      </c>
+    </row>
+    <row r="1953">
+      <c r="A1953" t="inlineStr">
+        <is>
+          <t>OKVED_Q_UstKap_24</t>
+        </is>
+      </c>
+    </row>
+    <row r="1954">
+      <c r="A1954" t="inlineStr">
+        <is>
+          <t>OKVED_Q_SebPro</t>
+        </is>
+      </c>
+    </row>
+    <row r="1955">
+      <c r="A1955" t="inlineStr">
+        <is>
+          <t>OKVED_Q_Pri(ubOtPro</t>
+        </is>
+      </c>
+    </row>
+    <row r="1956">
+      <c r="A1956" t="inlineStr">
+        <is>
+          <t>OKVED_Q_ChiPri(ubOtcPer</t>
+        </is>
+      </c>
+    </row>
+    <row r="1957">
+      <c r="A1957" t="inlineStr">
+        <is>
+          <t>OKVED_Q_PriUby(-DoNalKChiAktV%</t>
+        </is>
+      </c>
+    </row>
+    <row r="1958">
+      <c r="A1958" t="inlineStr">
+        <is>
+          <t>OKVED_88_UstKap_23</t>
+        </is>
+      </c>
+    </row>
+    <row r="1959">
+      <c r="A1959" t="inlineStr">
+        <is>
+          <t>OKVED_88_UstKap_24</t>
+        </is>
+      </c>
+    </row>
+    <row r="1960">
+      <c r="A1960" t="inlineStr">
+        <is>
+          <t>OKVED_88_SebPro</t>
+        </is>
+      </c>
+    </row>
+    <row r="1961">
+      <c r="A1961" t="inlineStr">
+        <is>
+          <t>OKVED_88_Pri(ubOtPro</t>
+        </is>
+      </c>
+    </row>
+    <row r="1962">
+      <c r="A1962" t="inlineStr">
+        <is>
+          <t>OKVED_88_ChiPri(ubOtcPer</t>
+        </is>
+      </c>
+    </row>
+    <row r="1963">
+      <c r="A1963" t="inlineStr">
+        <is>
+          <t>OKVED_88_PriUby(-DoNalKChiAktV%</t>
+        </is>
+      </c>
+    </row>
+    <row r="1964">
+      <c r="A1964" t="inlineStr">
+        <is>
+          <t>OKVED_R_UstKap_24</t>
+        </is>
+      </c>
+    </row>
+    <row r="1965">
+      <c r="A1965" t="inlineStr">
+        <is>
+          <t>OKVED_R_SebPro</t>
+        </is>
+      </c>
+    </row>
+    <row r="1966">
+      <c r="A1966" t="inlineStr">
+        <is>
           <t>OKVED_93_UstKap_24</t>
+        </is>
+      </c>
+    </row>
+    <row r="1967">
+      <c r="A1967" t="inlineStr">
+        <is>
+          <t>OKVED_93_SebPro</t>
         </is>
       </c>
     </row>

</xml_diff>